<commit_message>
docs: reframe low-altitude PhD topic from literature
</commit_message>
<xml_diff>
--- a/research/low_altitude_phd_20261013/04_literature_review.xlsx
+++ b/research/low_altitude_phd_20261013/04_literature_review.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="文献梳理" sheetId="1" r:id="R94af11b68e5742d2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="书目与证据" sheetId="2" r:id="Rc63a7c3d18b940d5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="全文获取状态" sheetId="3" r:id="Rcf558de8c71741a3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="文献梳理" sheetId="1" r:id="Rfecadfbcfdeb4dad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="书目与证据" sheetId="2" r:id="R42d84954a4744d4e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="全文获取状态" sheetId="3" r:id="Rf31aacc681454fc5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -208,8 +208,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="LiteratureReviewTable" displayName="LiteratureReviewTable" ref="A1:H34" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:H34"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="LiteratureReviewTable" displayName="LiteratureReviewTable" ref="A1:H36" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:H36"/>
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="题名（年）"/>
@@ -225,8 +225,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="BibliographyEvidenceTable" displayName="BibliographyEvidenceTable" ref="A1:Q34" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:Q34"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="BibliographyEvidenceTable" displayName="BibliographyEvidenceTable" ref="A1:Q36" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:Q36"/>
   <x:tableColumns count="17">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="完整作者（★为第一作者）"/>
@@ -251,8 +251,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="MissingFullTextTable" displayName="MissingFullTextTable" ref="A5:I8" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:I8"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="MissingFullTextTable" displayName="MissingFullTextTable" ref="A5:I9" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:I9"/>
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="题名（年）"/>
@@ -534,10 +534,10 @@
 作者指出仍需推广到更高且异质的 preferred-velocity 范围，并进行包含多场景选择行为的全局优化。</x:v>
       </x:c>
       <x:c r="F2" s="4" t="str">
-        <x:v>全文评价：证明了局部规则与密度、通信延迟之间的关系，但共同目的地附近缺少显式排序，恰是终端区的关键业务；通量峰值不能直接等同于有服务时间约束的降落容量。</x:v>
+        <x:v>全文评价：已比较局部规则、场景、密度与通信延迟并给出基本图；共同目标附近未显式排序为作者边界。规则相关流量与车道已有先例，通量定义不能直接换算为其他业务的完成出流。</x:v>
       </x:c>
       <x:c r="G2" s="4" t="str">
-        <x:v>作为自组织规则、延迟敏感性和瓶颈形成的基础文献。</x:v>
+        <x:v>局部规则、延迟和密度共同改变通量的基础，用于限定机理与基本图贡献。</x:v>
       </x:c>
       <x:c r="H2" s="11" t="str">
         <x:v>FULL_TEXT</x:v>
@@ -573,10 +573,10 @@
 可观察设定：网络为随机图、时间/能耗/容量权重人为给定，优化目标主要分开处理时间或能耗；没有飞行动力学、障碍物或真实城市网络验证。</x:v>
       </x:c>
       <x:c r="F3" s="4" t="str">
-        <x:v>全文评价：随机多层图和人为边权便于算法比较，但网络流可行不等于连续飞行轨迹可行；局部信息策略的优势依赖所测网络与权重，尚需现实几何和服务资源验证。</x:v>
+        <x:v>全文评价：随机多层图和人为边权便于比较，但图上流可行不等于连续轨迹可行；局部信息策略优势依赖所测网络和权重，需现实几何与通信条件验证。</x:v>
       </x:c>
       <x:c r="G3" s="4" t="str">
-        <x:v>借鉴局部拥堵信息驱动路径选择，补足轨迹与瓶颈约束。</x:v>
+        <x:v>局部拥堵信息驱动分布式选路的参考，区分图层分配与连续执行。</x:v>
       </x:c>
       <x:c r="H3" s="11" t="str">
         <x:v>FULL_TEXT</x:v>
@@ -616,7 +616,7 @@
         <x:v>全文评价：综述揭示结构与风险并非单调关系，并已覆盖动态空域概念；异质来源的定性排名不等于统一实验下的容量排序。适合据此选有限固定对照构形，不能据其宣称某种结构普适最优（PDF pp.12、15、20、22–24）。</x:v>
       </x:c>
       <x:c r="G4" s="4" t="str">
-        <x:v>用于筛选有限固定对照构形与说明结构、风险、技术能力的条件权衡，不把综述排名当统一容量证据。</x:v>
+        <x:v>方向分层、结构谱系及条件权衡的综述依据，不把异质概念排名当统一容量证据。</x:v>
       </x:c>
       <x:c r="H4" s="11" t="str">
         <x:v>FULL_TEXT</x:v>
@@ -651,7 +651,7 @@
         <x:v>全文评价：城市几何与个体解脱已经被结合；但空间结构静态、起降阶段未纳入，且需求未触达容量，因此不能依据其安全改善推断吞吐也提高。</x:v>
       </x:c>
       <x:c r="G5" s="4" t="str">
-        <x:v>固定构形对照的强参考，动态需求和起降瓶颈应在其基础上检验。</x:v>
+        <x:v>方向组织与局部解脱的固定结构对照，分开评价安全、资源和是否达到容量。</x:v>
       </x:c>
       <x:c r="H5" s="11" t="str">
         <x:v>FULL_TEXT</x:v>
@@ -683,7 +683,7 @@
         <x:v>全文评价：定性打分依赖准则和权重，适合分类筛选，不足以确定实际安全容量或运行最优构形；应把这些结论当设计假设，随后以共同约束下的仿真验证。</x:v>
       </x:c>
       <x:c r="G6" s="4" t="str">
-        <x:v>用于有限构形集合的初筛，不把加权评分当容量模型。</x:v>
+        <x:v>空域概念分类和规则初筛参考，加权评价不能替代运行容量辨识。</x:v>
       </x:c>
       <x:c r="H6" s="11" t="str">
         <x:v>FULL_TEXT</x:v>
@@ -713,7 +713,7 @@
         <x:v>摘要评价，待全文确认：已明确结构自由度与拥堵存在需求相关权衡，不能再把发现该权衡作为新贡献。尚需核实其需求生成、局部算法和是否进行在线构形调整。</x:v>
       </x:c>
       <x:c r="G7" s="4" t="str">
-        <x:v>保留为需求相关结构权衡的摘要证据；用户已决定不继续追索全文，不据摘要补写未经核验的机制或限制。</x:v>
+        <x:v>需求相关结构权衡的摘要证据；停止追索，不外推未经核验机制或局限。</x:v>
       </x:c>
       <x:c r="H7" s="13" t="str">
         <x:v>ABSTRACT_ONLY</x:v>
@@ -745,10 +745,10 @@
 作者建议实飞复现时增大 avoidance radius，以消除偶发的危险最小距离峰值。</x:v>
       </x:c>
       <x:c r="F8" s="4" t="str">
-        <x:v>全文评价：大规模实飞是强证据，但开放空间、多旋翼与分层目标流仍不同于完整起降服务系统；无碰撞不等于没有间隔违规，实飞中偶发低于参考间隔的情况须保留。</x:v>
+        <x:v>全文评价：已有各向异性参数优化、航向分层、基本图和100架实飞，方向机制不是空白。1/3/5层同时改变可用空间、层内密度与方向一致性，不能全归因单一变量。无碰撞不等于无间隔违规，实飞偶发低于参考间隔须保留（PDF pp.6–7、17–20）。</x:v>
       </x:c>
       <x:c r="G8" s="4" t="str">
-        <x:v>局部自组织的强基线；起降服务瓶颈及构形收益递减直接支持研究范围选择。</x:v>
+        <x:v>核心自组织与方向机制基线，分离方向一致性、层内密度和额外空间贡献。</x:v>
       </x:c>
       <x:c r="H8" s="11" t="str">
         <x:v>FULL_TEXT</x:v>
@@ -778,10 +778,10 @@
 MITL 试验假定理想感知/无扰动，随后用 SITL 和硬件推进；正文没有给出城市尺度或多类型飞行器验证。</x:v>
       </x:c>
       <x:c r="F9" s="4" t="str">
-        <x:v>基于已访问正文评价：局部交通结构与实飞执行结合得较具体，但小规模交汇试验尚不能给出城市或终端服务容量；螺旋结构缓解冲突同时增加通行时间，需在总等待口径下权衡。</x:v>
+        <x:v>基于已访问正文评价：结构与实飞执行结合具体，但小规模交汇试验不足以确定城市网络容量；螺旋结构减小冲突同时增加通行时间。全文媒介为公开HTML，没有本地PDF不等于未读。</x:v>
       </x:c>
       <x:c r="G9" s="4" t="str">
-        <x:v>参考合流结构与实际执行机制；PDF缺失或正文不完整时按获取状态复核。</x:v>
+        <x:v>流向、合流和旋转指导的工程参考，同时评价冲突缓解与通行时间。</x:v>
       </x:c>
       <x:c r="H9" s="11" t="str">
         <x:v>FULL_TEXT</x:v>
@@ -813,10 +813,10 @@
 可观察设定边界：单一到达高度、无静态障碍、不能悬停、常规控制只改 heading，且一次只能有一个 VTOL zone landing maneuver；这些条件不能直接代表完整 UAM 终端区。</x:v>
       </x:c>
       <x:c r="F10" s="4" t="str">
-        <x:v>全文评价：已实现自组织进场与缩比实飞，不能再以此作为首次创新；简化服务占用、能源表达及非合作/无意图通信假设限制向完整终端运行外推，固定几何自身不作为缺点。入口保护前后事故结果必须分开，不能只报保护后安全结果。</x:v>
+        <x:v>全文评价：已实现自组织进场与缩比实飞，不是首次创新空白；简化服务占用、能源表达及非合作/无意图通信假设限制更一般业务外推。固定几何自身不作为缺点；入口保护前后事故结果必须分开。</x:v>
       </x:c>
       <x:c r="G10" s="4" t="str">
-        <x:v>最接近的基线之一，比较固定几何下服务资源、等待、能源与意图共享机制。</x:v>
+        <x:v>特定进场业务的外围自组织参考；保留共享策略和入口保护，不移植服务或能源设定为前提。</x:v>
       </x:c>
       <x:c r="H10" s="11" t="str">
         <x:v>FULL_TEXT</x:v>
@@ -850,155 +850,219 @@
         <x:v>全文评价：通信与让行用例覆盖较广，但统一规模下的容量、长尾等待和失效边界验证有限；局部规则组合尚不能自动推导整个系统的效率或公平性。</x:v>
       </x:c>
       <x:c r="G11" s="4" t="str">
-        <x:v>用于构造意图广播、优先权与局部合流规则。</x:v>
+        <x:v>通信、让行及多向交汇局部规则参考，区分战术用例与网络完成效率。</x:v>
       </x:c>
       <x:c r="H11" s="11" t="str">
         <x:v>FULL_TEXT</x:v>
       </x:c>
     </x:row>
-    <x:row r="12" ht="206" customHeight="1">
+    <x:row r="12" ht="178" customHeight="1">
       <x:c r="A12" s="4" t="str">
+        <x:v>A11</x:v>
+      </x:c>
+      <x:c r="B12" s="4" t="str">
+        <x:v>Coordinated Dense Aerial Traffic with Self-Driving Drones（2018）</x:v>
+      </x:c>
+      <x:c r="C12" s="4" t="str">
+        <x:v>方法：分布式速度控制叠加各向异性排斥、选择性速度对齐、可调切向自驱与径向虚拟排队。参数A按同向/对向关系改变排斥方向，加速同向车道形成；自驱用近邻几何迭代改变期望速度。CMA-ES结合局部参数扫描和人工轨迹检查完成调参，再用密度扫描和户外实飞验证。
+场景/设定：二维开放水平空域；crosswalk为两侧往返交叉流，star为中心共同目标与边界目标交替。仿真含有限通信范围、时延、传感噪声和有限加速度；优化用100架、250 m方形区域，最终实飞为30架、150×150 m、期望速度6 m/s、无风晴天。</x:v>
+      </x:c>
+      <x:c r="D12" s="4" t="str">
+        <x:v>主要结论：局部交互使同向链/车道、避让与虚拟排队形成，缓解振荡和共同目标拥堵；Fig.5给出有效速度、通量和碰撞风险随平均自由程变化，通量存在中间密度峰值。实飞在初始过渡后形成平稳交叉流。图中order parameters含目标方向有效速度和邻距，不等同于全局航向极化有序度。
+定量结果：Crosswalk密度扫描用100架；每个测量点平均20次10 min仿真，Fig.5标最大通量0.096/s，位于平均自由程36 m；通量定义为有效速度/平均自由程，非城市网络完成出流。
+Star场景在48个平均自由程值22–365 m上，每点20次仿真；到达中心的平均间隔约12±1 s，各次仿真报告零碰撞。
+30架户外实飞在150×150 m区域、6 m/s期望速度下进行；Fig.8为15 min飞行日志，归一化目标方向有效速度约0.4–0.5。</x:v>
+      </x:c>
+      <x:c r="E12" s="4" t="str">
+        <x:v>作者指出量化fitness不能充分刻画轨迹平顺性等整体质量，最终参数经过人工检查、局部扫描和实飞调节；不能将其描述为全自动最优参数。
+起飞间隔仅5–7 m、初始即处于排斥范围时出现不规则过渡运动；作者指出当前行为主要预防风险，并非专为从高风险初态恢复设计。
+任意障碍物和飞行器异质性/层级被列为后续扩展；本篇实飞为空旷、无风、二维crosswalk场景。</x:v>
+      </x:c>
+      <x:c r="F12" s="4" t="str">
+        <x:v>全文评价：已有各向异性排斥、选择性对齐、切向自驱和虚拟排队；CMA-ES、局部扫描和人工检查调参，密度曲线及30架实飞展示自组织。fitness未充分刻画平顺性，初始高风险过渡及无障碍同质二维条件须保留；通量是有效速度/平均自由程，非网络完成出流（PDF pp.2–8）。</x:v>
+      </x:c>
+      <x:c r="G12" s="4" t="str">
+        <x:v>密集自组织与方向交互的核心早期基线；区分已有参数优化、初始过渡和需求改变后的组织调整假设。</x:v>
+      </x:c>
+      <x:c r="H12" s="11" t="str">
+        <x:v>FULL_TEXT</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="206" customHeight="1">
+      <x:c r="A13" s="4" t="str">
+        <x:v>A12</x:v>
+      </x:c>
+      <x:c r="B13" s="4" t="str">
+        <x:v>Metropolis II: Benefits of Centralised Separation Management in High-Density Urban Airspace（2022）</x:v>
+      </x:c>
+      <x:c r="C13" s="4" t="str">
+        <x:v>方法：在BlueSky中比较集中战略、集中战略加分布式战术的混合概念、分布式战术概念；同时采用不同水平网格、航向分层、航路规划和起飞延迟规则。分布式概念仍由中央实体监测约束空域交通并更新成本，单机可选择是否据此重规划。比较密度分布、冲突、侵入、效率、延误和延误分散。
+场景/设定：维也纳中心8 km宽、500 ft高的圆柱空域，包含街道约束空域、开放空域和地理围栏；16个垂直层。两类简化Matrice 600 Pro机型巡航20/30 kts，四类任务与四级优先级；5档交通水平，风速0/1/3/5 kts，非合作机0/33/66/100架，各设置9次随机重复。</x:v>
+      </x:c>
+      <x:c r="D13" s="4" t="str">
+        <x:v>主要结论：混合概念在所测场景中侵入最少，但绕行和巡航空间减少导致效率下降、延误较大。集中与分布式概念侵入和需求延误相近，分布式延误分散较低。对照同时改变空域结构、分离职责与可巡航空间；作者明确不能把差异全归因于centralisation。环路提高方向一致性和空间分散，安全收益伴随路径效率代价。
+定量结果：Table II将5档交通列为平均同时在飞机数1660/3340/4990/6650/8290；每设置9次重复。仅首小时安排起飞，仿真运行90–180 min直到全部到达；不得混同小时总架次。
+高密度设置下，混合概念在约束空域的峰值密度约为另两概念一半，但消退更慢；高/极高需求下分布式每航班冲突数比其他概念高约一个数量级，侵入差异远小于冲突差异。
+混合概念专用解脱层使可巡航垂直空间仅为集中概念一半；所有密度下其侵入最少，但需求延误较高，且高密度下延误分散也高于集中概念。</x:v>
+      </x:c>
+      <x:c r="E13" s="4" t="str">
+        <x:v>作者在Sec. V明确指出对照并非只改变中心化程度；水平空域结构、巡航/解脱层空间和航路偏好共同影响安全与容量。
+风扰动仅取均匀风场沿航向分量来改变速度/时间，不含侧风；这是作者在Sec. III-E声明的有限风效应仿真。
+结论提出改进混合方案的路径规划及放松战略规划以容纳更高密度；当前混合方案安全收益伴随路径效率和延误代价。</x:v>
+      </x:c>
+      <x:c r="F13" s="4" t="str">
+        <x:v>全文评价：分布式概念已有中央监测成本与可选个体重规划。各对照同时改变水平结构、职责及可巡航空间，作者明确不能全归因中心化；混合侵入更少伴随绕行和延误，冲突与侵入差异不可互换，不能单独识别单一引导因素（PDF pp.2–8）。</x:v>
+      </x:c>
+      <x:c r="G13" s="4" t="str">
+        <x:v>公共信息引导与个体决策的直接先例，支持同资源机制分离；不把中心化或结构标签当单因素因果证据。</x:v>
+      </x:c>
+      <x:c r="H13" s="11" t="str">
+        <x:v>FULL_TEXT</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="206" customHeight="1">
+      <x:c r="A14" s="4" t="str">
         <x:v>B01</x:v>
       </x:c>
-      <x:c r="B12" s="4" t="str">
+      <x:c r="B14" s="4" t="str">
         <x:v>Macroscopic Fundamental Diagram for Airplane Traffic: Empirical Findings（2025）</x:v>
       </x:c>
-      <x:c r="C12" s="4" t="str">
+      <x:c r="C14" s="4" t="str">
         <x:v>方法：将 Edie 流量定义扩展到三维空域：以空域体积×时间归一化飞行时间形成密度，以飞机起点到终点的恒高度大圆最短距离形成有效产出，并以有效距离/飞行时间形成有效速度；按 30 min 聚合 ADS-B 轨迹构造产出-密度 MFD，同时将实际航迹长度与有效航迹长度分开以分解速度损失和绕行损失。
 场景/设定：Amsterdam Schiphol 附近五个荷兰 CTA 合并区域，面积 42,807 km²，高度 5,500-19,500 ft，体积 182,667 km³；使用 Delft 接收的 ADS-B 数据，覆盖 2019 年 4 月、8 月和 2020 年 4 月、8 月，包含进出 Schiphol 及邻近机场的航班；单个 30 min 聚合区间通常有 60 架以上飞机。</x:v>
       </x:c>
-      <x:c r="D12" s="4" t="str">
+      <x:c r="D14" s="4" t="str">
         <x:v>主要结论：观测到密度增大时有效速度下降，但在观测密度范围内产出仍随密度增加，没有达到道路交通中常见的流量下降分支。速度损失是产出下降的主要来源，航迹绕行造成的效率损失较小。作者将现有机场运行中的地面等待、holding stack、主动放行与最低飞行速度视为类似 perimeter control 的机制。
 定量结果：观测密度约 0-0.0002 架/km³；基于 5 nmi 水平和 ±1000 ft 垂直间隔的理论紧密填充上限约 0.0051 架/km³（PDF p.9，正文 p.7）。
 拟合 Greenshields 抛物线的自由流速度为 442 km/h（239 knots）；拟合的 jam density 为 7.8×10^-4 架/km³，最大流量对应密度为 3.9×10^-4 架/km³（PDF pp.9-10，正文 pp.7-8）。
 低密度区的 free-flow efficiency 略高于 80%；2020 年 4 月航班量比 2019 年 4 月少 87%；邻近机场相关航班平均约占研究空域航班 17%（PDF pp.7-8、10）。</x:v>
       </x:c>
-      <x:c r="E12" s="4" t="str">
+      <x:c r="E14" s="4" t="str">
         <x:v>研究聚合了几个月内的全部运行条件；恶劣天气、强风、天气单元导致的可用空域减少、改航会改变容量和地速。
 研究将 CTA 交通孤立处理，未显式分离跑道资源限制、终端区不同机型尾流间隔等会影响 CTA 的约束；作者建议按类别拆分数据或用仿真继续研究（PDF pp.11-12，正文 pp.9-10）。
 研究区域相对大且主要航路占用空间有限，当前观测密度未达到最大流量区；作者指出更靠近机场可能更密集，但会更受结构化和集中管制影响（PDF pp.10-11，正文 pp.8-9）。</x:v>
       </x:c>
-      <x:c r="F12" s="4" t="str">
+      <x:c r="F14" s="4" t="str">
         <x:v>全文评价：实测常规航空数据是重要证据，但观测范围未进入拥堵下降支，拟合的临界密度不能当实测容量；受管制机场的三维交通也不能直接代表低空多旋翼交通。</x:v>
       </x:c>
-      <x:c r="G12" s="4" t="str">
-        <x:v>借鉴变量定义及有效产出测量，审慎迁移基本图。</x:v>
-      </x:c>
-      <x:c r="H12" s="11" t="str">
-        <x:v>FULL_TEXT</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13" ht="276" customHeight="1">
-      <x:c r="A13" s="4" t="str">
+      <x:c r="G14" s="4" t="str">
+        <x:v>聚合测量与有效产出定义参考，区分观测区间、拟合临界值和真实容量。</x:v>
+      </x:c>
+      <x:c r="H14" s="11" t="str">
+        <x:v>FULL_TEXT</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="276" customHeight="1">
+      <x:c r="A15" s="4" t="str">
         <x:v>B02</x:v>
       </x:c>
-      <x:c r="B13" s="4" t="str">
+      <x:c r="B15" s="4" t="str">
         <x:v>Complexity optimal air traffic assignment in multi-layer transport network for Urban Air Mobility operations（2022）</x:v>
       </x:c>
-      <x:c r="C13" s="4" t="str">
+      <x:c r="C15" s="4" t="str">
         <x:v>方法：在给定三维双向多层网络上，将各OD需求的路径份额作为战略静态分配变量。以密度加权WMMSE分别拟合节点汇聚/发散的三维线性动力系统，使用特征值与能量加权流量形成网络复杂度目标。约束包含份额守恒、最小有效流、路径航程/续航，以及相对最短能量分配的加权能耗预算；先用模拟退火搜索，再用Dafermos边际成本转移改进，求启发式解（PDF pp.2–10 §2–4，P1、Algorithm1）。
 场景/设定：新加坡包裹配送固定网络：63节点、110链路、24组OD、3水平层，含3个droneport、5个配送站和55个waypoint，层距15 m且有垂直连接。Case1为随OD序号增长的对称双向需求，Case2为不平衡随机需求；同类航空器水平120 km/h、垂直5 km/h，最大航程20 km、续航2000 s。每种非AON算法运行100个随机种子，与AON、SA、DA、MSA等比较（PDF pp.10–13 §5，Table2–4）。</x:v>
       </x:c>
-      <x:c r="D13" s="4" t="str">
+      <x:c r="D15" s="4" t="str">
         <x:v>主要结论：两阶段分配降低节点LDS复杂度，将双向OD分往不同路径并分散至多层；中部及垂直连接节点改善明显，低层仍是主要拥堵层。复杂度是代理目标，其下降不等于实际冲突或间隔违规下降；实验输出为路径流、复杂度、时间、距离及加权能量，并未实施微观解脱反馈。全文已纳入航程、续航和能耗约束，但未引入逐机动态SOC；相较最短路AON，降低复杂度伴随更长路径和更高能耗（PDF pp.3–6、12–19）。
 定量结果：PDF p.13 Table3：Case1相对随机初始分配的复杂度680081.00降至65005.20，降幅90.44%±0.53%（95%CI）；两阶段总耗时13.62±0.52 s，100种子。
 PDF p.13 Table4：Case2相对随机初始复杂度665702.86降至52450.41，降幅92.12%±0.35%（95%CI）；总耗时14.12±0.33 s，100种子。
 PDF p.13 Table3：Case1方案平均航程10.27±0.08 km、时间323.83±2.52 s、加权能量184.68±1.43；AON分别7.16 km、248.00 s、130.27，指标及比较对象不可互换。
 PDF p.13 Table4：Case2方案平均10.39±0.06 km、328.58±1.84 s、加权能量179.49±1.11；AON为7.48 km、258.21 s、131.06。能量数值为模型加权指标，非kWh或SOC。</x:v>
       </x:c>
-      <x:c r="E13" s="4" t="str">
+      <x:c r="E15" s="4" t="str">
         <x:v>选址与新加坡网络构建受运行和地理限制；动态时变需求、多目标噪声/延误、多类别交通和更大网络列为未来工作（PDF p.19 Conclusion）。
 非可分、高维NP-hard问题采用启发式求合理时间内的优质解；SA/DA收敛受初解及非严格凸性影响，不给全局最优保证（PDF pp.6、9）。
 模型假设配送站与droneport可充电/补给维护；若不成立，航程和续航限制还须覆盖返程（PDF pp.3–4 §2.2）。</x:v>
       </x:c>
-      <x:c r="F13" s="4" t="str">
-        <x:v>全文评价：已有航程、续航及能耗预算，不能说忽视能量。静态路径份额优化及LDS复杂度降幅不等于真实冲突降幅，且相对最短路航程、时间与加权能耗可能增加；其约束仍不同于逐机动态SOC及终端资源执行（PDF pp.3–6、13、19）。</x:v>
-      </x:c>
-      <x:c r="G13" s="4" t="str">
-        <x:v>作为战略网络分配参考，保留复杂度、航程与能耗权衡，区分聚合预算与逐机动态SOC/终端资源约束。</x:v>
-      </x:c>
-      <x:c r="H13" s="11" t="str">
-        <x:v>FULL_TEXT</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14" ht="276" customHeight="1">
-      <x:c r="A14" s="4" t="str">
+      <x:c r="F15" s="4" t="str">
+        <x:v>全文评价：已有航程、续航和能耗预算。静态路径份额和LDS复杂度降幅不等于真实冲突降幅，相对最短路的航程、时间及加权能耗可能增加；网络预算不等于动态连续执行保障（PDF pp.3–6、13、19）。</x:v>
+      </x:c>
+      <x:c r="G15" s="4" t="str">
+        <x:v>战略分配和复杂度代理参考，保留航程/能耗权衡，明确与局部软引导尺度不同。</x:v>
+      </x:c>
+      <x:c r="H15" s="11" t="str">
+        <x:v>FULL_TEXT</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="276" customHeight="1">
+      <x:c r="A16" s="4" t="str">
         <x:v>B03</x:v>
       </x:c>
-      <x:c r="B14" s="4" t="str">
+      <x:c r="B16" s="4" t="str">
         <x:v>A quasi-dynamic air traffic assignment model for mitigating air traffic complexity and congestion for high-density UAM operations（2023）</x:v>
       </x:c>
-      <x:c r="C14" s="4" t="str">
+      <x:c r="C16" s="4" t="str">
         <x:v>方法：提出准动态空中交通分配QATA，在预先已知时变OD需求、给定节点和备选路径下，将规划时域分为等长区间，按自由流旅行时间传播前段残余流。采用滚动时域反复求修改静态分配，目标结合密度加权三维LDS复杂度、线性能量加权流与二次拥堵成本；并行模拟退火增量计算节点成本并在候选路径间转移流。份额守恒、最小有效流和链路进出容量约束作用于聚合流，非逐机连续轨迹（PDF pp.4–12 §2–3，Algorithms1–2）。
 场景/设定：预设计新加坡包裹配送网络含332节点、745链路、7个vertiport、12个配送站和84组OD；150/175/200/225/250 ft五层，垂直连接受限，采用多样K最短路径。仿真文本给09:00–15:00六个需求时段；同类航空器水平54 km/h、垂直15 km/h，链路容量15000 veh/h、最小有效流20 veh/h。Java在i7-12700H/16 GB上运行100个随机种子，比较PSA及DA等代表算法（PDF pp.13–16，Tables2–4）。</x:v>
       </x:c>
-      <x:c r="D14" s="4" t="str">
+      <x:c r="D16" s="4" t="str">
         <x:v>主要结论：优化随时段改变路径份额、更多使用中间层，降低总复杂度与拥堵，但部分链路可能更拥堵。预知需求和名义速度下的残余传播使静态分配带有时间维度；论文并未展示感知实际需求、微观避碰偏差再反馈重分配的闭环。能量以飞行阶段和距离权重进入拥堵代价，无动态SOC。复杂度/拥堵改善同时存在平均航程与旅行时间增长，不能将计算时间解释为逐机实时或把代理指标降幅当冲突率降幅（PDF pp.6–9、15–20）。
 定量结果：PDF p.15 Table4：100种子下PSA总目标67157.45±146.87，相对初始99081.42±368.48降低32.20%±0.29%；耗时143.47±3.74 s，均95%CI，属整个聚合分配实验。
 PDF p.15 Table4：PSA复杂度302743.55±1574.53，初始585380.95±3627.11；拥堵40981.22±36.90，初始45048.14±27.92。二者均为模型指标，不是实测冲突次数。
 PDF p.15 Table4：PSA时间1233.61±0.48 s、航程18.28±0.01 km，初始1201.94±0.41 s、17.84±0.01 km；DA为1198.18±0.38 s、17.78±0.01 km。
 PDF pp.14–15 §4.1.1：1–20线程各计时10000次转移，约3倍加速，8线程后无明显继续改善；此为转移计算加速，非逐机闭环周期。</x:v>
       </x:c>
-      <x:c r="E14" s="4" t="str">
+      <x:c r="E16" s="4" t="str">
         <x:v>私人PSU/USS参与集中式信息共享的动机和机制尚不明确；多实体联合运行需要更成熟技术（PDF p.20 §5.1）。
 将QATA输出交给拉格朗日个体航班优化属于明确未来工作；本文仅给预飞战略路径流模式（PDF pp.2、20）。
 低空障碍限制预设计替代路线，传统动态分配的凸性/解析成本条件不完全成立；算法对照为代表性而非穷尽比较（PDF pp.9、13、15）。</x:v>
       </x:c>
-      <x:c r="F14" s="4" t="str">
+      <x:c r="F16" s="4" t="str">
         <x:v>全文评价：预先已知时变需求的准动态分配不等于实际感知和避碰闭环。固定自由速度、容量约束、代理指标及路径增长限制外推；微观个体优化被作者明确列为未来，不能将143 s聚合分配求解称为逐机实时（PDF pp.4–12、15、20）。</x:v>
       </x:c>
-      <x:c r="G14" s="4" t="str">
-        <x:v>用于比较预飞时变分配与实际运行反馈的接口，保留名义传播、计算时域和效率代价条件。</x:v>
-      </x:c>
-      <x:c r="H14" s="11" t="str">
-        <x:v>FULL_TEXT</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15" ht="262" customHeight="1">
-      <x:c r="A15" s="4" t="str">
+      <x:c r="G16" s="4" t="str">
+        <x:v>预飞时变分配与反馈接口参考，保留需求先验、名义传播和求解时域条件。</x:v>
+      </x:c>
+      <x:c r="H16" s="11" t="str">
+        <x:v>FULL_TEXT</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="262" customHeight="1">
+      <x:c r="A17" s="4" t="str">
         <x:v>B04</x:v>
       </x:c>
-      <x:c r="B15" s="4" t="str">
+      <x:c r="B17" s="4" t="str">
         <x:v>Airspace Congestion, flow Relations, and 4-D fundamental Diagrams for advanced urban air mobility（2024）</x:v>
       </x:c>
-      <x:c r="C15" s="4" t="str">
+      <x:c r="C17" s="4" t="str">
         <x:v>方法：以气体动理论近似建立密度—成对预测冲突—速度损失—有效流量的宏观链条。随机均匀航向给出相对速度近似，冲突数随密度平方、间隔截面和探测前视时间变化；通过每次冲突平均速度损失构造实际/有效速度及基本图，再用微观仿真标定与验证。微观解脱采用按冲突程度顺序执行的分散式非线性优化，调航向与速度、允许悬停；本文做模型识别而非滚动分配控制（PDF pp.3–7、11–14，式1–16）。
 场景/设定：无结构空域中，在围绕中心测量区的圆周交替配置起终vertiport以近似随机航向；正态出发时刻产生密度升降。每次仿真5000 s，按300 s窗口聚合；间隔和最大速度各设五档，速度80/100/120/150/180 mph。尽管模拟器有三维起降过程，测量区刻意排除起降影响，巡航全部同高度且禁止垂直绕行；冲突数实验关闭解脱而保留探测，速度/流量实验启用解脱（PDF pp.11–18 §5，Figs12–20）。</x:v>
       </x:c>
-      <x:c r="D15" s="4" t="str">
+      <x:c r="D17" s="4" t="str">
         <x:v>主要结论：理论与仿真均显示密度增加导致实际/有效速度非线性下降；间隔增大带来更大速度损失、更低容量与临界密度。提高最大速度改善低密度出流，但临界密度下降，高密度速度趋同。模型已有微观冲突探测与解脱验证，冲突却指预测侵入分离包络，并非碰撞或实际LOS。各参数下拟合质量不一致，随机航向均值近似和二维巡航设定限制向强方向结构化终端外推（PDF pp.4–7、13–20）。
 定量结果：PDF pp.13–14 Figs12–13：间隔0.5556/0.4444/0.3333 mile时冲突—密度拟合R²为0.912/0.889/0.869；180/150/120/100/80 mph时为0.819/0.810/0.914/0.925/0.922。
 PDF p.16 Fig15：间隔按0.5556至0.1111 mile五档递减，实际速度—密度R²为0.888/0.931/0.802/0.914/0.567；不能概括所有场景均高拟合。
 PDF p.17 Figs17–18：有效速度—密度R²在五档间隔下为0.864/0.885/0.709/0.926/0.657，在180至80 mph五档下为0.836/0.747/0.828/0.864/0.930。
 PDF p.18 Fig19：有效流—密度R²在间隔0.5556/0.4444/0.3333/0.2222/0.1111 mile时为0.870/0.927/0.524/0.963/0.971；为拟合优度，不是容量或安全改善百分比。</x:v>
       </x:c>
-      <x:c r="E15" s="4" t="str">
+      <x:c r="E17" s="4" t="str">
         <x:v>只适用于无结构随机航向空域；向结构化走廊扩展须修改相对速度项并重新测试（PDF pp.4、18–20 §3.3、6–7）。
 验证实际为同高度二维巡航，禁止高度解脱；简化模拟器未纳入航空器物理/加速度，个体航迹保真度有限（PDF pp.12、19–20）。
 高密度AAM实测数据不足，采用仿真而非真实运行验证；每次冲突的平均速度损失仍需标定（PDF pp.11、14、19）。</x:v>
       </x:c>
-      <x:c r="F15" s="4" t="str">
-        <x:v>全文评价：随机航向无结构空域的均值近似，以及同高度二维、未含物理加速度的模拟，限制向结构化终端强方向流外推。该文已用微观冲突探测/解脱验证，不能说完全无微观；也不应仅以新增FD本身作为贡献（PDF pp.4–7、11–14、19–20）。</x:v>
-      </x:c>
-      <x:c r="G15" s="4" t="str">
-        <x:v>作为平均流机理和参数敏感性参考，迁移到方向性终端流时需检验其适用条件，而非重复提出基本图。</x:v>
-      </x:c>
-      <x:c r="H15" s="11" t="str">
-        <x:v>FULL_TEXT</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16" ht="304" customHeight="1">
-      <x:c r="A16" s="4" t="str">
+      <x:c r="F17" s="4" t="str">
+        <x:v>全文评价：相对航向、解脱算法与每冲突速度损失已有机理和微观验证；随机航向、同高度二维和未含物理加速度限制结构化强方向流外推。作者明确应改相对速度项并进一步测试，方向影响或新增FD本身不足为贡献（PDF pp.4–7、11–14、19–20）。</x:v>
+      </x:c>
+      <x:c r="G17" s="4" t="str">
+        <x:v>相对航向、冲突及速度损失的核心机理依据，检验强方向流下条件供给的适用范围。</x:v>
+      </x:c>
+      <x:c r="H17" s="11" t="str">
+        <x:v>FULL_TEXT</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="304" customHeight="1">
+      <x:c r="A18" s="4" t="str">
         <x:v>B05</x:v>
       </x:c>
-      <x:c r="B16" s="4" t="str">
+      <x:c r="B18" s="4" t="str">
         <x:v>Macroscopic Fundamental Diagrams for Low-Altitude Air city Transport（2023）</x:v>
       </x:c>
-      <x:c r="C16" s="4" t="str">
+      <x:c r="C18" s="4" t="str">
         <x:v>方法：以分散式人工势场和Lyapunov型吸引/屏障函数控制逐机速度，采用位置—速度动力学、速度饱和及滤波位置，在安全、避让、探测空间约束下实现waypoint或目的地线/平面到达。将轨迹按广义Edie定义聚合为流量、密度、速度、累积与完成出流，拟合指数型MFD。微观仿真0.5 s、聚合60 s同步运行；本篇建立识别平台，MFD网络反馈控制列为未来，但附录已有安全检查引起的起飞排队（PDF pp.3–10、20、22–24）。
 场景/设定：固定无结构网络内起终点在边界均匀随机，无预设航路/交叉口；默认最大速度20 m/s、加速度5 m/s²，安全/避让/探测半径15/22.5/45.5 m，梯形需求、一般运行1.5 h。六组实验比较2×2、1×1、0.5×0.5 km二维网络，10/15/20 m安全半径，随机半径与速度异质性，waypoint与目的地线，以及0.5×0.5×0.1 km三维网络；三维运行0.5 h（PDF pp.9–16 §4）。</x:v>
       </x:c>
-      <x:c r="D16" s="4" t="str">
+      <x:c r="D18" s="4" t="str">
         <x:v>主要结论：完整MFD在多种设置下均出现自由流和拥堵支；安全半径增大使容量/临界密度下降，异质半径和速度增加速度基本图散布。动态加载已经观察滞回，三维场景临界附近散布更大，拥堵可更快出现和消散；目的地线因放宽到达点而提高出流。拥堵中仍有局部避让移动，所以绝对流量Q可非零而完成出流G为零。固定几何中的情景比较不等于在线重构，拟合峰值也须与单点观测区分（PDF pp.11–20）。
 定量结果：PDF p.12 Fig9：2×2 km waypoint观测临界点为229架、1.8667架/s，而拟合曲线峰值为283.86架、1.47架/s；两者不得混写。
 PDF p.18 Table2：同rs=15 m、vmax=20 m/s时，2×2/1×1/0.5×0.5 km拟合临界累积为283.86/80.49/21.57架，峰值出流1.47/0.80/0.45架/s。
@@ -1006,298 +1070,298 @@
 PDF p.18 Table1：同0.5×0.5 km、rs15、vmax20，waypoint与目的地线峰值0.45/0.54架/s，临界累积21.57/22.62架；不是共同到达点不变的纯算法收益。
 PDF p.18 Table2：三维0.5×0.5×0.1 km waypoint拟合临界累积42.00架、峰值1.10架/s；为仿真拟合，不是实测容量。</x:v>
       </x:c>
-      <x:c r="E16" s="4" t="str">
+      <x:c r="E18" s="4" t="str">
         <x:v>全部测试网络无结构；结构化空域及其容量影响为未来方向（PDF p.20 §5）。
 本文使用人工势场避碰，未来应比较其他微观模型和避碰方法（PDF pp.19–20 §5）。
 先进MFD网络控制策略为后续研究；滞回机理仍在持续研究（PDF p.12 §4.2.1、p.20 §5）。
 显式假设边界：航空器充分可控、探测范围足够、初始滤波位置安全分离、静态目标点满足分离条件，方支撑所述避碰/收敛性质（PDF pp.4–7，Assumptions1–5）。</x:v>
       </x:c>
-      <x:c r="F16" s="4" t="str">
-        <x:v>全文评价：已做异质机群、动态加载/滞回和3D，不能再将这些笼统列为空白。具体局部人工势场与无结构网络决定了模型条件；结构化共享服务资源和有限等待预算下能否保持简洁聚合关系，仍须检验（PDF pp.4–7、10–20）。</x:v>
-      </x:c>
-      <x:c r="G16" s="4" t="str">
-        <x:v>用于约束宏微观建模创新边界，比较结构化共享服务资源、有限等待预算下的聚合行为。</x:v>
-      </x:c>
-      <x:c r="H16" s="11" t="str">
-        <x:v>FULL_TEXT</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17" ht="262" customHeight="1">
-      <x:c r="A17" s="4" t="str">
+      <x:c r="F18" s="4" t="str">
+        <x:v>全文评价：已研究异质、动态加载/滞回、3D及到达指导规则变化后的MFD。destination line放宽单点到达要求，不能当作同任务的纯算法收益；APF和无结构场景决定其条件（PDF pp.4–7、10–20）。</x:v>
+      </x:c>
+      <x:c r="G18" s="4" t="str">
+        <x:v>条件MFD、指导规则变化及滞回的直接基础，新贡献需同任务同资源和跨需求验证。</x:v>
+      </x:c>
+      <x:c r="H18" s="11" t="str">
+        <x:v>FULL_TEXT</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="262" customHeight="1">
+      <x:c r="A19" s="4" t="str">
         <x:v>B06</x:v>
       </x:c>
-      <x:c r="B17" s="4" t="str">
+      <x:c r="B19" s="4" t="str">
         <x:v>Urban low-altitude air transport management: Bridging dynamic traffic control and static network equilibrium（2025）</x:v>
       </x:c>
-      <x:c r="C17" s="4" t="str">
+      <x:c r="C19" s="4" t="str">
         <x:v>方法：先将乘客OD、起降vertiport组合聚合为链路流，以固定接驳/巡航时间和随流增长的起降等待成本求弹性需求系统最优SO分配。再按区域建立准入点队列与MFD累积动力学，从SO导出准入容量和自由流支目标累积；最大吞吐排队控制与内外生出流份额耦合的MBC共同调节，需求模式改变时重算目标。主控制实验更新聚合方程；另以逐机差异速度示例展示流量调节潜力，但详细MBC到速度映射留待未来（PDF pp.6–13、20–21）。
 场景/设定：跨河/海两区域概念网络，8个固定vertiport、4组OD，两空域均2×2×1 km且采用full mix；假设起降独立并可同时进行、航空器有避碰与留区能力。MFD由此前1 km立方体微观轨迹拟合并按面积扩展。两组120 min聚合实验在60 min切换工作日/假日模式，与固定初始SO目标比较；同控制器、峰值需求超目标20%、0.5%高斯噪声。附录另有两区域各9六角柱单元的900 s微观速度试验（PDF pp.5–6、13–21）。</x:v>
       </x:c>
-      <x:c r="D17" s="4" t="str">
+      <x:c r="D19" s="4" t="str">
         <x:v>主要结论：随需求模式调整SO目标能匹配准入容量，在上调需求时降低队列并增加完成出流；下调时避免追踪过高目标。收敛证明限于需求过饱和、初态自由流及给定MFD等条件，不直接保证逐机轨迹可执行。已有起降等待模型、分vertiport子队列讨论及微观速度实验，不能称完全没有终端或微观；附录只显示限速改变后内外生完成流的方向性响应，尚未给出MBC输入到逐机速度的完整闭环映射（PDF pp.8–13、16–23）。
 定量结果：PDF p.16 §4.2.1：120 min工作日→假日、60 min改目标的方案，相对始终固定工作日SO基线，平均排队时间降低42.3%、最大队长降低52.6%、最大完成流提高26.9%；同控制器、同需求。
 PDF p.15：工作日/假日目标累积分别(43.6,36.3)/(82.8,69.0)架；两区域临界累积110.4架，所选目标不是直接设为MFD临界点。
 PDF pp.14–15：工作日准入容量四分量(0.108,0.245,0.160,0.048)架/s，假日(0.157,0.300,0.245,0.114)架/s；由各SO分配聚合而来。
 PDF pp.20–21 Appendix A：内/外生流入各0.5架/s，前450 s均限20 m/s，之后限10/30 m/s；450–600 s内生完成流下降、外生上升，未报告闭环映射或该试验的百分比增益。</x:v>
       </x:c>
-      <x:c r="E17" s="4" t="str">
+      <x:c r="E19" s="4" t="str">
         <x:v>详细MBC微观实现机制留未来；附录以条件语气说明若能把控制量映到限速，才可完成微观执行（PDF p.10 §2.3.2、pp.20–21 Appendix A）。
 独立起降假设忽略二者资源交互，依赖航空器较强避碰能力；需求简化为一系列稳定/周期常值模式（PDF pp.5–6）。
 静态规划把接驳/巡航/离场时间视为常值，忽略巡航拥堵增长；作者假定规划准入不导致空中拥堵（PDF p.6 §2.2）。
 收敛结论要求过饱和需求与不拥堵初态；作者提出可用MPC等改善瞬态（PDF p.13 Proposition2；pp.22–23 Appendix C）。</x:v>
       </x:c>
-      <x:c r="F17" s="4" t="str">
-        <x:v>全文评价：已有起降等待模型、子队列讨论和微观速度示例，不能说完全无终端或微观。起降独立假设及MBC到逐机速度映射尚未完整落实；主宏观稳定性结论受MFD、准入及初态条件约束，不直接保证终端轨迹可执行（PDF pp.5–13、20–23）。</x:v>
-      </x:c>
-      <x:c r="G17" s="4" t="str">
-        <x:v>用于比较SO目标、准入与区域控制如何连接逐机执行，保留其已有等待建模和微观实验。</x:v>
-      </x:c>
-      <x:c r="H17" s="11" t="str">
-        <x:v>FULL_TEXT</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18" ht="234" customHeight="1">
-      <x:c r="A18" s="4" t="str">
+      <x:c r="F19" s="4" t="str">
+        <x:v>全文评价：明确讨论控制改变MFD/容量和需求变化后目标调整，已有起降等待及微观差异速度示例。主实验仍基于聚合动力学，结论受给定MFD、准入和初态约束；详细MBC到逐机速度映射为未来（PDF pp.3、5–13、20–23）。</x:v>
+      </x:c>
+      <x:c r="G19" s="4" t="str">
+        <x:v>控制影响供给、目标调整和准入协同的强对照，区分聚合验证与逐机实现。</x:v>
+      </x:c>
+      <x:c r="H19" s="11" t="str">
+        <x:v>FULL_TEXT</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="234" customHeight="1">
+      <x:c r="A20" s="4" t="str">
         <x:v>B07</x:v>
       </x:c>
-      <x:c r="B18" s="4" t="str">
+      <x:c r="B20" s="4" t="str">
         <x:v>Airspace Partitioning for Urban Air Mobility: A Macroscopic Approach with a Realistic Network（2025）</x:v>
       </x:c>
-      <x:c r="C18" s="4" t="str">
+      <x:c r="C20" s="4" t="str">
         <x:v>方法：对给定单层单向走廊图作静态区域划分，以降低区域内部密度差异、提取低散布NMFD。先用Haversine距离DBSCAN生成空间种子，经密度差与邻近度加权的区域生长建立单元，再用遗传算法将单元分为互斥连通区域，最小化区域内单元平均密度方差并限制区域单元数。BlueSky逐机轨迹形成链路密度和长度加权区域流密度；区域标签调整不改变真实通道，也未实装周界控制（PDF pp.1–3、5）。
 场景/设定：纽约既有FAA直升机航路构建17 vertiport网络，按2023出租车/TNC出行时间节省估计UAM需求。工作日08:00–11:00出发，约11:30排空，4个随机场景；同类可悬停EC-135、500 m固定高度、100 km/h巡航、Dijkstra最短路。战术探测为线性前视、分散式成对减速解脱，h(v)=200 m+20 s×v；原点设最小出发间隔和安全延后。只模拟航路巡航，需求估计中的起降固定时间并非终端仿真（PDF pp.3–5）。</x:v>
       </x:c>
-      <x:c r="D18" s="4" t="str">
+      <x:c r="D20" s="4" t="str">
         <x:v>主要结论：10:15快照产生三分区，其中两个轻载区相似，离线以两分区重跑后合并而保留中心拥堵区；作者认为本场景拥堵空间分布稳定，因此静态区域足够。外围NMFD处于自由流，中心区出现拥堵下降支，长度加权聚合得到较低散布关系。论文展示的是既有走廊上的密度聚类与NMFD识别，不是在线改变空域结构、在途迁移或终端资源调度；未来才考虑不同路径和gating/perimeter控制（PDF pp.5–6，Figs4–7）。
 定量结果：PDF p.5：10:15密度快照、4 min测量窗；DBSCAN MinPts=3、epsilon约2.5 km、theta=0.2，先K=3且每区≤3单元，再K=2且每区≤6单元，均为离线分区。
 PDF pp.5–6 Fig7：每5 s存轨迹、4 min聚合；中心Region2临界密度约0.7–0.9架/km、容量约60架/h；是给定航路/分离/需求下的长度加权区域NMFD。
 PDF pp.4–6：4个同设置随机场景，外围平均密度≤0.5架/km；未报告相对无分区的统一散布改善百分比或控制收益，不能据图虚构降幅。</x:v>
       </x:c>
-      <x:c r="E18" s="4" t="str">
+      <x:c r="E20" s="4" t="str">
         <x:v>只建模en-route走廊，终端区未模拟；多航道、超越区等结构留未来（PDF pp.2–3）。
 详细方式选择超出范围，以简单时间节省门槛估计出租车需求可转化比例（PDF p.4 §III.A）。
 其他参数、路径策略及缓解中心区过饱和的gating/perimeter控制为后续工作；本篇尚未验证这些控制（PDF p.5 Conclusions and Outlook）。</x:v>
       </x:c>
-      <x:c r="F18" s="4" t="str">
-        <x:v>全文评价：静态分区旨在降低NMFD散布，并未模拟终端区；密度聚类不改变真实通道，不能当作在线空域重构。10:15数据快照及稳定拥堵空间图景使其结果的动态外推受限（PDF pp.1–5）。</x:v>
-      </x:c>
-      <x:c r="G18" s="4" t="str">
-        <x:v>明确区分聚合区域标签和实际运行空域构形，作为静态均质化与NMFD识别参考。</x:v>
-      </x:c>
-      <x:c r="H18" s="11" t="str">
-        <x:v>FULL_TEXT</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19" ht="248" customHeight="1">
-      <x:c r="A19" s="4" t="str">
+      <x:c r="F20" s="4" t="str">
+        <x:v>全文评价：静态分区降低NMFD散布，密度聚类不改变真实通道，不是在线物理重构；10:15快照及稳定拥堵空间图景限制动态外推（PDF pp.1–5）。</x:v>
+      </x:c>
+      <x:c r="G20" s="4" t="str">
+        <x:v>区域均质化与NMFD识别参考，区分统计标签和实际组织规则。</x:v>
+      </x:c>
+      <x:c r="H20" s="11" t="str">
+        <x:v>FULL_TEXT</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="248" customHeight="1">
+      <x:c r="A21" s="4" t="str">
         <x:v>B08</x:v>
       </x:c>
-      <x:c r="B19" s="4" t="str">
+      <x:c r="B21" s="4" t="str">
         <x:v>有人机-无人机混合低空交通建模：微观-宏观耦合框架 / Modeling mixed low-altitude traffic of manned aircraft and unmanned aerial vehicles: a micro-macroscopic coupled framework（2026）</x:v>
       </x:c>
-      <x:c r="C19" s="4" t="str">
+      <x:c r="C21" s="4" t="str">
         <x:v>方法：建立 MM-ATM 微观-宏观联合框架：先构造包含制动距离、感知/控制误差、机型速度差和响应时延补偿的结构化静态安全间隔；再用刺激-响应机制和速度差/间距误差反馈建立异构飞行器速度控制；最后把速度与间隔状态离散化，用一阶马尔科夫链稳态分布推导平均速度以及流量-密度-速度三参数基本图。
 场景/设定：二维单层固定中心线航道、单方向纵向运行，不考虑交叉、并线和换层；横向宽度 40 m，典型高度 60-300 m。有人机用 Cessna 172、无人机用翼龙-2 作为性能尺度，Python 3.11 的 MM-ATM 平台仿真 600 s、步长 0.1 s，飞行器数量 0-200 架，每个密度 3 次重复，约 200 次仿真。</x:v>
       </x:c>
-      <x:c r="D19" s="4" t="str">
+      <x:c r="D21" s="4" t="str">
         <x:v>主要结论：混合运行相对同构系统使临界密度右移，高密度出现由动态间隔调节形成的低速稳定平台而非完全速度塌缩；速度匹配和适度间距可同时改善容量与稳定性。研究把微观安全间隔/响应差异明确传到宏观基本图，形成容量评估和策略调参工具。
 定量结果：初始间距为静态阈值的 1.0-1.3 倍、无人机巡航速度约为有人机 110%、响应时延小于 1.5 s 时，在 10-13 架/km 密度区间取得容量与稳定性较优平衡（PDF pp.1-2、10-12，正文 pp.132-133、140-143）。
 无人机速度敏感性设置 33.3-72.2 m/s（120-260 km/h），有人机固定 55.6 m/s；作者建议无人机约 55.6-66.7 m/s 时兼顾容量和稳定性（PDF p.10，正文 p.140）。
 有人机速度设置 52.8-100.0 m/s；作者报告 66.7-72.2 m/s 区间相对兼顾容量和稳定性，高速度会出现流量回落与曲线拉伸（PDF pp.10-11，正文 pp.140-141）。
 仿真覆盖约 10^4 量级稳态样本；高密度响应时间实验显示快速响应可抑制扰动，慢响应会因延迟补偿导致容量受限（PDF pp.8-12，正文 pp.139-143）。</x:v>
       </x:c>
-      <x:c r="E19" s="4" t="str">
+      <x:c r="E21" s="4" t="str">
         <x:v>模型仅考虑二维单层航路，未显式描述三维分层、交汇并线和换层；扩展到三维需处理垂直规则、跨层冲突传播和计算复杂度（PDF p.12，正文 p.143）。
 一阶马尔科夫链可能难以刻画高密度或长队列扰动的长程相关性，适用边界仍需验证（PDF p.12，正文 p.143）。
 宏观稳态依赖遍历性与收敛性假设；提高离散精度会使转移矩阵膨胀，数值稳定性和计算效率尚待系统分析（PDF p.12，正文 p.143）。
 参数主要面向有人机和中大型固定翼无人机，平台参数跨度有限；作者建议引入多等级平台（PDF p.12，正文 p.143）。</x:v>
       </x:c>
-      <x:c r="F19" s="4" t="str">
-        <x:v>全文评价：微观响应经马尔科夫链连接宏观基本图，已直接覆盖耦合建模；但单向中心线交通没有交汇与换层，稳态和一阶记忆假设的边界也限制了向动态终端区迁移。</x:v>
-      </x:c>
-      <x:c r="G19" s="4" t="str">
-        <x:v>中文直接相关研究；可借鉴行为到流量的映射，但不沿用其固定翼参数。</x:v>
-      </x:c>
-      <x:c r="H19" s="11" t="str">
-        <x:v>FULL_TEXT</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20" ht="206" customHeight="1">
-      <x:c r="A20" s="4" t="str">
+      <x:c r="F21" s="4" t="str">
+        <x:v>全文评价：局部响应经马尔科夫链连接宏观基本图已有直接耦合；单向中心线没有交汇/换层，稳态和一阶记忆假设限制向动态多向交通迁移。</x:v>
+      </x:c>
+      <x:c r="G21" s="4" t="str">
+        <x:v>局部行为到聚合关系的直接中文参考，检验单向稳态模型向多向动态交汇的边界。</x:v>
+      </x:c>
+      <x:c r="H21" s="11" t="str">
+        <x:v>FULL_TEXT</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="206" customHeight="1">
+      <x:c r="A22" s="4" t="str">
         <x:v>B09</x:v>
       </x:c>
-      <x:c r="B20" s="4" t="str">
+      <x:c r="B22" s="4" t="str">
         <x:v>Traffic Flow Analysis for Package Delivery Drones using a Queueing Model（2023）</x:v>
       </x:c>
-      <x:c r="C20" s="4" t="str">
+      <x:c r="C22" s="4" t="str">
         <x:v>方法：针对给定交叉航路网络，把相邻飞行器间距和交叉点不同航路的时间间隔约束转化为最大流约束；用 modified max-flow 求每条路线均匀流上界，再把流率变为起飞时隙，并将 depot 建模为队列服务器，比较 FCFS、Round-Robin 和 Random 三种订单处理策略。
 场景/设定：小型 UAS package delivery 的 depot-to-customer 网络，含固定空间 operational-volume blocks、交叉 waypoint、恒定巡航地速和单向巡航阶段；仿真示例含 2 个 depot、4 个 customer、3 个 crossing waypoint，2D 平面网络用于巡航分析；每个 depot 一个 vertipad，假设一次只能起飞一架。</x:v>
       </x:c>
-      <x:c r="D20" s="4" t="str">
+      <x:c r="D22" s="4" t="str">
         <x:v>主要结论：流量上界和队列模型可以把原本组合困难的个体起飞调度转为可分析的战略放行问题。Operational-volume 长度增大时，起飞等待、地面延误和未能发射的订单增加，吞吐下降；在给定按需到达下，FCFS 表现最好，Round-Robin 次之，Random 最差。
 定量结果：仿真将 OV block 长度 L 从 100 m 到 1000 m 以 100 m 递增，固定宽度 W=20 m；每组仿真 10,000 s，depot 订单为平均 100 orders/h 的 Poisson 到达（PDF pp.7-8）。
 随着 L 增大，三种队列策略的 ground delay 和等待队列数上升，能够发射的无人机/订单比例下降；作者报告吞吐在超过 max-flow 密度后快速下降（PDF pp.1、8-9）。
 作者在均匀间隔段落说明交叉点最小时间间隔 Δt 会使每条边至少保持 2×Δt 间隔，并明确将所计算的均匀流解表述为真实最优解的 upper bound，因为流被过度约束；全文检索未见 lower bound 表述（PDF p.3）。</x:v>
       </x:c>
-      <x:c r="E20" s="4" t="str">
+      <x:c r="E22" s="4" t="str">
         <x:v>网络和 operational-volume 位置固定，研究只处理时间去冲突，不处理空间网络/空域构形优化；巡航后固定地速，不进行途中速度调整（PDF pp.2-3）。
 作者明确指出均匀流假设使流被过度约束，并说明非均匀流允许通过调整各无人机起飞时间形成任意相邻间隔；本文未研究该全局组合优化，作者因此把所计算均匀流解称为真实最优解的 upper bound（PDF p.3）。
 假设 depot 永远有可用无人机、仅有 depot-to-customer 单向流，忽略返程和闭合无人机状态；作者将返程、闭合模型、不同网络、多 vertipad 同时运行、双向流等列为未来工作（PDF pp.4、9）。
 采用同一类型无人机、恒定速度和固定 OV blocks，并把 wind/不确定性通过额外时间间隔留作扩展，未在本文验证异构性能和环境扰动（PDF pp.1-3、9）。</x:v>
       </x:c>
-      <x:c r="F20" s="4" t="str">
+      <x:c r="F22" s="4" t="str">
         <x:v>全文评价：等间隔巡航流、固定网络与无限可用无人机简化了真实闭合配送系统；非均匀放行和途中调速未覆盖。文中的界限表述需结合目标与约束理解，不直接当任意调度的容量上界。</x:v>
       </x:c>
-      <x:c r="G20" s="4" t="str">
-        <x:v>简单可复现的排队与放行基线，可用于评估复杂算法是否必要。</x:v>
-      </x:c>
-      <x:c r="H20" s="11" t="str">
-        <x:v>FULL_TEXT</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="21" ht="234" customHeight="1">
-      <x:c r="A21" s="4" t="str">
+      <x:c r="G22" s="4" t="str">
+        <x:v>可复现的排队与放行基线，检验联合引导是否超出简单准入的增益。</x:v>
+      </x:c>
+      <x:c r="H22" s="11" t="str">
+        <x:v>FULL_TEXT</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="234" customHeight="1">
+      <x:c r="A23" s="4" t="str">
         <x:v>B10</x:v>
       </x:c>
-      <x:c r="B21" s="4" t="str">
+      <x:c r="B23" s="4" t="str">
         <x:v>Analysis of Traffic Flow in Structured Urban Airspace Networks With MFD-Based Feedback Control（2024）</x:v>
       </x:c>
-      <x:c r="C21" s="4" t="str">
+      <x:c r="C23" s="4" t="str">
         <x:v>方法：在 BlueSky 快时域微观仿真中建立带多车道和换道行为的结构化城市空域网络，按 5 min 滑动窗口用 Edie 型定义提取 flow、speed、occupancy MFD；依据 MFD 选 occupancy setpoint，再在各 source vertiport 配置去中心化 departure-metering PI 控制器，并用 holding function 比较 open-loop 与闭环放行。
 场景/设定：4 km² lattice multi-lane sky corridor，lane spacing 200 m、纵向邻近节点间距 2 km；source vertiports 0/5/10，destination 4/9/14；每个 source 的小时需求 50、150、400 veh/h 分段升降，最大 400 veh/h。仿真步长 0.05 s，1 Hz 采样，单一 Amazon Drone 类型，不计风，不施加到达率限制。</x:v>
       </x:c>
-      <x:c r="D21" s="4" t="str">
+      <x:c r="D23" s="4" t="str">
         <x:v>主要结论：结构化多车道场景出现 flow-occupancy 低散布线性段和约 600 veh/h 的饱和段，60 vehicles 被选为 occupancy setpoint。去中心化放行计量可把网络车辆占用维持在 setpoint 附近，减少 holding 峰值并平滑到达率，但代价是吞吐和出发队列上升。
 定量结果：MFD 在 occupancy 0-60 vehicles 时 flow 近似线性增至 600 veh/h，之后散布增大并在约 600 veh/h 饱和；据此选择 60 vehicles setpoint（PDF pp.9-10）。
 无控制时总 departure 在第 10 h 超过 5000 vehicles、峰值 departure rate 超过 800 veh/h；控制后总 departure 略超 2500、departure rate 稳定约 275 veh/h（PDF pp.10-11）。
 无控制时 source queues 峰值约 450/300/100 vehicles；控制后约 1400/1000/400 vehicles（PDF p.11）。
 无控制时 total occupancy 在第 6 h 短暂约 140、holding 最多约 60；控制后 total 近似恒定，holding 平均约 8，holding 峰值约减少 80%，arrival throughput 约减少 20%（PDF pp.12-13）。</x:v>
       </x:c>
-      <x:c r="E21" s="4" t="str">
+      <x:c r="E23" s="4" t="str">
         <x:v>作者未来工作要求更真实、更复杂、更大规模场景，并在 vertiports 施加 arrival-rate limits。
 作者提出应研究天气导致的 dynamic network configurations，以及更高效的 conflict detection/resolution 以加快数据生成。
 当前 holding 用固定且可重置的 holding time 近似，作者建议改为显式 holding zone（PDF p.13，Conclusion/Future work）。
 实验仅使用一种 Amazon Drone、固定 200 m departure separation、无风、无 vertiport arrival-rate limit，且研究场景只有一个 MFD、未做网络分区（PDF pp.8-10）。</x:v>
       </x:c>
-      <x:c r="F21" s="4" t="str">
-        <x:v>全文评价：减少空中holding伴随吞吐下降和地面队列增加，不能称所有效率指标同时改善。未限制到达服务率、holding被简化，需在完整排队成本和起降瓶颈下重评估。</x:v>
-      </x:c>
-      <x:c r="G21" s="4" t="str">
-        <x:v>对照价值很高，直接支持同时计算空中与外部等待并保留负结果。</x:v>
-      </x:c>
-      <x:c r="H21" s="11" t="str">
-        <x:v>FULL_TEXT</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="22" ht="262" customHeight="1">
-      <x:c r="A22" s="4" t="str">
+      <x:c r="F23" s="4" t="str">
+        <x:v>全文评价：减少空中holding伴随吞吐下降和地面队列增加，不能称所有效率指标同时改善。未限制到达服务率且holding被简化，结论受其排队统计和服务假设约束。</x:v>
+      </x:c>
+      <x:c r="G23" s="4" t="str">
+        <x:v>准入控制效率代价对照，完整计入外部/内部等待、吞吐与未完成任务。</x:v>
+      </x:c>
+      <x:c r="H23" s="11" t="str">
+        <x:v>FULL_TEXT</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="262" customHeight="1">
+      <x:c r="A24" s="4" t="str">
         <x:v>B11</x:v>
       </x:c>
-      <x:c r="B22" s="4" t="str">
+      <x:c r="B24" s="4" t="str">
         <x:v>Traffic flow modeling and feedback control for future Low-Altitude Air city Transport: An MFD-based approach（2021）</x:v>
       </x:c>
-      <x:c r="C22" s="4" t="str">
+      <x:c r="C24" s="4" t="str">
         <x:v>方法：先以双积分逐机模型、30 s前视轨迹共享及BARON协调解脱仿真识别MFD；再把固定多层/多区域的虚拟网关流写成守恒动力学，包含输入/状态时延与非线性交互。基于局部线性化模型设计分散式自适应MRAC，使用区域状态/跟踪误差反馈，并按阈值事件触发采样保持网关控制。证明在A1–A4下信号有界、误差渐近趋零且无Zeno；主控制测试为聚合模型，并未给逐机命令转换（PDF pp.5–12、16–18）。
 场景/设定：MFD识别为100 m边长正方形，起终点在不同边；well-clear 15 m、速度上限20 m/s、加速度5 m/s²、前视30 s，不安全起飞者在区外悬停后重试。各恒定流入运行30 min，最高65架/min，每30 s估计后整次平均。控制测试另设两层共3聚合区，MFD比例G2=0.8G1、G3=1.2G1，按0.85倍临界累积局部线性化并归一化/缩放时间；比较两组事件阈值，同控制器不重调（PDF pp.6、12–15）。</x:v>
       </x:c>
-      <x:c r="D22" s="4" t="str">
+      <x:c r="D24" s="4" t="str">
         <x:v>主要结论：微观仿真支持完成出流—累积的MFD及拥堵支；鲁棒分散式边界反馈则在区域动力学与时延、扰动假设下验证跟踪。已有微观识别与宏观反馈，不能再把二者概念本身当空白；但两阶段并非B12式微观plant与个体命令的完整闭环。控制实验报告跟踪误差、控制量、需求和等效扰动，未给TTS及空地等待分解；式中时延主要为控制/状态/通信延迟，不等于航班排队延误（PDF pp.5–6、9–16）。
 定量结果：PDF pp.12–13 §5：三区域测试选ncr1=80架、指数a1=0.73，G2=0.8G1、G3=1.2G1，线性化点0.85ncr；均为选定聚合仿真参数，不是三块真实空域容量。
 PDF p.6：100 m平方、15 m well-clear、20 m/s速度下，以≤65架/min恒定需求各运行30 min；30 s聚合后整次平均为一MFD点，非动态加载滞回试验。
 PDF p.13：归一化/时间缩放后输入时延h12/h13/h21/h23/h31/h32=3/0.1/3/0.2/1/0.7；不能不加换算直接当实际秒级执行周期。
 PDF p.12 Theorem1及pp.16–18 Appendix：A1–A4下误差渐近为0、信号有界，事件间隔有正下界；这是理论性质，未给效率改善百分比。</x:v>
       </x:c>
-      <x:c r="E22" s="4" t="str">
+      <x:c r="E24" s="4" t="str">
         <x:v>只发表一组MFD识别案例，采用不同平稳加载；其他航空器/运行参数和微观控制算法、动态需求与滞回为未来/进行中研究（PDF p.16 §6）。
 输入供给函数及上游区域之间容量分享为未来建模内容（PDF p.16 §6）。
 累积相关输入时延的物理含义及其与MFD的解析关系仍需研究（PDF p.8 Principal observations）。
 当前固定事件阈值与状态反馈设计；相对/自适应/切换阈值及输出反馈修改列为扩展（PDF p.11 Remark1、p.12 Remark3）。</x:v>
       </x:c>
-      <x:c r="F22" s="4" t="str">
+      <x:c r="F24" s="4" t="str">
         <x:v>全文评价：早已用微观仿真识别MFD并提出宏观鲁棒边界反馈，后者在聚合动力学和时延假设下测试，不等同完整逐机闭环。其平稳加载限制已被后续B05的动态加载等实验部分补足，不再当整个领域未解决的问题（PDF pp.5–6、8–16）。</x:v>
       </x:c>
-      <x:c r="G22" s="4" t="str">
-        <x:v>作为宏观反馈基础参考，区分MFD识别、聚合控制验证和逐机执行闭环的不同证据层次。</x:v>
-      </x:c>
-      <x:c r="H22" s="11" t="str">
-        <x:v>FULL_TEXT</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="23" ht="248" customHeight="1">
-      <x:c r="A23" s="4" t="str">
+      <x:c r="G24" s="4" t="str">
+        <x:v>宏观边界反馈基础，区分微观识别、聚合控制和逐机闭环。</x:v>
+      </x:c>
+      <x:c r="H24" s="11" t="str">
+        <x:v>FULL_TEXT</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="248" customHeight="1">
+      <x:c r="A25" s="4" t="str">
         <x:v>B12</x:v>
       </x:c>
-      <x:c r="B23" s="4" t="str">
+      <x:c r="B25" s="4" t="str">
         <x:v>Integrated departure and boundary control for low-altitude air city transport systems（2024）</x:v>
       </x:c>
-      <x:c r="C23" s="4" t="str">
+      <x:c r="C25" s="4" t="str">
         <x:v>方法：构建区分旅行累积、地面起飞队列和空中边界队列的多区域MFD控制模型，以MPC优化累积和放行/边界控制偏差。不同于控制模型，plant为有局部APF避碰的逐机LAAT-Flow；轨迹及队列状态每60 s反馈初始化MPC，预测5步。Algorithm2将宏观放行比变为逐机起飞时间延后，Algorithm3按比例随机指定边界buffer悬停，再经安全空间检查重入。故已实现宏→微命令与微→宏状态闭环（PDF pp.4–10、12）。
 场景/设定：固定1.5×1.5 km、120 m高无预设航路网络，中心与外围两区，地面均匀随机OD、VTOL和区域上方buffer。相同飞机vmax20 m/s、amax5 m/s²、安全/避让/探测半径15/22.5/45.5 m；仿真1 h、0.5 s步长，聚合/控制/MPC离散均60 s，预测300 s。NC/DC/BC/DBC同用梯形峰值2.5架/s，对照识别容量2.3架/s；各控制器分别标定权重（PDF pp.11–13 Table1）。</x:v>
       </x:c>
-      <x:c r="D23" s="4" t="str">
+      <x:c r="D25" s="4" t="str">
         <x:v>主要结论：所测过饱和需求下DBC保持稳定自由流并提高速度/出流；DC避免锁死但有波动，NC与BC形成拥堵，中心区主导网络性能。性能直接从微观plant计算TTS=TTT+TDD+TBD，已包括旅行、地面起飞等待及空中边界等待；反馈与完整等待核算都已明确实现。更大边界惩罚体现悬停耗能动机，但未形成量化SOC/能量可行约束。随机排队、权重及具体需求分布是其案例条件（PDF pp.12–16，Figs4–9）。
 定量结果：PDF pp.13、15 Figs7–8：同峰值2.5架/s、1 h需求与微观网络下，DC/BC/DBC的TTS相对NC分别降低32%/6.7%/40%；不是所有指标同比下降。
 PDF p.15 Fig8：以NC的TTS为共同分母，DC/DBC地面延误为2.5%/4.1%，DBC边界延误0.4%，换来额外8个百分点TTS下降；不是各策略内部组成比。
 PDF p.12：区域临界累积33/135架，累积与相应起飞/边界队列上界99/405架；网络识别容量2.3架/s，小于比较需求2.5架/s。
 PDF pp.11–12 Table1：0.5 s逐机仿真、60 s聚合和控制、5步预测；权重分别标定，不是同一固定目标权重下的纯动作维度对照。</x:v>
       </x:c>
-      <x:c r="E23" s="4" t="str">
+      <x:c r="E25" s="4" t="str">
         <x:v>区域增多时目标权重难校准，当前配置只匹配测试设置；其他情景需再配置/标定（PDF p.16 §4）。
 控制器仅在特定区域需求分布下测试，需比较其他分布、其他MPC以外方法（PDF p.16 §4）。
 逐机命令只展示一种特定随机排队方案，空域结构有限，其他命令与构形需测试（PDF p.16 §4）。
 buffer悬停可能增加冲突和电池消耗，量化能源为另项进行中研究；行为时间价值、等待/移动权重也可后续研究（PDF pp.3、12、15）。
 起飞队列简化假设高峰vertiport饱和或过饱和，作者说明可换用更一般守恒方程（PDF p.7 footnote2）。</x:v>
       </x:c>
-      <x:c r="F23" s="4" t="str">
-        <x:v>全文评价：已有完整宏→微命令、微→宏状态反馈及TTT+TDD+TBD核算，反馈与完整等待不是新贡献。随机边界分配、特定权重/需求以及悬停能源未量化为SOC可行性，使个体选择、资源占用和能量裕度协同可作为待检验增量（PDF pp.4–16）。</x:v>
-      </x:c>
-      <x:c r="G23" s="4" t="str">
-        <x:v>最直接的闭环对照之一；逐项比较具体个体选择、资源占用与动态能量裕度，而不重复宣称首次微宏反馈。</x:v>
-      </x:c>
-      <x:c r="H23" s="11" t="str">
-        <x:v>FULL_TEXT</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="24" ht="206" customHeight="1">
-      <x:c r="A24" s="4" t="str">
+      <x:c r="F25" s="4" t="str">
+        <x:v>全文评价：已有宏→微命令、微→宏状态及TTT+TDD+TBD完整核算，反馈和全部等待不是新贡献。随机边界分配、特定权重/需求和构形为案例条件；悬停能源未量化为SOC是真实边界，不作为新题目立题前提（PDF pp.4–16）。</x:v>
+      </x:c>
+      <x:c r="G25" s="4" t="str">
+        <x:v>成熟准入/边界闭环强基线，检验条件供给与组织过渡支持的额外增量。</x:v>
+      </x:c>
+      <x:c r="H25" s="11" t="str">
+        <x:v>FULL_TEXT</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="206" customHeight="1">
+      <x:c r="A26" s="4" t="str">
         <x:v>C01</x:v>
       </x:c>
-      <x:c r="B24" s="4" t="str">
+      <x:c r="B26" s="4" t="str">
         <x:v>Strategic and Tactical Path Planning for Urban Air Mobility: Overview and Application to Real-World Use Cases（2023）</x:v>
       </x:c>
-      <x:c r="C24" s="4" t="str">
+      <x:c r="C26" s="4" t="str">
         <x:v>方法：提出战略—战术两层规划框架。战略层使用定制的batch informed trees（BIT*，基于OMPL）在3D/4D环境中以路径长度、备降着陆点、地面风险和能耗加权代价搜索可行轨迹；对不同GNSS覆盖图生成候选路径，进行多项式平滑和导航误差协方差检验后选最低代价解。战术层按复杂度递增提供三种处理：Level 1只缩放速度时间历程，Level 2用定制RRT在事件附近局部改道并回归战略路径，Level 3从未受影响点用RRT全局重规划；运行可用层并比较可行输出后更新飞行计划。
 场景/设定：两个用例均位于意大利Naples及周边。空中出租车从Capodichino机场飞往Naples商业中心或港口；医疗配送从大陆Monte di Procida药房飞往Procida岛医疗单元，直线约4 km，用以对比船运约16 min且冬季班次不足的情况。两类任务均使用真实地理/环境地图；医疗场景最高飞行高度150 m，统一风速5 m/s，未进行实飞。</x:v>
       </x:c>
-      <x:c r="D24" s="4" t="str">
+      <x:c r="D26" s="4" t="str">
         <x:v>主要结论：战略层在真实地理约束下生成满足禁飞区、飞行器和导航误差要求的候选路径；战术层分别通过速度时间缩放、局部RRT和全局RRT处理移动障碍或环境变化。医疗用例中Level 2保持战略路径代价几乎不变并只增加少量飞行时间，Level 1可能造成很长等待；作者报告战略与战术计算时间可用于相应规划窗口。
 定量结果：医疗用例战略方案D1–D3的总目标代价约26,675–33,962，单方案计算时间53.0–60.3 s（表2）；战术解的总目标代价约26,686–30,160，计算时间1.7–5.2 s（表3），最大导航误差约1.19–1.25 m。论文结论称战略路径计算低于约60 s、战术层约5 s，适合约10 s级更新窗口；用例结果中规划路径均可飞行。</x:v>
       </x:c>
-      <x:c r="E24" s="4" t="str">
+      <x:c r="E26" s="4" t="str">
         <x:v>第6节明确提出后续需在很高交通密度下评估架构性能，并加入飞行规则和结构化空域；还需进一步降低战术规划计算负担、改善软件工程和算法。</x:v>
       </x:c>
-      <x:c r="F24" s="4" t="str">
+      <x:c r="F26" s="4" t="str">
         <x:v>全文评价：战略与战术规划的接口有价值，但路径可行与计算可完成并不等于高密度交通稳定；需要进一步连接需求增长、排队和实际完成出流。</x:v>
       </x:c>
-      <x:c r="G24" s="4" t="str">
-        <x:v>作为规划与执行分层的参考，不把分层结构本身当作新贡献。</x:v>
-      </x:c>
-      <x:c r="H24" s="11" t="str">
-        <x:v>FULL_TEXT</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="25" ht="304" customHeight="1">
-      <x:c r="A25" s="4" t="str">
+      <x:c r="G26" s="4" t="str">
+        <x:v>规划与执行分层接口参考，分层结构本身不是新贡献。</x:v>
+      </x:c>
+      <x:c r="H26" s="11" t="str">
+        <x:v>FULL_TEXT</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="304" customHeight="1">
+      <x:c r="A27" s="4" t="str">
         <x:v>C02</x:v>
       </x:c>
-      <x:c r="B25" s="4" t="str">
+      <x:c r="B27" s="4" t="str">
         <x:v>Automated flight planning of high-density urban air mobility（2021）</x:v>
       </x:c>
-      <x:c r="C25" s="4" t="str">
+      <x:c r="C27" s="4" t="str">
         <x:v>方法：AFPS顺序连接空域管理LAMS和交通管理LTMS：以LiDAR三维城市地图、障碍包络和分层visibility graph生成各vertiport对的绕障路径并预存交点；给定OD、起飞时刻与速度，检测交叉/同向/反向共线冲突，通过飞行层指派获得4D计划。一目标最小总generalized flying cost，另一以Nash Social Welfare最大化运营方相对最坏参考成本的收益乘积，并转为混合整数SOCP。未联合决定起飞时刻/调速（PDF pp.5–12 §3）。
 场景/设定：Tampa Bay 30个vertiport、7机场禁飞区及cuboid建筑包络，500–1400 ft共10层、层距100 ft；垂直起降后定层水平巡航，130 knots、垂直1000 fpm、最小分离0.3 NM。45 min内按5或3 min/takeoff需求生成270或450飞行，2/4/6运营方、四档NHHI；起飞时刻在2 min窗内均匀抽取。两模型分别用Gurobi与CPLEX，i7-4790/16 GB，未实施战术偏差回馈闭环（PDF pp.12–18 §4–5）。</x:v>
       </x:c>
-      <x:c r="D25" s="4" t="str">
+      <x:c r="D27" s="4" t="str">
         <x:v>主要结论：在给定速度、时刻、定层与线性外推设定下形成无冲突分层计划，已覆盖战略路径及运营方公平。乘积模型可改善相对参考收益的分配，总系统成本略增，但并非每家收益均上升；高密度部分实例求解至千秒，作者只说多数秒级。电池监测、充电及含不确定性的战术决定向规划约束回馈明确为未来；不能把系统图当已实现闭环，也不能把generalized cost或飞行时间差写成地面延误收益（PDF pp.7–10、14–18）。
 定量结果：PDF p.12 Table1/§4.1：30 vertiport、10层、0.3 NM分离，45 min内270/450飞行；安全结论限于给定时刻和速度模型。
 PDF pp.14–15 Fig11：求和模型两需求的系统成本2653/4380，乘积模型相对差不超过0.5%；原文该句不标成本物理单位，不换写成延误分钟或kWh。
@@ -1305,62 +1369,62 @@
 PDF p.16 Tables2–3：5 min/takeoff、4运营方、NHHI=0.5，求和UBR=0.986/0.987/0.918/0.962，乘积=0.968/0.971/1.000/0.994；公平改善不等于各家收益增加。
 PDF p.16 Fig13：低密度图纵轴至1.6 s，高密度至1600 s；高密度低NHHI部分乘积求解约千秒。图读量级，不把全部实验称为实时。</x:v>
       </x:c>
-      <x:c r="E25" s="4" t="str">
+      <x:c r="E27" s="4" t="str">
         <x:v>起飞时间位移与速度控制、战略和含不确定性战术解脱的耦合为进行中工作（PDF p.5 §2.5、p.17 §5）。
 算例路径网络较简单，爬升占总时间小；更复杂障碍与更高飞行层的影响仍待验证（PDF p.14 §4.2）。
 成本函数需完善运营商业利益表达，天气需要纳入但可靠高分辨率城市天气数据不足（PDF p.17 §5）。
 电池与充电排程依赖任务连接和充电能力，未来才将这些战术决定聚合进入规划形成closed-loop（PDF pp.17–18 §5）。</x:v>
       </x:c>
-      <x:c r="F25" s="4" t="str">
+      <x:c r="F27" s="4" t="str">
         <x:v>全文评价：已有战略路径/分层规划与运营方公平；电池及含不确定性的战术回馈闭环明确为未来。高密度部分有千秒级求解，不能泛称实时；分离可行限于给定速度、起飞时刻和检测模型，不等于现实全动力学安全保证（PDF pp.5–18）。</x:v>
       </x:c>
-      <x:c r="G25" s="4" t="str">
-        <x:v>作为集中式战略规划与公平参照，比较给定计划同实际执行反馈的差异，并如实保留高密度计算代价。</x:v>
-      </x:c>
-      <x:c r="H25" s="11" t="str">
-        <x:v>FULL_TEXT</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="26" ht="108" customHeight="1">
-      <x:c r="A26" s="4" t="str">
+      <x:c r="G27" s="4" t="str">
+        <x:v>集中式战略规划和公平参考，保留高密度代价与计划—执行差异。</x:v>
+      </x:c>
+      <x:c r="H27" s="11" t="str">
+        <x:v>FULL_TEXT</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="108" customHeight="1">
+      <x:c r="A28" s="4" t="str">
         <x:v>C03</x:v>
       </x:c>
-      <x:c r="B26" s="4" t="str">
+      <x:c r="B28" s="4" t="str">
         <x:v>Vertiport Planning for Urban Aerial Mobility: An Adaptive Discretization Approach（2022）</x:v>
       </x:c>
-      <x:c r="C26" s="4" t="str">
+      <x:c r="C28" s="4" t="str">
         <x:v>方法：构建联合vertiport数量、位置、容量与战术运行的规划模型，需求函数和飞行距离使模型含非凸项。使用混合整数二阶锥可处理部分、精确自适应离散化将非凸需求近似为分段常数，并给出保守可行解、松弛界和逐步收敛的全局优化方法。
 场景/设定：城市空中交通网络的vertiport规划与乘客需求分配；出版商摘要/页面描述不同候选网络、容量和需求情形，完整网络规模及实验设置未获全文。</x:v>
       </x:c>
-      <x:c r="D26" s="4" t="str">
+      <x:c r="D28" s="4" t="str">
         <x:v>主要结论：自适应离散化在解质量、运行时间和最优性保证上优于固定离散化，并逐步收敛到全局最优。少数高容量vertiport更倾向服务长距离需求；网络规划和客户需求变化会显著影响盈利能力。
 定量结果：出版商摘要明确报告可达到1%的最优性间隙；未获得正文实验表格，其他规模和时间数值无法核验。</x:v>
       </x:c>
-      <x:c r="E26" s="4" t="str">
+      <x:c r="E28" s="4" t="str">
         <x:v>正式全文不可访问；出版商摘要未给出作者明确列出的局限性，不能据摘要外推。</x:v>
       </x:c>
-      <x:c r="F26" s="4" t="str">
+      <x:c r="F28" s="4" t="str">
         <x:v>摘要评价，待全文确认：主要解决设施网络及容量规划，其最优性是该规划模型内的结论，不能直接解释运行中的局部避碰和构形切换。该范围差异不是算法错误。</x:v>
       </x:c>
-      <x:c r="G26" s="4" t="str">
-        <x:v>用于区分长期规划与运行控制，帮助限制博士课题范围。</x:v>
-      </x:c>
-      <x:c r="H26" s="13" t="str">
+      <x:c r="G28" s="4" t="str">
+        <x:v>长期设施规划的外围参考，区分运行引导的决策尺度并维持摘要限界。</x:v>
+      </x:c>
+      <x:c r="H28" s="13" t="str">
         <x:v>ABSTRACT_ONLY</x:v>
       </x:c>
     </x:row>
-    <x:row r="27" ht="304" customHeight="1">
-      <x:c r="A27" s="4" t="str">
+    <x:row r="29" ht="304" customHeight="1">
+      <x:c r="A29" s="4" t="str">
         <x:v>C04</x:v>
       </x:c>
-      <x:c r="B27" s="4" t="str">
+      <x:c r="B29" s="4" t="str">
         <x:v>Urban air mobility: from complex tactical conflict resolution to network design and fairness insights（2023）</x:v>
       </x:c>
-      <x:c r="C27" s="4" t="str">
+      <x:c r="C29" s="4" t="str">
         <x:v>方法：在固定单层有向track与无冲突战略名义计划上，对扰动后整个剩余计划求集中式global MILP，联合未起飞航班地面holding与空中航班节点调速。用追随及合并/分流危险区的时间分离约束和最早/最晚过点区间保证模型内安全，最小非优先航班巡航waypoint时间绝对偏差并高权保护priority；另比较只调整直接冲突航班的local版本与到达延误离均差公平目标。网络设计见解来自固定拓扑比较，非联合改网（PDF pp.7–17）。
 场景/设定：三类合成单高度网络：Grid 8 vertiport、Airport 5、Metroplex 9且两中心单廊连接；每类两套名义计划，五个10 min需求批次，总时域约50 min。测试随机漂移/地面延误、新priority、固定直线noncooperative intruder；巡航150 mph、最小分离0.5 NM，速度可±5%或−5%/+10%，节点调速、边内匀速，爬升速度固定。MILP在扰动/检测时重排剩余全部航班（PDF pp.17–21 Tables1–5）。</x:v>
       </x:c>
-      <x:c r="D27" s="4" t="str">
+      <x:c r="D29" s="4" t="str">
         <x:v>主要结论：global同时考虑初始冲突及调整诱发冲突，可调原未直接冲突航班，因此比受限local版本更有可行性；这不构成对所有分布式算法的普遍结论。合作程度下降后地面hold/调速常不足，intruder多数无可行解。公平版本改善航班到达延误均等性却明显增加总延误及调速频次。分离条件充分非必要、有保守性，固定网络并未做在线重构；能耗模型和非合作轨迹不确定性留未来（PDF pp.12、21–32）。
 定量结果：PDF pp.21–23 Tables2–3：随机扰动60例中59可行，平均/最大CPU0.27/1.65 s；priority 60例全部可行，0.32/1.81 s，55%有priority延误。
 PDF p.25 Table4：intruder 180例中52可行、128不可行；r=1/5/10 min各60例不可行55/45/28，故r=10组内为28/60=46.7%，不能用28/180说该组仅15%。
@@ -1368,62 +1432,62 @@
 PDF p.30 Table6：公平目标在random/priority/intruder逐实例百分比平均中改善35.06%/39.87%/45.29%，总arrival delay劣化478.76%/430.39%/397.72%；不能用均值之比替代这些百分比。
 PDF p.30 Table6：总arrival delay均值原→公平为9.74→37.62、35.93→65.39、35.43→77.50 min；约半数实例每架平均调速原≤2次、公平可至13次（p.31 Fig11）。</x:v>
       </x:c>
-      <x:c r="E27" s="4" t="str">
+      <x:c r="E29" s="4" t="str">
         <x:v>短期内graph固定、单层巡航；边内匀速仅节点调速、climb固定；危险区分离为充分非必要保守条件（PDF pp.8、12、16）。
 测试仅单个新priority或intruder且即刻检测，低合作时动作不足；rerouting、hovering、退出走廊为未来补充（PDF pp.20–26、32）。
 相关可比方法少，使用自家local版本作对照，不是全面benchmark（PDF p.26 §6.3.4）。
 明确未来包括能耗模型、共同轨迹调整、对未来扰动的鲁棒性、intruder轨迹不确定性与多巡航高度；公平收益是否抵代价取决于所选目标及实例（PDF pp.29–32）。</x:v>
       </x:c>
-      <x:c r="F27" s="4" t="str">
+      <x:c r="F29" s="4" t="str">
         <x:v>全文评价：固定网络战术global MILP已联合地面holding与空中调速，不能写成网络设计联合优化。合作程度下降时大量不可行，公平成本高且能源模型为未来；应作为集中式强参考，不能把局部算法更快直接等同更好（PDF pp.7–17、21–32）。</x:v>
       </x:c>
-      <x:c r="G27" s="4" t="str">
-        <x:v>作为集中式强对照，比较可行率、完整延误、调速与公平代价；不把固定拓扑敏感性误称在线网络设计。</x:v>
-      </x:c>
-      <x:c r="H27" s="11" t="str">
-        <x:v>FULL_TEXT</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="28" ht="178" customHeight="1">
-      <x:c r="A28" s="4" t="str">
+      <x:c r="G29" s="4" t="str">
+        <x:v>集中式强对照，比较可行率、总延误、调速和公平代价，不误称在线结构联优。</x:v>
+      </x:c>
+      <x:c r="H29" s="11" t="str">
+        <x:v>FULL_TEXT</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="178" customHeight="1">
+      <x:c r="A30" s="4" t="str">
         <x:v>C05</x:v>
       </x:c>
-      <x:c r="B28" s="4" t="str">
+      <x:c r="B30" s="4" t="str">
         <x:v>Integrated Conflict Management for UAM With Strategic Demand Capacity Balancing and Learning-Based Tactical Deconfliction（2024）</x:v>
       </x:c>
-      <x:c r="C28" s="4" t="str">
+      <x:c r="C30" s="4" t="str">
         <x:v>方法：提出ICMP，将战略层需求—容量平衡（DCB）与战术层冲突消解串联：DCB用优化算法或启发式算法分配地面延误、预先控制瓶颈流量；战术层用多智能体强化学习（MARL）输出速度建议，并与规则型速度冲突消解基线比较。仿真采用BlueSky及LoWC/NMAC/MAC风险指标。
 场景/设定：BlueSky中三条共享航路：N-7→N-1→N-2→N-3、N-9→N-1→N-2→N-3、M-2→N-2→M-4；资源为N-1/N-2。表I含30个飞行计划和100张调度表；MARL训练150,000回合（2×RTX3090，约4 h），观测半径1500 m，同高度运行，时间窗200 s。安全阈值：LoWC 500 m、NMAC 150 m、MAC 10 m，风险比β=0.005。</x:v>
       </x:c>
-      <x:c r="D28" s="4" t="str">
+      <x:c r="D30" s="4" t="str">
         <x:v>主要结论：战略DCB先把需求限制在可承受容量，再由规则或MARL处理局部冲突。无DCB时难以在较高需求下维持目标安全水平；在给定案例中，DCB+MARL允许更高的200 s窗容量并保持较低估计MAC，同一需求水平下其地面延误低于DCB+规则，但DCB会引入地面延误。作者同时指出DCB与战术速度改变之间存在ETA不一致。
 定量结果：仅DCB时可行容量C=1/200 s；规则战术可到C=4；MARL可到C=7。表III估计MAC/100,000 h：C=4时无战术75.51、规则0.74、MARL0.85；C=7时无战术122.14、规则115.34、MARL0.66；MARL在C=8、10时分别3.70、23.49。表IV高/中/低需求下，DCB+MARL（C=7）的LoWC为45.6/62.8/49.6，估计MAC为0.66/0.65/0.51，空中延误30.8/32.9/22.2 s、地面延误158.4/74.4/19.9 s；DCB+规则（C=4）的LoWC为25.9/34.8/30.8，估计MAC为0.74/0.77/0.92。</x:v>
       </x:c>
-      <x:c r="E28" s="4" t="str">
+      <x:c r="E30" s="4" t="str">
         <x:v>第VI节（arXiv预印本pp.11–12）明确指出战略DCB使用确定性估计飞行时间，而战术速度改变会改变ETA，差异在复杂网络中累积并削弱预条件化效果；未来需要随机ETA模型。第V节p.10还说明规则基线为简化而未建模替代机动。</x:v>
       </x:c>
-      <x:c r="F28" s="4" t="str">
-        <x:v>全文评价：战略层确定性到达时间会被战术调速改变，两层之间仍需更充分的反馈。不同方法使用不同可承受容量，结果不能被简化成同一负荷下的纯算法收益；估计MAC风险也不是实测事故率。</x:v>
-      </x:c>
-      <x:c r="G28" s="4" t="str">
-        <x:v>最接近宏微观协同的核心基线之一；研究实际执行反馈和构形变化的增量价值。</x:v>
-      </x:c>
-      <x:c r="H28" s="11" t="str">
-        <x:v>FULL_TEXT</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="29" ht="318" customHeight="1">
-      <x:c r="A29" s="4" t="str">
+      <x:c r="F30" s="4" t="str">
+        <x:v>全文评价：已用Monte Carlo识别不同战术策略满足目标安全水平的容量，再据此DCB，策略相关容量不是空白。战略确定性ETA被战术调速改变仍需处理；不同方法容量设定不同，不能视为同负荷纯算法收益，估计MAC不是实测事故率（§V–VI）。</x:v>
+      </x:c>
+      <x:c r="G30" s="4" t="str">
+        <x:v>策略相关安全容量和战略—战术衔接的核心先例，比较需求预调节与执行失配。</x:v>
+      </x:c>
+      <x:c r="H30" s="11" t="str">
+        <x:v>FULL_TEXT</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="318" customHeight="1">
+      <x:c r="A31" s="4" t="str">
         <x:v>C06</x:v>
       </x:c>
-      <x:c r="B29" s="4" t="str">
+      <x:c r="B31" s="4" t="str">
         <x:v>A heuristic approach for scheduling advanced air mobility aircraft at vertiports（2023）</x:v>
       </x:c>
-      <x:c r="C29" s="4" t="str">
+      <x:c r="C31" s="4" t="str">
         <x:v>方法：将单vertiport起飞与到达反向四阶段流程建模为blocking hybrid flowshop：taxiway1—gates—taxiway2—TLOF，arrival逆序。MILP联合各阶段服务位指派/排序，限制单资源排他、下游未空时占用当前组件阻塞及同pad分离；分别最小makespan和对外生目标时刻的绝对偏差。H1以随机种子和首次可用组件、最长闲置插入改进，H2以整体slack种子和近目标插入改进。arrival目标使用完整流程stage1完成时刻，非触地时刻（PDF pp.5–11）。
 场景/设定：合成n=10/20/30/40/50架次、起飞比例30%/50%/70%，三布局均一条taxiway1和taxiway2，gate/pad各2、3或4。TLOF处理15–90 s、gate30–600 s、taxiway5–90 s均匀抽样，同pad分离90 s；目标Tj按各阶段处理和及n生成随机窗。CPLEX限1800 s，Python启发式100000迭代，i7-10870H/16 GB。流程不允许额外缓冲区，等待会继续占当前组件（PDF pp.5–6、11–13 Table2）。</x:v>
       </x:c>
-      <x:c r="D29" s="4" t="str">
+      <x:c r="D31" s="4" t="str">
         <x:v>主要结论：已充分联合多类地面资源和起降相反流阻塞，不能概括为只排pad或忽略终端服务。小规模MILP较好，大规模时限内难给可行解，启发式有实用收益但缺紧下界，不能称近最优。作者用目标时刻体现电池动机；模型实际没有SOC演化或硬能量界，实验目标来自随机生成。到达偏差按最终stage1完成语义，不能称最晚触地截止；空中进近仅处理时间，不生成避碰轨迹（PDF pp.5–8、12–18）。
 定量结果：PDF p.12：5起飞5到达、3 gate/3 pad示例，makespan模型1118 s；另一目标偏差模型总偏差908 s、makespan1203 s，两个目标不可视为同一个最优值。
 PDF p.13 §6.3：MILP仅n=10证最优，部分n=40及全部n=50在1800 s无可行解；n=10已知最优对照下H1平均makespan相对误差21.11%，不代表大例近优。
@@ -1431,166 +1495,166 @@
 PDF p.14 Table3：2 gate/2 pad、50架各半起飞到达，MILP两目标1800 s无可行解；H1 makespan8238 s/CPU283.61 s，H2偏差16552 s/283.52 s。
 PDF pp.17–18 Table6：small/medium/large的H1均值5126.40/3691.54/2048.78 s，对NEH7367.72/5581.68/3162.94 s；原Difference用H1作分母，不能说相对NEH降低43.72%/51.20%/54.38%。</x:v>
       </x:c>
-      <x:c r="E29" s="4" t="str">
+      <x:c r="E31" s="4" t="str">
         <x:v>作者明确缺少准确下界，CPLEX不证最优时无法知道启发式距最优多远；经典下界未含blocking与分离（PDF p.13 §6.3）。
 显式假设所有航班经gate装卸、阶段内组件同质、目标时刻预先已知；最终进近开始后不允许抢占/暂停（PDF pp.6–8）。
 航空器routing、容量分析、绕过gate的额外taxiway、异质飞机及gate/pad、其他延误目标与更强精确算法为未来方向（PDF pp.17–18 §7）。
 变量/约束核对的模型边界而非作者自称缺陷：电池由外生目标时刻体现，目标偏差是软惩罚，无动态SOC或硬最晚着陆能量约束；arrival目标为stage1完成（PDF pp.6–8）。</x:v>
       </x:c>
-      <x:c r="F29" s="4" t="str">
-        <x:v>全文评价：地面资源阻塞与起降联排已经充分考虑。电池仅通过外生目标时间表达动机，尚无动态SOC或硬着陆能量界；启发式缺紧下界，不能称近最优。arrival指标按完整流程stage1完成语义，不能称触地截止（PDF pp.5–8、13、17–18）。</x:v>
-      </x:c>
-      <x:c r="G29" s="4" t="str">
-        <x:v>保留多类服务资源联排与阻塞能力作为基线，比较动态能量反馈，并按完整arrival流程完成时间解释目标。</x:v>
-      </x:c>
-      <x:c r="H29" s="11" t="str">
-        <x:v>FULL_TEXT</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="30" ht="136" customHeight="1">
-      <x:c r="A30" s="4" t="str">
+      <x:c r="F31" s="4" t="str">
+        <x:v>全文评价：地面资源阻塞与起降联排已充分考虑。电池通过外生target表达动机，尚非动态SOC或硬着陆能量界；启发式缺紧下界，不能称近最优。arrival按完整流程stage1完成，不是触地截止（PDF pp.5–8、13、17–18）。这些为其业务边界，不作为新题目立题前提。</x:v>
+      </x:c>
+      <x:c r="G31" s="4" t="str">
+        <x:v>多服务资源联排与阻塞的外围参考，借鉴完成事件语义，不引入设施或电池主线。</x:v>
+      </x:c>
+      <x:c r="H31" s="11" t="str">
+        <x:v>FULL_TEXT</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="136" customHeight="1">
+      <x:c r="A32" s="4" t="str">
         <x:v>C07</x:v>
       </x:c>
-      <x:c r="B30" s="4" t="str">
+      <x:c r="B32" s="4" t="str">
         <x:v>Introducing digital air-traffic controllers for urban-air mobility to ensure safe and energy-efficient flight operations（2025）</x:v>
       </x:c>
-      <x:c r="C30" s="4" t="str">
+      <x:c r="C32" s="4" t="str">
         <x:v>方法：设计UAM Digital Controller（UDC），把经过验证的时隙与4D轨迹算法接入数字空中交通管制流程。作者将运行概念拆为10条运行规则、5项需求、42项运行任务和25项技术需求，并用理论walkthrough检查任务链、放行、重规划和hold决策。
 场景/设定：汉堡机场控制区内VFR空中出租车；本文评价取自一次人机仿真场景中的15架空中出租车航班。到达交通在同一路线上采用1500 ft高度、离场交通采用2000 ft高度进行垂直分离。5分钟内超过6架时触发hold，walkthrough中4架收到交通负荷hold命令；Vertiport East另有4次holding decision。</x:v>
       </x:c>
-      <x:c r="D30" s="4" t="str">
+      <x:c r="D32" s="4" t="str">
         <x:v>主要结论：UDC walkthrough中45项活动均可执行完成，Vertiport East的航路重叠触发4次hold；作者据此展示了数字控制器如何以时隙、4D轨迹和地面/空中hold协调终端区流量。论文同时将系统需求映射到技术任务，为后续验证提供接口。
 定量结果：相关DLR人机仿真中10名管制员在最高15架空中出租车/小时交通负荷下工作负荷约增加30%（引言/§2，属于相关工作数字）；本文walkthrough使用一次场景的15架空中出租车航班，4架收到交通负荷hold命令，另有Vertiport East的4次holding decision，共计算45项活动且所有航班到达终点。</x:v>
       </x:c>
-      <x:c r="E30" s="4" t="str">
+      <x:c r="E32" s="4" t="str">
         <x:v>§4.4 pp.345–346和§5 pp.347–348明确列出：当前模型假设输入按顺序且同步，缺少数据同步机制；hold后何时解除及多个hold如何继续未定义；没有限制指令传输数量，可能产生过快或同步消息；人与数字控制器的协同/故障接管尚未详细设计；规则源自汉堡案例，其他机场可能需要不同规则；尚未验证故障场景。§6 p.348提出后续进行human-in-the-loop验证。</x:v>
       </x:c>
-      <x:c r="F30" s="4" t="str">
+      <x:c r="F32" s="4" t="str">
         <x:v>全文评价：主要是数字管制流程及理论走查，流程走通不能证明高密度下效率或安全性能。hold解除、同步和故障接管未充分定义，正是运行闭环中不能省略的环节。</x:v>
       </x:c>
-      <x:c r="G30" s="4" t="str">
-        <x:v>用于明确等待解除、资源确认与异常流程，不把概念验证当性能基准。</x:v>
-      </x:c>
-      <x:c r="H30" s="11" t="str">
-        <x:v>FULL_TEXT</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="31" ht="136" customHeight="1">
-      <x:c r="A31" s="4" t="str">
+      <x:c r="G32" s="4" t="str">
+        <x:v>等待解除、确认与异常流程参考，概念验证不当高密度性能证据。</x:v>
+      </x:c>
+      <x:c r="H32" s="11" t="str">
+        <x:v>FULL_TEXT</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="136" customHeight="1">
+      <x:c r="A33" s="4" t="str">
         <x:v>C08</x:v>
       </x:c>
-      <x:c r="B31" s="4" t="str">
+      <x:c r="B33" s="4" t="str">
         <x:v>A collaborative system of systems simulation of urban air mobility（2025）</x:v>
       </x:c>
-      <x:c r="C31" s="4" t="str">
+      <x:c r="C33" s="4" t="str">
         <x:v>方法：构建基于agent的混合系统仿真，将出行需求/方式选择、车辆设计、机队管理、vertiport空侧、UTM/轨迹和成本收益工具通过RCE黑箱接口耦合。空域采用slot-based或trajectory-based管理，并以名义条件下的协同工作流运行汉堡案例。
 场景/设定：汉堡20个vertiport、30架倾转旋翼机（3名乘客+1名飞行员），仿真时长4小时，票价2 EUR/km。本文轨迹工具采用爬升/下降3.556 m/s、巡航高度457 m、横向0.002°、垂直250 m、时间60 s间隔；共处理1239个飞行请求，其中43个UAM请求，模式份额3.4%。</x:v>
       </x:c>
-      <x:c r="D31" s="4" t="str">
+      <x:c r="D33" s="4" t="str">
         <x:v>主要结论：系统证明了多个领域工具通过RCE协同仿真并输出需求、航班、vertiport和轨迹结果的可行性。框架定义了slot-based与trajectory-based两种路线管理方式；本次4 h汉堡研究实际采用slot-based空域管理并生成名义运行结果。文章把主要贡献定位为proof-of-concept，不把示例结果作为普适结论。
 定量结果：仿真含20个vertiport、30架飞机、4 h、1239个飞行请求、43个UAM请求和3.4%模式份额；票价为2 EUR/km。冲突处理通过改变出发/到达时间，使用横向0.002°、垂直250 m、时间60 s约束。</x:v>
       </x:c>
-      <x:c r="E31" s="4" t="str">
+      <x:c r="E33" s="4" t="str">
         <x:v>§3 pp.741–742和§4 pp.742–743明确指出：结果只是示范/概念验证，未形成结论性发现，需要完整情景、敏感性和比较研究；当前只模拟名义条件，天气、通信、需求波动等随机off-nominal事件留待未来；成本收益与车辆分配工具为缩短运行时间而省略，地面替代方式只有汽车，人员/监管者不是主动参与者；RCE分布式工作流要求所有工具在线，可能超过半天且调试困难，失败后需重启。</x:v>
       </x:c>
-      <x:c r="F31" s="4" t="str">
+      <x:c r="F33" s="4" t="str">
         <x:v>全文评价：跨领域工具联动证明系统集成可行，但名义示例不足以判断控制策略的因果收益和拥堵边界。完整系统范围很广，直接复制其全部子系统会显著增加博士实施负担。</x:v>
       </x:c>
-      <x:c r="G31" s="4" t="str">
-        <x:v>说明全城市系统课题的工作量；借鉴接口与指标，不扩展到全部需求和经济模块。</x:v>
-      </x:c>
-      <x:c r="H31" s="11" t="str">
-        <x:v>FULL_TEXT</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="32" ht="150" customHeight="1">
-      <x:c r="A32" s="4" t="str">
+      <x:c r="G33" s="4" t="str">
+        <x:v>系统集成及指标接口的外围参考，帮助控范围而不复制全城市子系统。</x:v>
+      </x:c>
+      <x:c r="H33" s="11" t="str">
+        <x:v>FULL_TEXT</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="150" customHeight="1">
+      <x:c r="A34" s="4" t="str">
         <x:v>C09</x:v>
       </x:c>
-      <x:c r="B32" s="4" t="str">
+      <x:c r="B34" s="4" t="str">
         <x:v>Simulated Evaluation of Strategic Conflict Management Capabilities for Urban Air Mobility Operations（2024）</x:v>
       </x:c>
-      <x:c r="C32" s="4" t="str">
+      <x:c r="C34" s="4" t="str">
         <x:v>方法：在NASA X5 PSU原型中串联战略需求容量平衡（DCB）和Sequencing &amp; Scheduling（S&amp;S）。DCB按vertiport容量和时间窗给出地面延误，S&amp;S在控制航路点按到达时间分配起飞前延误以满足最小间隔；比较DCB-only、S&amp;S-only、带时间间隔的DCB→S&amp;S和无间隔DCB→S&amp;S。
 场景/设定：DFW网络7个vertiport、10条OD航路、4个排序控制航路点；vertiport容量2次/12 min bin，控制点最小间隔2 min。单一飞机类型/速度；40架次、1.5 h，2个运营方各20架、每条航路每运营方2架。DCB提前6 min，S&amp;S在新起飞时刻前1 min或紧接DCB运行，最大延误1 h。</x:v>
       </x:c>
-      <x:c r="D32" s="4" t="str">
+      <x:c r="D34" s="4" t="str">
         <x:v>主要结论：DCB能够把需求分配到容量以内，但会产生较大地面延误；只用S&amp;S时吞吐量和地面延误较好，却经常违反既有DCB容量；串联顺序和DCB与S&amp;S之间的时间间隔改变延误分配、峰值并发量和取消情况。
 定量结果：DCB案例每个运营方最多约8/7架并发，S&amp;S-only最多24架；启用DCB的案例因1 h最大延误各取消1架（40架中39架激活），S&amp;S-only无取消。Case 3中98.2%的地面延误来自DCB，25架/39架受延误；两个运营方各14架延误，平均分别23.7和27.6 min/架。DCB案例峰值并发量13。</x:v>
       </x:c>
-      <x:c r="E32" s="4" t="str">
+      <x:c r="E34" s="4" t="str">
         <x:v>§V pp.11–12明确指出当前DCB会产生较大地面延误并低效使用空域；需要研究速度控制和网络级计划优化。S&amp;S-only虽延误短却造成许多DCB违规；需要确定DCB与S&amp;S的时间间隔及更广泛的交互。公平性不是本实验重点，延误分配可能依赖初始计划、提交时间和分配方法，后续需研究高效且公平的运行。</x:v>
       </x:c>
-      <x:c r="F32" s="4" t="str">
+      <x:c r="F34" s="4" t="str">
         <x:v>全文评价：40架次、单一机型与给定网络下的战略试验尚不能覆盖大规模局部执行偏差。仅缩短地面延误会伴随容量违规，必须把容量、取消和完整等待一起比较。</x:v>
       </x:c>
-      <x:c r="G32" s="4" t="str">
-        <x:v>支持准入与排序需要协调的判断，并提供对照实验及公平性指标。</x:v>
-      </x:c>
-      <x:c r="H32" s="11" t="str">
-        <x:v>FULL_TEXT</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="33" ht="150" customHeight="1">
-      <x:c r="A33" s="4" t="str">
+      <x:c r="G34" s="4" t="str">
+        <x:v>战略准入、排序和公平评价参考，完整计入容量违规、取消与等待。</x:v>
+      </x:c>
+      <x:c r="H34" s="11" t="str">
+        <x:v>FULL_TEXT</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="150" customHeight="1">
+      <x:c r="A35" s="4" t="str">
         <x:v>C10</x:v>
       </x:c>
-      <x:c r="B33" s="4" t="str">
+      <x:c r="B35" s="4" t="str">
         <x:v>Real-time traffic simulation and management for large-scale urban air mobility: Integrating route guidance and collision avoidance（2026）</x:v>
       </x:c>
-      <x:c r="C33" s="4" t="str">
+      <x:c r="C35" s="4" t="str">
         <x:v>方法：提出面向大规模UAM的分层实时交通管理：中心化区域route guidance在空间与时间维度分配4D航路/waypoint，局部飞机采用分布式速度障碍/ORCA型碰撞避免。空域划分为六边形区域，依据区域占用进行速度调节，并使用快速近似方法处理多机路径和动态禁飞区。
 场景/设定：抽象城市六边形空域和点对点需求，比较单层z=500 m、单层范围450–550/400–600 m及双层z=400/600 m；区域半径250 m、探测半径200 m、安全半径50 m、最大速度20 m/s、控制增益5、步长1 s。三种OD需求图案（+、#、*）和临界流附近固定需求；基线为无冲突虚拟走廊/自由飞行策略。</x:v>
       </x:c>
-      <x:c r="D33" s="4" t="str">
+      <x:c r="D35" s="4" t="str">
         <x:v>主要结论：route guidance使空间和时间分配更均匀，碰撞避免在waypoint间生成安全轨迹；在示例中提出方法保持接近自由流状态并改善安全、速度、完成率和能耗，同时保留空气交通宏观基本图（MFD）的均匀性前提。双层相对单层进一步改善间隔、速度和完成率。
 定量结果：单层表3中，基线→提出方法：平均最小间距153.3→303.9 m（+98.2%），平均速度11.39→19.39 m/s（+70.2%），完成率0.083→0.191 trip/s（+130%），能耗0.0148→0.0114 kWh/trip（−23.0%），计算效率0.91→4.85 iteration/s（+433%）。双层相对单层平均最小间距+56.3%、速度+38.9%、完成率+40.1%。</x:v>
       </x:c>
-      <x:c r="E33" s="4" t="str">
+      <x:c r="E35" s="4" t="str">
         <x:v>§2.2 p.7明确假设电量充足、指令精确执行、没有通信/尾流/执行延误和不确定性，且不控制起降，飞机按点粒子处理；未来需加入能量管理、执行器约束和动态不确定性。§2.1 p.5提出需要适配不同空域构形；§3.2.2 p.20提出更复杂网络构形留待未来。</x:v>
       </x:c>
-      <x:c r="F33" s="4" t="str">
-        <x:v>全文评价：已经结合全局路线引导与局部避碰，是必须正面对比的工作；但起降阶段被排除，能源、执行与延迟被简化。可研究终端服务瓶颈和过渡可执行性，不能再次宣称首次宏微观融合。</x:v>
-      </x:c>
-      <x:c r="G33" s="4" t="str">
-        <x:v>用于限定创新边界；对比对象应保留其空间均匀化和路线协调能力。</x:v>
-      </x:c>
-      <x:c r="H33" s="11" t="str">
-        <x:v>FULL_TEXT</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="34" ht="206" customHeight="1">
-      <x:c r="A34" s="4" t="str">
+      <x:c r="F35" s="4" t="str">
+        <x:v>全文评价：已有全局路线引导、局部避碰及聚合曲线，不能再称首次融合。高度范围对照改变可用空间，不能单独识别同资源组织收益；起降被排除，能源、执行和延迟被简化，真实假设须保留（作者稿§2.2、§3.2、§4）。</x:v>
+      </x:c>
+      <x:c r="G35" s="4" t="str">
+        <x:v>路线引导、局部避碰和聚合曲线的核心强对照，保留其均匀化能力并控制资源差异。</x:v>
+      </x:c>
+      <x:c r="H35" s="11" t="str">
+        <x:v>FULL_TEXT</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" ht="206" customHeight="1">
+      <x:c r="A36" s="4" t="str">
         <x:v>C11</x:v>
       </x:c>
-      <x:c r="B34" s="4" t="str">
+      <x:c r="B36" s="4" t="str">
         <x:v>Integrated take-off management and trajectory optimization for merging control in urban air mobility corridors（2026）</x:v>
       </x:c>
-      <x:c r="C34" s="4" t="str">
+      <x:c r="C36" s="4" t="str">
         <x:v>方法：提出结构化起飞空域和分层协同起飞—合流管理（HCTMM）。结构化起飞空域用TM section、多层走廊和direct/indirect connectivity简化eVTOL动力学与障碍约束；战术层依据安全性和有效性原则，以规则型搜索选择动态合流点并协调起飞时刻；运行层用最优控制/伪谱GPOPS-II求解起飞爬升—合流轨迹，联合最小化飞行时间和控制代价并显式满足动力学、机械、安全和边界约束。比较固定合流点ATFM、动态点贪心穷举GES和规则穷举RES。
 场景/设定：Case 1为单走廊—单vertiport：走廊段长度Lc=305 m，起飞时刻[6,36,66,96,126,156] s，6架合流eVTOL；走廊流量以Bernoulli进入概率ρ=0.05（轻流）或0.15（重流）生成，初始5架走廊eVTOL，轻/重场景另有39/59架通过观察区。Case 2为多走廊—vertiport协同，4个vertiport、19架合流eVTOL和61架走廊eVTOL；参数含Tmax=230 s、Ls=50 m、T=6 s、最大速度40 m/s、最大爬升率9 m/s，使用MATLAB R2022b/GPOPS-II。</x:v>
       </x:c>
-      <x:c r="D34" s="4" t="str">
+      <x:c r="D36" s="4" t="str">
         <x:v>主要结论：HCTMM在轻流和重流下为动态合流点保持前后机安全间隔，并通过起飞时刻协调把空中等待转化为受控地面延误；相对于固定合流点ATFM，合流轨迹更平滑、完成/旅行时间和大多数控制代价更低。与GES/RES相比，HCTMM在轻/重流下选择与RES相同的合流对，但计算时间显著更短；多vertiport案例中所有合流eVTOL均成功进入走廊，结构化TM section使计算时间保持实时量级。
 定量结果：Case 1表2中，轻流6架任务的HCTMM完成时间为41.1、71.1、101.1、131.1、180.9、191.1 s；重流为41.1、71.1、101.1、131.1、193.9、216.8 s，ATFM在重流M6未在Tmax内完成。表3 HCTMM计算时间为轻流4.42 s、重流5.83 s；RES为9.67/10.84 s；GES为15.94/68.80 s，保留规划时间阈值T=6 s。Case 2含19架合流和61架走廊eVTOL，TM section将平均计算时间保持在6 s以下，约为无TM设计的二分之一至三分之一。</x:v>
       </x:c>
-      <x:c r="E34" s="4" t="str">
+      <x:c r="E36" s="4" t="str">
         <x:v>§6 p.24明确提出未来需研究更复杂走廊结构（例如多航道），并研究走廊eVTOL协同控制，以权衡合流eVTOL的起飞延误与走廊内协调合流产生的额外延误。</x:v>
       </x:c>
-      <x:c r="F34" s="4" t="str">
-        <x:v>全文评价：已经把起飞调度、动态合流点和动力学约束轨迹联合，“调度加可执行轨迹”不是空白。其走廊与起飞合流场景可用于比较终端在场流协作、服务资源和动态能量反馈；在线构形变化仅作为可选扩展。</x:v>
-      </x:c>
-      <x:c r="G34" s="4" t="str">
-        <x:v>作为最新直接对照，重点比较终端在场流、资源占用与动态能量反馈，不能仅改为降落就称创新；在线构形仅可选扩展。</x:v>
-      </x:c>
-      <x:c r="H34" s="11" t="str">
+      <x:c r="F36" s="4" t="str">
+        <x:v>全文评价：已联合起飞调度、动态合流点与动力学轨迹，调度加可执行轨迹不是空白。其固定走廊起飞合流业务与多向独立OD软引导不同；范围差异本身不证明创新或性能。</x:v>
+      </x:c>
+      <x:c r="G36" s="4" t="str">
+        <x:v>合流与轨迹联合决策的边界参考，区分保留个体决策的软引导与全轨迹集中优化。</x:v>
+      </x:c>
+      <x:c r="H36" s="11" t="str">
         <x:v>FULL_TEXT</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re1bd1916123f4f1c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra96a0f183dd44cbd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2292,107 +2356,224 @@
 备注：属于 U2U tactical deconfliction 方法邻域；其系统级动态空域构形和宏观反馈仍未展开。</x:v>
       </x:c>
     </x:row>
-    <x:row r="12" ht="150" customHeight="1">
+    <x:row r="12" ht="192" customHeight="1">
       <x:c r="A12" s="4" t="str">
-        <x:v>B01</x:v>
+        <x:v>A11</x:v>
       </x:c>
       <x:c r="B12" s="4" t="str">
-        <x:v>★ Victor L. Knoop; Joost Ellerbroek; Mark ter Heide; Serge Hoogendoorn</x:v>
+        <x:v>★ Boldizsár Balázs; Gábor Vásárhelyi</x:v>
       </x:c>
       <x:c r="C12" s="4" t="str">
-        <x:v>Transportation Research Record, 2679(2), 960-970</x:v>
+        <x:v>2018 IEEE International Conference on Robotics and Automation (ICRA), pp. 6365–6372</x:v>
       </x:c>
       <x:c r="D12" s="4" t="n">
-        <x:v>2025</x:v>
+        <x:v>2018</x:v>
       </x:c>
       <x:c r="E12" s="4" t="str">
-        <x:v>10.1177/03611981241265683</x:v>
+        <x:v>10.1109/ICRA.2018.8461073</x:v>
       </x:c>
       <x:c r="F12" s="4" t="str">
-        <x:v>https://journals.sagepub.com/doi/10.1177/03611981241265683</x:v>
+        <x:v>https://ieeexplore.ieee.org/document/8461073</x:v>
       </x:c>
       <x:c r="G12" s="4" t="str">
-        <x:v>https://repository.tudelft.nl/file/File_94afefaf-db6e-407b-9418-5a5711cc64d2?download=1</x:v>
-      </x:c>
-      <x:c r="H12" s="4" t="str">
-        <x:v>originals/B01.pdf</x:v>
-      </x:c>
-      <x:c r="I12" s="4" t="str">
-        <x:v>extracted/B01.txt</x:v>
-      </x:c>
+        <x:v>https://hal.elte.hu/~vasarhelyi/doc/balazs2018coordinated.pdf</x:v>
+      </x:c>
+      <x:c r="H12" s="4" t="str"/>
+      <x:c r="I12" s="4" t="str"/>
       <x:c r="J12" s="4" t="str">
         <x:v>publisher</x:v>
       </x:c>
       <x:c r="K12" s="4" t="str">
+        <x:v>二维开放水平空域；crosswalk为两侧往返交叉流，star为中心共同目标与边界目标交替。仿真含有限通信范围、时延、传感噪声和有限加速度；优化用100架、250 m方形区域，最终实飞为30架、150×150 m、期望速度6 m/s、无风晴天。</x:v>
+      </x:c>
+      <x:c r="L12" s="4" t="str">
+        <x:v>Crosswalk密度扫描用100架；每个测量点平均20次10 min仿真，Fig.5标最大通量0.096/s，位于平均自由程36 m；通量定义为有效速度/平均自由程，非城市网络完成出流。
+Star场景在48个平均自由程值22–365 m上，每点20次仿真；到达中心的平均间隔约12±1 s，各次仿真报告零碰撞。
+30架户外实飞在150×150 m区域、6 m/s期望速度下进行；Fig.8为15 min飞行日志，归一化目标方向有效速度约0.4–0.5。</x:v>
+      </x:c>
+      <x:c r="M12" s="4" t="str">
+        <x:v>PDF p.1 / printed p.6365：标题、两名作者、IEEE ICRA 2018会议信息与摘要。
+PDF pp.2–4, Sec. II-A–E, Eqs.2–10：各向异性参数A、选择性对齐、切向参数T、自驱和虚拟排队。
+PDF pp.5–6, Sec. III, Table I, Figs.4–5：两种场景、CMA-ES与人工调参、密度曲线、0.096/s峰值及star的12±1 s。
+PDF pp.6–8, Sec. IV–V, Figs.6–8：户外平台和30架实飞、初始过渡局限、全文讨论结尾与参考文献。</x:v>
+      </x:c>
+      <x:c r="N12" s="11" t="str">
+        <x:v>FULL_TEXT</x:v>
+      </x:c>
+      <x:c r="O12" s="4" t="str">
+        <x:v>PUBLISHED_CONFERENCE</x:v>
+      </x:c>
+      <x:c r="P12" s="4" t="str">
+        <x:v>VERIFIED</x:v>
+      </x:c>
+      <x:c r="Q12" s="4" t="str">
+        <x:v>历史访问尝试：公开作者PDF由web工具成功读取，8页，全文文本行0–956已分段连续核对，含方法、实验、讨论、图注及参考文献。
+本地普通沙箱下载遇WinError10013；获网络审批后的Python HTTPS遇SSL EOF，Windows Invoke-WebRequest重试仍SSL失败；同一已核作者站HTTP入口仅追加尝试一次，也返回请求发送错误；没有生成A11.pdf或A11.txt。
+IEEE文档8461073页面返回JavaScript机器人检查；正式发表信息由带IEEE版权和页码的公开正文核实，DOI另由Springer正式A07参考文献核对；未绕过访问限制。
+备注：2026-10-22补充。公开作者副本保留IEEE出版排版；FULL_TEXT表示本次已阅读全文8页，不表示本地PDF存在。local_pdf/local_text为空，因为本地下载失败；不虚构本地路径。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="206" customHeight="1">
+      <x:c r="A13" s="4" t="str">
+        <x:v>A12</x:v>
+      </x:c>
+      <x:c r="B13" s="4" t="str">
+        <x:v>★ A. M. Veytia; C. A. Badea; J. Ellerbroek; J. Hoekstra; N. Patrinopoulou; I. Daramouskas; V. Lappas; V. Kostopoulos; V. de Vries; J. van Ham; E. Sunil; P. Menendez Ponte Alonso; J. Rodrigo Villazon Terrazas; D. Bereziat; A. Vidosavljevic; L. Sedov</x:v>
+      </x:c>
+      <x:c r="C13" s="4" t="str">
+        <x:v>SESAR Innovation Days 2022</x:v>
+      </x:c>
+      <x:c r="D13" s="4" t="n">
+        <x:v>2022</x:v>
+      </x:c>
+      <x:c r="E13" s="4" t="str"/>
+      <x:c r="F13" s="4" t="str">
+        <x:v>https://www.sesarju.eu/sites/default/files/documents/sid/2022/paper_88.pdf</x:v>
+      </x:c>
+      <x:c r="G13" s="4" t="str">
+        <x:v>https://www.sesarju.eu/sites/default/files/documents/sid/2022/paper_88.pdf</x:v>
+      </x:c>
+      <x:c r="H13" s="4" t="str">
+        <x:v>originals/A12.pdf</x:v>
+      </x:c>
+      <x:c r="I13" s="4" t="str">
+        <x:v>extracted/A12.txt</x:v>
+      </x:c>
+      <x:c r="J13" s="4" t="str">
+        <x:v>publisher</x:v>
+      </x:c>
+      <x:c r="K13" s="4" t="str">
+        <x:v>维也纳中心8 km宽、500 ft高的圆柱空域，包含街道约束空域、开放空域和地理围栏；16个垂直层。两类简化Matrice 600 Pro机型巡航20/30 kts，四类任务与四级优先级；5档交通水平，风速0/1/3/5 kts，非合作机0/33/66/100架，各设置9次随机重复。</x:v>
+      </x:c>
+      <x:c r="L13" s="4" t="str">
+        <x:v>Table II将5档交通列为平均同时在飞机数1660/3340/4990/6650/8290；每设置9次重复。仅首小时安排起飞，仿真运行90–180 min直到全部到达；不得混同小时总架次。
+高密度设置下，混合概念在约束空域的峰值密度约为另两概念一半，但消退更慢；高/极高需求下分布式每航班冲突数比其他概念高约一个数量级，侵入差异远小于冲突差异。
+混合概念专用解脱层使可巡航垂直空间仅为集中概念一半；所有密度下其侵入最少，但需求延误较高，且高密度下延误分散也高于集中概念。</x:v>
+      </x:c>
+      <x:c r="M13" s="4" t="str">
+        <x:v>PDF p.1：题名、16名作者及机构分列、摘要；官方SESAR路径sid/2022核验会议年份，未核到DOI。
+PDF pp.2–3, Sec. II, Table I：三种组织概念、不同空域结构、航向分层、混合巡航/解脱层、中央交通成本与可选单机重规划。
+PDF pp.3–4, Sec. III, Table II：空域/机型/任务、交通数量、9次重复、32 m与25 ft分离、10 s前视和仿真时长。
+PDF pp.4–7, Sec. IV, Figs.2–13：密度/冲突/侵入/效率/延误/公平及异常条件结果。
+PDF pp.7–8, Sec. V–VI：结构与职责的混杂、混合仅半数巡航空间、环路方向一致性与绕行代价、结论和改进建议；p.8参考文献。</x:v>
+      </x:c>
+      <x:c r="N13" s="11" t="str">
+        <x:v>FULL_TEXT</x:v>
+      </x:c>
+      <x:c r="O13" s="4" t="str">
+        <x:v>PUBLISHED_CONFERENCE</x:v>
+      </x:c>
+      <x:c r="P13" s="4" t="str">
+        <x:v>VERIFIED_PRIMARY</x:v>
+      </x:c>
+      <x:c r="Q13" s="4" t="str">
+        <x:v>历史访问尝试：官方SESAR PDF由web全文打开；Windows Invoke-WebRequest通过获准网络下载4,354,780 bytes。
+本地PDF头为%PDF-，pypdf成功解析8页，逐页提取并完整阅读标题、方法、实验、结果、讨论、结论及参考文献。
+PDF封面按作者行核验16名作者，机构行未混入作者；未核到DOI，故留空。
+备注：2026-10-22补充；为SESAR Innovation Days 2022正式会议公开稿。对照同时改变结构、职责和可巡航空间，不能把效果全部归因中心化程度；本篇不是经方向有序度识别的MFD控制论文。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="150" customHeight="1">
+      <x:c r="A14" s="4" t="str">
+        <x:v>B01</x:v>
+      </x:c>
+      <x:c r="B14" s="4" t="str">
+        <x:v>★ Victor L. Knoop; Joost Ellerbroek; Mark ter Heide; Serge Hoogendoorn</x:v>
+      </x:c>
+      <x:c r="C14" s="4" t="str">
+        <x:v>Transportation Research Record, 2679(2), 960-970</x:v>
+      </x:c>
+      <x:c r="D14" s="4" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="E14" s="4" t="str">
+        <x:v>10.1177/03611981241265683</x:v>
+      </x:c>
+      <x:c r="F14" s="4" t="str">
+        <x:v>https://journals.sagepub.com/doi/10.1177/03611981241265683</x:v>
+      </x:c>
+      <x:c r="G14" s="4" t="str">
+        <x:v>https://repository.tudelft.nl/file/File_94afefaf-db6e-407b-9418-5a5711cc64d2?download=1</x:v>
+      </x:c>
+      <x:c r="H14" s="4" t="str">
+        <x:v>originals/B01.pdf</x:v>
+      </x:c>
+      <x:c r="I14" s="4" t="str">
+        <x:v>extracted/B01.txt</x:v>
+      </x:c>
+      <x:c r="J14" s="4" t="str">
+        <x:v>publisher</x:v>
+      </x:c>
+      <x:c r="K14" s="4" t="str">
         <x:v>Amsterdam Schiphol 附近五个荷兰 CTA 合并区域，面积 42,807 km²，高度 5,500-19,500 ft，体积 182,667 km³；使用 Delft 接收的 ADS-B 数据，覆盖 2019 年 4 月、8 月和 2020 年 4 月、8 月，包含进出 Schiphol 及邻近机场的航班；单个 30 min 聚合区间通常有 60 架以上飞机。</x:v>
       </x:c>
-      <x:c r="L12" s="4" t="str">
+      <x:c r="L14" s="4" t="str">
         <x:v>观测密度约 0-0.0002 架/km³；基于 5 nmi 水平和 ±1000 ft 垂直间隔的理论紧密填充上限约 0.0051 架/km³（PDF p.9，正文 p.7）。
 拟合 Greenshields 抛物线的自由流速度为 442 km/h（239 knots）；拟合的 jam density 为 7.8×10^-4 架/km³，最大流量对应密度为 3.9×10^-4 架/km³（PDF pp.9-10，正文 pp.7-8）。
 低密度区的 free-flow efficiency 略高于 80%；2020 年 4 月航班量比 2019 年 4 月少 87%；邻近机场相关航班平均约占研究空域航班 17%（PDF pp.7-8、10）。</x:v>
       </x:c>
-      <x:c r="M12" s="4" t="str">
+      <x:c r="M14" s="4" t="str">
         <x:v>PDF pp.3-5（摘要、研究目的与三维 Edie 定义）
 PDF pp.6-8（30 min 聚合、Schiphol CTA 数据与 ADS-B 处理）
 PDF pp.9-11（MFD、442 km/h、拟合密度、效率与航迹）
 PDF pp.11-12（Conclusions and Potential Applications 及作者限制）</x:v>
       </x:c>
-      <x:c r="N12" s="11" t="str">
-        <x:v>FULL_TEXT</x:v>
-      </x:c>
-      <x:c r="O12" s="4" t="str">
+      <x:c r="N14" s="11" t="str">
+        <x:v>FULL_TEXT</x:v>
+      </x:c>
+      <x:c r="O14" s="4" t="str">
         <x:v>PUBLISHED</x:v>
       </x:c>
-      <x:c r="P12" s="4" t="str">
+      <x:c r="P14" s="4" t="str">
         <x:v>VERIFIED_PRIMARY</x:v>
       </x:c>
-      <x:c r="Q12" s="4" t="str">
+      <x:c r="Q14" s="4" t="str">
         <x:v>历史访问尝试：TU Delft Institutional Repository 公开 PDF：HTTP 200，文件头 %PDF，pypdf 解析 13 页。
 SAGE DOI/期刊页：标题、作者、DOI、卷期页码和日期核验通过；官方页标明 online first 为 2024-08-24，卷2679(2)期刊出版为 2025-02。
 备注：常规飞机机场 CTA 经验研究；作为低空 UAV 宏观模型的迁移背景保留。TU Delft 文件标示为 final published version，并附 Taverne 公开说明。卷期引用采用 issue year 2025；2024 为 online-first 年份。</x:v>
       </x:c>
     </x:row>
-    <x:row r="13" ht="206" customHeight="1">
-      <x:c r="A13" s="4" t="str">
+    <x:row r="15" ht="206" customHeight="1">
+      <x:c r="A15" s="4" t="str">
         <x:v>B02</x:v>
       </x:c>
-      <x:c r="B13" s="4" t="str">
+      <x:c r="B15" s="4" t="str">
         <x:v>★ Zhengyi Wang; Daniel Delahaye; Jean-Loup Farges; Sameer Alam</x:v>
       </x:c>
-      <x:c r="C13" s="4" t="str">
+      <x:c r="C15" s="4" t="str">
         <x:v>Transportation Research Part C: Emerging Technologies, 142, 103776</x:v>
       </x:c>
-      <x:c r="D13" s="4" t="n">
+      <x:c r="D15" s="4" t="n">
         <x:v>2022</x:v>
       </x:c>
-      <x:c r="E13" s="4" t="str">
+      <x:c r="E15" s="4" t="str">
         <x:v>10.1016/j.trc.2022.103776</x:v>
       </x:c>
-      <x:c r="F13" s="4" t="str">
+      <x:c r="F15" s="4" t="str">
         <x:v>https://www.sciencedirect.com/science/article/pii/S0968090X22002054</x:v>
       </x:c>
-      <x:c r="G13" s="4" t="str">
+      <x:c r="G15" s="4" t="str">
         <x:v>https://www.sciencedirect.com/science/article/pii/S0968090X22002054</x:v>
       </x:c>
-      <x:c r="H13" s="4" t="str">
+      <x:c r="H15" s="4" t="str">
         <x:v>supplement/1-s2.0-S0968090X22002054-main.pdf</x:v>
       </x:c>
-      <x:c r="I13" s="4" t="str">
+      <x:c r="I15" s="4" t="str">
         <x:v>extracted/supplement_B02.txt</x:v>
       </x:c>
-      <x:c r="J13" s="4" t="str">
+      <x:c r="J15" s="4" t="str">
         <x:v>publisher</x:v>
       </x:c>
-      <x:c r="K13" s="4" t="str">
+      <x:c r="K15" s="4" t="str">
         <x:v>新加坡包裹配送固定网络：63节点、110链路、24组OD、3水平层，含3个droneport、5个配送站和55个waypoint，层距15 m且有垂直连接。Case1为随OD序号增长的对称双向需求，Case2为不平衡随机需求；同类航空器水平120 km/h、垂直5 km/h，最大航程20 km、续航2000 s。每种非AON算法运行100个随机种子，与AON、SA、DA、MSA等比较（PDF pp.10–13 §5，Table2–4）。</x:v>
       </x:c>
-      <x:c r="L13" s="4" t="str">
+      <x:c r="L15" s="4" t="str">
         <x:v>PDF p.13 Table3：Case1相对随机初始分配的复杂度680081.00降至65005.20，降幅90.44%±0.53%（95%CI）；两阶段总耗时13.62±0.52 s，100种子。
 PDF p.13 Table4：Case2相对随机初始复杂度665702.86降至52450.41，降幅92.12%±0.35%（95%CI）；总耗时14.12±0.33 s，100种子。
 PDF p.13 Table3：Case1方案平均航程10.27±0.08 km、时间323.83±2.52 s、加权能量184.68±1.43；AON分别7.16 km、248.00 s、130.27，指标及比较对象不可互换。
 PDF p.13 Table4：Case2方案平均10.39±0.06 km、328.58±1.84 s、加权能量179.49±1.11；AON为7.48 km、258.21 s、131.06。能量数值为模型加权指标，非kWh或SOC。</x:v>
       </x:c>
-      <x:c r="M13" s="4" t="str">
+      <x:c r="M15" s="4" t="str">
         <x:v>p1 title,DOI
 pp2–6 network/assumptions/P1/LDS
 pp7–10 algorithm
@@ -2400,63 +2581,63 @@
 p19 conclusion and future work
 pp19–22 WMMSE/SVD and LDS proofs/typical situations;pp22–23 references</x:v>
       </x:c>
-      <x:c r="N13" s="11" t="str">
-        <x:v>FULL_TEXT</x:v>
-      </x:c>
-      <x:c r="O13" s="4" t="str">
+      <x:c r="N15" s="11" t="str">
+        <x:v>FULL_TEXT</x:v>
+      </x:c>
+      <x:c r="O15" s="4" t="str">
         <x:v>PUBLISHED</x:v>
       </x:c>
-      <x:c r="P13" s="4" t="str">
+      <x:c r="P15" s="4" t="str">
         <x:v>VERIFIED_PRIMARY</x:v>
       </x:c>
-      <x:c r="Q13" s="4" t="str">
+      <x:c r="Q15" s="4" t="str">
         <x:v>历史访问尝试：ScienceDirect publisher record：标题、作者、2022、卷 142、文章号 103776 和 DOI 核验通过；全文受组织访问限制。
 HAL/ResearchGate 等公开候选页面检索；未找到可直接、稳定且合法下载的该正式论文全文。
 2026-10-22：用户提供正式PDF，直接核对标题/DOI并阅读全文（23页）；本次本地文件为 research/low_altitude_phd_20261013/supplement/1-s2.0-S0968090X22002054-main.pdf。此前访问失败记录仅为历史，不代表当前缺全文。
 备注：2026-10-22用户提供23页正式期刊PDF，已阅读全文。LDS复杂度降幅以随机初始分配为分母；已有航程/续航/能耗预算，不等于逐机SOC闭环。</x:v>
       </x:c>
     </x:row>
-    <x:row r="14" ht="192" customHeight="1">
-      <x:c r="A14" s="4" t="str">
+    <x:row r="16" ht="192" customHeight="1">
+      <x:c r="A16" s="4" t="str">
         <x:v>B03</x:v>
       </x:c>
-      <x:c r="B14" s="4" t="str">
+      <x:c r="B16" s="4" t="str">
         <x:v>★ Zhengyi Wang; Daniel Delahaye; Jean-Loup Farges; Sameer Alam</x:v>
       </x:c>
-      <x:c r="C14" s="4" t="str">
+      <x:c r="C16" s="4" t="str">
         <x:v>Transportation Research Part C: Emerging Technologies, 154, 104279</x:v>
       </x:c>
-      <x:c r="D14" s="4" t="n">
+      <x:c r="D16" s="4" t="n">
         <x:v>2023</x:v>
       </x:c>
-      <x:c r="E14" s="4" t="str">
+      <x:c r="E16" s="4" t="str">
         <x:v>10.1016/j.trc.2023.104279</x:v>
       </x:c>
-      <x:c r="F14" s="4" t="str">
+      <x:c r="F16" s="4" t="str">
         <x:v>https://www.sciencedirect.com/science/article/abs/pii/S0968090X23002681</x:v>
       </x:c>
-      <x:c r="G14" s="4" t="str">
+      <x:c r="G16" s="4" t="str">
         <x:v>https://enac.hal.science/hal-04180867/file/DTIS22224.1693569649_postprint.pdf</x:v>
       </x:c>
-      <x:c r="H14" s="4" t="str">
+      <x:c r="H16" s="4" t="str">
         <x:v>supplement/1-s2.0-S0968090X23002681-main.pdf</x:v>
       </x:c>
-      <x:c r="I14" s="4" t="str">
+      <x:c r="I16" s="4" t="str">
         <x:v>extracted/supplement_B03.txt</x:v>
       </x:c>
-      <x:c r="J14" s="4" t="str">
+      <x:c r="J16" s="4" t="str">
         <x:v>publisher</x:v>
       </x:c>
-      <x:c r="K14" s="4" t="str">
+      <x:c r="K16" s="4" t="str">
         <x:v>预设计新加坡包裹配送网络含332节点、745链路、7个vertiport、12个配送站和84组OD；150/175/200/225/250 ft五层，垂直连接受限，采用多样K最短路径。仿真文本给09:00–15:00六个需求时段；同类航空器水平54 km/h、垂直15 km/h，链路容量15000 veh/h、最小有效流20 veh/h。Java在i7-12700H/16 GB上运行100个随机种子，比较PSA及DA等代表算法（PDF pp.13–16，Tables2–4）。</x:v>
       </x:c>
-      <x:c r="L14" s="4" t="str">
+      <x:c r="L16" s="4" t="str">
         <x:v>PDF p.15 Table4：100种子下PSA总目标67157.45±146.87，相对初始99081.42±368.48降低32.20%±0.29%；耗时143.47±3.74 s，均95%CI，属整个聚合分配实验。
 PDF p.15 Table4：PSA复杂度302743.55±1574.53，初始585380.95±3627.11；拥堵40981.22±36.90，初始45048.14±27.92。二者均为模型指标，不是实测冲突次数。
 PDF p.15 Table4：PSA时间1233.61±0.48 s、航程18.28±0.01 km，初始1201.94±0.41 s、17.84±0.01 km；DA为1198.18±0.38 s、17.78±0.01 km。
 PDF pp.14–15 §4.1.1：1–20线程各计时10000次转移，约3倍加速，8线程后无明显继续改善；此为转移计算加速，非逐机闭环周期。</x:v>
       </x:c>
-      <x:c r="M14" s="4" t="str">
+      <x:c r="M16" s="4" t="str">
         <x:v>p1 title/DOI/publisher format
 pp2–3 UTM scope, prior static assumptions and contribution
 pp4–9 fixed graph, flow propagation, capacity,energy,LDS
@@ -2465,16 +2646,16 @@
 pp16–20 allocation/congestion outputs and limitations
 pp21–23 WMMSE/SVD and DA/PM comparison algorithms;pp23–25 references</x:v>
       </x:c>
-      <x:c r="N14" s="11" t="str">
-        <x:v>FULL_TEXT</x:v>
-      </x:c>
-      <x:c r="O14" s="4" t="str">
+      <x:c r="N16" s="11" t="str">
+        <x:v>FULL_TEXT</x:v>
+      </x:c>
+      <x:c r="O16" s="4" t="str">
         <x:v>PUBLISHED</x:v>
       </x:c>
-      <x:c r="P14" s="4" t="str">
+      <x:c r="P16" s="4" t="str">
         <x:v>VERIFIED_PRIMARY</x:v>
       </x:c>
-      <x:c r="Q14" s="4" t="str">
+      <x:c r="Q16" s="4" t="str">
         <x:v>历史访问尝试：ScienceDirect publisher abstract：HTTP 可检索，全文需组织访问。
 HAL postprint URL、preview URL、document URL：返回 503 或 anti-bot HTML，未保存为 PDF，故不声称已阅读全文。
 ResearchGate 页面可检索摘要/局部正文，但未将其作为本地全文来源。
@@ -2482,47 +2663,47 @@
 备注：2026-10-22用户提供25页出版社正式PDF，已全文阅读；本次版本为publisher，旧HAL accepted路径仅为历史来源。已知需求的准动态分配与实际微观感知闭环须区分。</x:v>
       </x:c>
     </x:row>
-    <x:row r="15" ht="206" customHeight="1">
-      <x:c r="A15" s="4" t="str">
+    <x:row r="17" ht="206" customHeight="1">
+      <x:c r="A17" s="4" t="str">
         <x:v>B04</x:v>
       </x:c>
-      <x:c r="B15" s="4" t="str">
+      <x:c r="B17" s="4" t="str">
         <x:v>★ Christopher Cummings; Hani Mahmassani</x:v>
       </x:c>
-      <x:c r="C15" s="4" t="str">
+      <x:c r="C17" s="4" t="str">
         <x:v>Transportation Research Part C: Emerging Technologies, 159, 104467</x:v>
       </x:c>
-      <x:c r="D15" s="4" t="n">
+      <x:c r="D17" s="4" t="n">
         <x:v>2024</x:v>
       </x:c>
-      <x:c r="E15" s="4" t="str">
+      <x:c r="E17" s="4" t="str">
         <x:v>10.1016/j.trc.2023.104467</x:v>
       </x:c>
-      <x:c r="F15" s="4" t="str">
+      <x:c r="F17" s="4" t="str">
         <x:v>https://www.sciencedirect.com/science/article/pii/S0968090X23004576</x:v>
       </x:c>
-      <x:c r="G15" s="4" t="str">
+      <x:c r="G17" s="4" t="str">
         <x:v>https://www.sciencedirect.com/science/article/pii/S0968090X23004576</x:v>
       </x:c>
-      <x:c r="H15" s="4" t="str">
+      <x:c r="H17" s="4" t="str">
         <x:v>supplement/1-s2.0-S0968090X23004576-main.pdf</x:v>
       </x:c>
-      <x:c r="I15" s="4" t="str">
+      <x:c r="I17" s="4" t="str">
         <x:v>extracted/supplement_B04.txt</x:v>
       </x:c>
-      <x:c r="J15" s="4" t="str">
+      <x:c r="J17" s="4" t="str">
         <x:v>publisher</x:v>
       </x:c>
-      <x:c r="K15" s="4" t="str">
+      <x:c r="K17" s="4" t="str">
         <x:v>无结构空域中，在围绕中心测量区的圆周交替配置起终vertiport以近似随机航向；正态出发时刻产生密度升降。每次仿真5000 s，按300 s窗口聚合；间隔和最大速度各设五档，速度80/100/120/150/180 mph。尽管模拟器有三维起降过程，测量区刻意排除起降影响，巡航全部同高度且禁止垂直绕行；冲突数实验关闭解脱而保留探测，速度/流量实验启用解脱（PDF pp.11–18 §5，Figs12–20）。</x:v>
       </x:c>
-      <x:c r="L15" s="4" t="str">
+      <x:c r="L17" s="4" t="str">
         <x:v>PDF pp.13–14 Figs12–13：间隔0.5556/0.4444/0.3333 mile时冲突—密度拟合R²为0.912/0.889/0.869；180/150/120/100/80 mph时为0.819/0.810/0.914/0.925/0.922。
 PDF p.16 Fig15：间隔按0.5556至0.1111 mile五档递减，实际速度—密度R²为0.888/0.931/0.802/0.914/0.567；不能概括所有场景均高拟合。
 PDF p.17 Figs17–18：有效速度—密度R²在五档间隔下为0.864/0.885/0.709/0.926/0.657，在180至80 mph五档下为0.836/0.747/0.828/0.864/0.930。
 PDF p.18 Fig19：有效流—密度R²在间隔0.5556/0.4444/0.3333/0.2222/0.1111 mile时为0.870/0.927/0.524/0.963/0.971；为拟合优度，不是容量或安全改善百分比。</x:v>
       </x:c>
-      <x:c r="M15" s="4" t="str">
+      <x:c r="M17" s="4" t="str">
         <x:v>p1 title/DOI
 pp3–7 variable definitions/theory/Eqs1–16
 pp8–11 theoretical patterns (arbitrary numeric values,not calibrated operational capacities)
@@ -2531,64 +2712,64 @@
 pp17–20 implications/author limitations/future work
 pp20–21 references</x:v>
       </x:c>
-      <x:c r="N15" s="11" t="str">
-        <x:v>FULL_TEXT</x:v>
-      </x:c>
-      <x:c r="O15" s="4" t="str">
+      <x:c r="N17" s="11" t="str">
+        <x:v>FULL_TEXT</x:v>
+      </x:c>
+      <x:c r="O17" s="4" t="str">
         <x:v>PUBLISHED</x:v>
       </x:c>
-      <x:c r="P15" s="4" t="str">
+      <x:c r="P17" s="4" t="str">
         <x:v>VERIFIED_PRIMARY</x:v>
       </x:c>
-      <x:c r="Q15" s="4" t="str">
+      <x:c r="Q17" s="4" t="str">
         <x:v>历史访问尝试：ScienceDirect publisher record：标题、作者、2024、卷 159、文章号 104467 和 DOI 核验通过；全文访问受限。
 未找到公开机构全文，未下载 PDF。
 2026-10-22：用户提供正式PDF，直接核对标题/DOI并阅读全文（21页）；本次本地文件为 research/low_altitude_phd_20261013/supplement/1-s2.0-S0968090X23004576-main.pdf。此前访问失败记录仅为历史，不代表当前缺全文。
 备注：2026-10-22用户提供21页正式期刊PDF，已阅读全文并核对关键图。标题4-D不代表实验已经验证三维巡航动力学；预测冲突数也不等于实际碰撞/LOS。</x:v>
       </x:c>
     </x:row>
-    <x:row r="16" ht="234" customHeight="1">
-      <x:c r="A16" s="4" t="str">
+    <x:row r="18" ht="234" customHeight="1">
+      <x:c r="A18" s="4" t="str">
         <x:v>B05</x:v>
       </x:c>
-      <x:c r="B16" s="4" t="str">
+      <x:c r="B18" s="4" t="str">
         <x:v>★ Yazan Safadi; Rao Fu; Quan Quan; Jack Haddad</x:v>
       </x:c>
-      <x:c r="C16" s="4" t="str">
+      <x:c r="C18" s="4" t="str">
         <x:v>Transportation Research Part C 152 (2023) 104141</x:v>
       </x:c>
-      <x:c r="D16" s="4" t="n">
+      <x:c r="D18" s="4" t="n">
         <x:v>2023</x:v>
       </x:c>
-      <x:c r="E16" s="4" t="str">
+      <x:c r="E18" s="4" t="str">
         <x:v>10.1016/j.trc.2023.104141</x:v>
       </x:c>
-      <x:c r="F16" s="4" t="str">
+      <x:c r="F18" s="4" t="str">
         <x:v>https://www.sciencedirect.com/science/article/pii/S0968090X23001304</x:v>
       </x:c>
-      <x:c r="G16" s="4" t="str">
+      <x:c r="G18" s="4" t="str">
         <x:v>https://www.sciencedirect.com/science/article/pii/S0968090X23001304</x:v>
       </x:c>
-      <x:c r="H16" s="4" t="str">
+      <x:c r="H18" s="4" t="str">
         <x:v>supplement/1-s2.0-S0968090X23001304-main.pdf</x:v>
       </x:c>
-      <x:c r="I16" s="4" t="str">
+      <x:c r="I18" s="4" t="str">
         <x:v>extracted/supplement_B05.txt</x:v>
       </x:c>
-      <x:c r="J16" s="4" t="str">
+      <x:c r="J18" s="4" t="str">
         <x:v>publisher</x:v>
       </x:c>
-      <x:c r="K16" s="4" t="str">
+      <x:c r="K18" s="4" t="str">
         <x:v>固定无结构网络内起终点在边界均匀随机，无预设航路/交叉口；默认最大速度20 m/s、加速度5 m/s²，安全/避让/探测半径15/22.5/45.5 m，梯形需求、一般运行1.5 h。六组实验比较2×2、1×1、0.5×0.5 km二维网络，10/15/20 m安全半径，随机半径与速度异质性，waypoint与目的地线，以及0.5×0.5×0.1 km三维网络；三维运行0.5 h（PDF pp.9–16 §4）。</x:v>
       </x:c>
-      <x:c r="L16" s="4" t="str">
+      <x:c r="L18" s="4" t="str">
         <x:v>PDF p.12 Fig9：2×2 km waypoint观测临界点为229架、1.8667架/s，而拟合曲线峰值为283.86架、1.47架/s；两者不得混写。
 PDF p.18 Table2：同rs=15 m、vmax=20 m/s时，2×2/1×1/0.5×0.5 km拟合临界累积为283.86/80.49/21.57架，峰值出流1.47/0.80/0.45架/s。
 PDF p.18 Table2：2×2 km中rs=10/15/20 m的拟合峰值出流3.05/1.47/0.89架/s；0.5×0.5 km中仅半径异质/仅速度异质/两者异质为0.38/0.41/0.32架/s，齐次对照0.45架/s。
 PDF p.18 Table1：同0.5×0.5 km、rs15、vmax20，waypoint与目的地线峰值0.45/0.54架/s，临界累积21.57/22.62架；不是共同到达点不变的纯算法收益。
 PDF p.18 Table2：三维0.5×0.5×0.1 km waypoint拟合临界累积42.00架、峰值1.10架/s；为仿真拟合，不是实测容量。</x:v>
       </x:c>
-      <x:c r="M16" s="4" t="str">
+      <x:c r="M18" s="4" t="str">
         <x:v>p.1 metadata
 pp.3-7 microscopic controller/assumptions/Equations 1-23
 pp.7-8 MFD definitions/Equations 24-30
@@ -2597,63 +2778,63 @@
 pp.19-20 conclusions/future work
 pp.22-24 Appendix B/Algorithms 1-7 including safety queue and aggregation</x:v>
       </x:c>
-      <x:c r="N16" s="11" t="str">
-        <x:v>FULL_TEXT</x:v>
-      </x:c>
-      <x:c r="O16" s="4" t="str">
+      <x:c r="N18" s="11" t="str">
+        <x:v>FULL_TEXT</x:v>
+      </x:c>
+      <x:c r="O18" s="4" t="str">
         <x:v>PUBLISHED</x:v>
       </x:c>
-      <x:c r="P16" s="4" t="str">
+      <x:c r="P18" s="4" t="str">
         <x:v>VERIFIED_PRIMARY</x:v>
       </x:c>
-      <x:c r="Q16" s="4" t="str">
+      <x:c r="Q18" s="4" t="str">
         <x:v>历史访问尝试：ScienceDirect publisher record：标题、作者、2023、卷 152、文章号 104141 和 DOI 核验通过；PDF 显示需组织/购买。
 Technion institutional page和公开会议摘要可访问，但会议摘要不冒充正式期刊全文。
 2026-10-22：用户提供正式PDF，直接核对标题/DOI并阅读全文（26页）；本次本地文件为 research/low_altitude_phd_20261013/supplement/1-s2.0-S0968090X23001304-main.pdf。此前访问失败记录仅为历史，不代表当前缺全文。
 备注：2026-10-22用户提供26页正式期刊PDF，已全文阅读。已做异质、动态加载/滞回与3D；本篇同步微观仿真和MFD识别，并未实施MFD反馈网络控制。</x:v>
       </x:c>
     </x:row>
-    <x:row r="17" ht="206" customHeight="1">
-      <x:c r="A17" s="4" t="str">
+    <x:row r="19" ht="206" customHeight="1">
+      <x:c r="A19" s="4" t="str">
         <x:v>B06</x:v>
       </x:c>
-      <x:c r="B17" s="4" t="str">
+      <x:c r="B19" s="4" t="str">
         <x:v>★ Canqiang Weng; Tianlu Pan; Can Chen; Renxin Zhong</x:v>
       </x:c>
-      <x:c r="C17" s="4" t="str">
+      <x:c r="C19" s="4" t="str">
         <x:v>Transportation Research Part C 178 (2025) 105237</x:v>
       </x:c>
-      <x:c r="D17" s="4" t="n">
+      <x:c r="D19" s="4" t="n">
         <x:v>2025</x:v>
       </x:c>
-      <x:c r="E17" s="4" t="str">
+      <x:c r="E19" s="4" t="str">
         <x:v>10.1016/j.trc.2025.105237</x:v>
       </x:c>
-      <x:c r="F17" s="4" t="str">
+      <x:c r="F19" s="4" t="str">
         <x:v>https://www.sciencedirect.com/science/article/pii/S0968090X25002414</x:v>
       </x:c>
-      <x:c r="G17" s="4" t="str">
+      <x:c r="G19" s="4" t="str">
         <x:v>https://www.sciencedirect.com/science/article/pii/S0968090X25002414</x:v>
       </x:c>
-      <x:c r="H17" s="4" t="str">
+      <x:c r="H19" s="4" t="str">
         <x:v>supplement/1-s2.0-S0968090X25002414-main.pdf</x:v>
       </x:c>
-      <x:c r="I17" s="4" t="str">
+      <x:c r="I19" s="4" t="str">
         <x:v>extracted/supplement_B06.txt</x:v>
       </x:c>
-      <x:c r="J17" s="4" t="str">
+      <x:c r="J19" s="4" t="str">
         <x:v>publisher</x:v>
       </x:c>
-      <x:c r="K17" s="4" t="str">
+      <x:c r="K19" s="4" t="str">
         <x:v>跨河/海两区域概念网络，8个固定vertiport、4组OD，两空域均2×2×1 km且采用full mix；假设起降独立并可同时进行、航空器有避碰与留区能力。MFD由此前1 km立方体微观轨迹拟合并按面积扩展。两组120 min聚合实验在60 min切换工作日/假日模式，与固定初始SO目标比较；同控制器、峰值需求超目标20%、0.5%高斯噪声。附录另有两区域各9六角柱单元的900 s微观速度试验（PDF pp.5–6、13–21）。</x:v>
       </x:c>
-      <x:c r="L17" s="4" t="str">
+      <x:c r="L19" s="4" t="str">
         <x:v>PDF p.16 §4.2.1：120 min工作日→假日、60 min改目标的方案，相对始终固定工作日SO基线，平均排队时间降低42.3%、最大队长降低52.6%、最大完成流提高26.9%；同控制器、同需求。
 PDF p.15：工作日/假日目标累积分别(43.6,36.3)/(82.8,69.0)架；两区域临界累积110.4架，所选目标不是直接设为MFD临界点。
 PDF pp.14–15：工作日准入容量四分量(0.108,0.245,0.160,0.048)架/s，假日(0.157,0.300,0.245,0.114)架/s；由各SO分配聚合而来。
 PDF pp.20–21 Appendix A：内/外生流入各0.5架/s，前450 s均限20 m/s，之后限10/30 m/s；450–600 s内生完成流下降、外生上升，未报告闭环映射或该试验的百分比增益。</x:v>
       </x:c>
-      <x:c r="M17" s="4" t="str">
+      <x:c r="M19" s="4" t="str">
         <x:v>p.1 metadata
 pp.4-6 motivating scenario/assumptions
 pp.6-8 SO assignment and queue equations
@@ -2664,62 +2845,62 @@
 pp.20-21 separate micro example/Figs.14-15
 pp.21-23 proposition proofs</x:v>
       </x:c>
-      <x:c r="N17" s="11" t="str">
-        <x:v>FULL_TEXT</x:v>
-      </x:c>
-      <x:c r="O17" s="4" t="str">
+      <x:c r="N19" s="11" t="str">
+        <x:v>FULL_TEXT</x:v>
+      </x:c>
+      <x:c r="O19" s="4" t="str">
         <x:v>PUBLISHED</x:v>
       </x:c>
-      <x:c r="P17" s="4" t="str">
+      <x:c r="P19" s="4" t="str">
         <x:v>VERIFIED_PRIMARY</x:v>
       </x:c>
-      <x:c r="Q17" s="4" t="str">
+      <x:c r="Q19" s="4" t="str">
         <x:v>历史访问尝试：ScienceDirect publisher record：标题、作者、2025、卷 178、文章号 105237 和 DOI 核验通过；全文需组织访问。
 作者公开页面检索到正式书目信息和摘要，未找到可公开下载正式全文。
 2026-10-22：用户提供正式PDF，直接核对标题/DOI并阅读全文（24页）；本次本地文件为 research/low_altitude_phd_20261013/supplement/1-s2.0-S0968090X25002414-main.pdf。此前访问失败记录仅为历史，不代表当前缺全文。
 备注：2026-10-22用户提供24页正式期刊PDF，已全文阅读。主实验为宏观SO—控制交互，另有微观限速验证；没有把二者误写成完整逐机执行闭环。</x:v>
       </x:c>
     </x:row>
-    <x:row r="18" ht="206" customHeight="1">
-      <x:c r="A18" s="4" t="str">
+    <x:row r="20" ht="206" customHeight="1">
+      <x:c r="A20" s="4" t="str">
         <x:v>B07</x:v>
       </x:c>
-      <x:c r="B18" s="4" t="str">
+      <x:c r="B20" s="4" t="str">
         <x:v>★ Magdalena Peksa; Mehdi Keyvan-Ekbatani; Klaus Bogenberger</x:v>
       </x:c>
-      <x:c r="C18" s="4" t="str">
+      <x:c r="C20" s="4" t="str">
         <x:v>2025 IEEE 28th International Conference on Intelligent Transportation Systems (ITSC), pp. 2995-3000</x:v>
       </x:c>
-      <x:c r="D18" s="4" t="n">
+      <x:c r="D20" s="4" t="n">
         <x:v>2025</x:v>
       </x:c>
-      <x:c r="E18" s="4" t="str">
+      <x:c r="E20" s="4" t="str">
         <x:v>10.1109/ITSC60802.2025.11423788</x:v>
       </x:c>
-      <x:c r="F18" s="4" t="str">
+      <x:c r="F20" s="4" t="str">
         <x:v>https://portal.fis.tum.de/en/publications/airspace-partitioning-for-urban-air-mobility-a-macroscopic-approa/</x:v>
       </x:c>
-      <x:c r="G18" s="4" t="str">
+      <x:c r="G20" s="4" t="str">
         <x:v>https://doi.org/10.1109/ITSC60802.2025.11423788</x:v>
       </x:c>
-      <x:c r="H18" s="4" t="str">
+      <x:c r="H20" s="4" t="str">
         <x:v>supplement/Airspace_Partitioning_for_Urban_Air_Mobility_A_Macroscopic_Approach_with_a_Realistic_Network.pdf</x:v>
       </x:c>
-      <x:c r="I18" s="4" t="str">
+      <x:c r="I20" s="4" t="str">
         <x:v>extracted/supplement_B07.txt</x:v>
       </x:c>
-      <x:c r="J18" s="4" t="str">
+      <x:c r="J20" s="4" t="str">
         <x:v>publisher</x:v>
       </x:c>
-      <x:c r="K18" s="4" t="str">
+      <x:c r="K20" s="4" t="str">
         <x:v>纽约既有FAA直升机航路构建17 vertiport网络，按2023出租车/TNC出行时间节省估计UAM需求。工作日08:00–11:00出发，约11:30排空，4个随机场景；同类可悬停EC-135、500 m固定高度、100 km/h巡航、Dijkstra最短路。战术探测为线性前视、分散式成对减速解脱，h(v)=200 m+20 s×v；原点设最小出发间隔和安全延后。只模拟航路巡航，需求估计中的起降固定时间并非终端仿真（PDF pp.3–5）。</x:v>
       </x:c>
-      <x:c r="L18" s="4" t="str">
+      <x:c r="L20" s="4" t="str">
         <x:v>PDF p.5：10:15密度快照、4 min测量窗；DBSCAN MinPts=3、epsilon约2.5 km、theta=0.2，先K=3且每区≤3单元，再K=2且每区≤6单元，均为离线分区。
 PDF pp.5–6 Fig7：每5 s存轨迹、4 min聚合；中心Region2临界密度约0.7–0.9架/km、容量约60架/h；是给定航路/分离/需求下的长度加权区域NMFD。
 PDF pp.4–6：4个同设置随机场景，外围平均密度≤0.5架/km；未报告相对无分区的统一散布改善百分比或控制收益，不能据图虚构降幅。</x:v>
       </x:c>
-      <x:c r="M18" s="4" t="str">
+      <x:c r="M20" s="4" t="str">
         <x:v>p1=printed2995:title,DOI10.1109/ITSC60802.2025.11423788;abstract;static/single-layer scope
 p2=2996:DBSCAN/SRG Eq1,GA Eq2,Algorithm1/Fig1,graph/region constraints
 p3=2997:en-route-only,Eq3 NMFD,h(v),Fig2,Eq4 departure law,17vertiports
@@ -2727,248 +2908,248 @@
 p5=2999:snapshot/partition parameters,K3-&gt;K2,Figs4–6,critical density/capacity,conclusion
 p6=3000:Fig7NMFDs,acknowledgment/references</x:v>
       </x:c>
-      <x:c r="N18" s="11" t="str">
-        <x:v>FULL_TEXT</x:v>
-      </x:c>
-      <x:c r="O18" s="4" t="str">
+      <x:c r="N20" s="11" t="str">
+        <x:v>FULL_TEXT</x:v>
+      </x:c>
+      <x:c r="O20" s="4" t="str">
         <x:v>PUBLISHED</x:v>
       </x:c>
-      <x:c r="P18" s="4" t="str">
+      <x:c r="P20" s="4" t="str">
         <x:v>VERIFIED_PRIMARY</x:v>
       </x:c>
-      <x:c r="Q18" s="4" t="str">
+      <x:c r="Q20" s="4" t="str">
         <x:v>历史访问尝试：TUM official page：标题、作者、2025、会议、页码和 DOI 核验通过。
 IEEE DOI 页面可定位出版记录，但未找到无需组织访问的 PDF。
 2026-10-22：用户提供正式PDF，直接核对标题/DOI并阅读全文（6页）；本次本地文件为 research/low_altitude_phd_20261013/supplement/Airspace_Partitioning_for_Urban_Air_Mobility_A_Macroscopic_Approach_with_a_Realistic_Network.pdf。此前访问失败记录仅为历史，不代表当前缺全文。
 备注：2026-10-22用户提供正式6页PDF，已逐页视觉阅读全文，reading_status统一FULL_TEXT。PDF正文无法常规提取；TXT仅含页眉/页脚及明确标记的人工逐页阅读笔记，非逐字全文。</x:v>
       </x:c>
     </x:row>
-    <x:row r="19" ht="192" customHeight="1">
-      <x:c r="A19" s="4" t="str">
+    <x:row r="21" ht="192" customHeight="1">
+      <x:c r="A21" s="4" t="str">
         <x:v>B08</x:v>
       </x:c>
-      <x:c r="B19" s="4" t="str">
+      <x:c r="B21" s="4" t="str">
         <x:v>★ 刘子聪 / LIU Zicong; 包丹文 / BAO Danwen; 仇逸芙 / QIU Yifu</x:v>
       </x:c>
-      <x:c r="C19" s="4" t="str">
+      <x:c r="C21" s="4" t="str">
         <x:v>交通运输工程与信息学报 / Journal of Transportation Engineering and Information, 24(4), 132-144</x:v>
       </x:c>
-      <x:c r="D19" s="4" t="n">
+      <x:c r="D21" s="4" t="n">
         <x:v>2026</x:v>
       </x:c>
-      <x:c r="E19" s="4" t="str">
+      <x:c r="E21" s="4" t="str">
         <x:v>10.19961/j.cnki.1672-4747.2025.12.002</x:v>
       </x:c>
-      <x:c r="F19" s="4" t="str">
+      <x:c r="F21" s="4" t="str">
         <x:v>https://jtgc.cbpt.cnki.net/portal/journal/portal/client/paper/a362e609dbc5a11b3acd1222f51edfc6</x:v>
       </x:c>
-      <x:c r="G19" s="4" t="str">
+      <x:c r="G21" s="4" t="str">
         <x:v>https://jtgc.cbpt.cnki.net/portal/journal/portal/client/updateDownLoadNumber/3267de1ba9b5f8303a1e9501e08277bf/1</x:v>
       </x:c>
-      <x:c r="H19" s="4" t="str">
+      <x:c r="H21" s="4" t="str">
         <x:v>originals/B08.pdf</x:v>
       </x:c>
-      <x:c r="I19" s="4" t="str">
+      <x:c r="I21" s="4" t="str">
         <x:v>extracted/B08.txt</x:v>
       </x:c>
-      <x:c r="J19" s="4" t="str">
+      <x:c r="J21" s="4" t="str">
         <x:v>publisher</x:v>
       </x:c>
-      <x:c r="K19" s="4" t="str">
+      <x:c r="K21" s="4" t="str">
         <x:v>二维单层固定中心线航道、单方向纵向运行，不考虑交叉、并线和换层；横向宽度 40 m，典型高度 60-300 m。有人机用 Cessna 172、无人机用翼龙-2 作为性能尺度，Python 3.11 的 MM-ATM 平台仿真 600 s、步长 0.1 s，飞行器数量 0-200 架，每个密度 3 次重复，约 200 次仿真。</x:v>
       </x:c>
-      <x:c r="L19" s="4" t="str">
+      <x:c r="L21" s="4" t="str">
         <x:v>初始间距为静态阈值的 1.0-1.3 倍、无人机巡航速度约为有人机 110%、响应时延小于 1.5 s 时，在 10-13 架/km 密度区间取得容量与稳定性较优平衡（PDF pp.1-2、10-12，正文 pp.132-133、140-143）。
 无人机速度敏感性设置 33.3-72.2 m/s（120-260 km/h），有人机固定 55.6 m/s；作者建议无人机约 55.6-66.7 m/s 时兼顾容量和稳定性（PDF p.10，正文 p.140）。
 有人机速度设置 52.8-100.0 m/s；作者报告 66.7-72.2 m/s 区间相对兼顾容量和稳定性，高速度会出现流量回落与曲线拉伸（PDF pp.10-11，正文 pp.140-141）。
 仿真覆盖约 10^4 量级稳态样本；高密度响应时间实验显示快速响应可抑制扰动，慢响应会因延迟补偿导致容量受限（PDF pp.8-12，正文 pp.139-143）。</x:v>
       </x:c>
-      <x:c r="M19" s="4" t="str">
+      <x:c r="M21" s="4" t="str">
         <x:v>PDF p.1（中英文摘要、书目信息）
 PDF pp.2-3（研究不足、框架和贡献）
 PDF pp.4-8（静态安全间隔、刺激-响应控制和马尔科夫宏观模型）
 PDF pp.8-12（仿真设置、MFD、间距/速度/响应敏感性）
 PDF pp.12-13（研究结论、未来方向和作者限制）</x:v>
       </x:c>
-      <x:c r="N19" s="11" t="str">
-        <x:v>FULL_TEXT</x:v>
-      </x:c>
-      <x:c r="O19" s="4" t="str">
+      <x:c r="N21" s="11" t="str">
+        <x:v>FULL_TEXT</x:v>
+      </x:c>
+      <x:c r="O21" s="4" t="str">
         <x:v>PUBLISHED</x:v>
       </x:c>
-      <x:c r="P19" s="4" t="str">
+      <x:c r="P21" s="4" t="str">
         <x:v>VERIFIED_PRIMARY</x:v>
       </x:c>
-      <x:c r="Q19" s="4" t="str">
+      <x:c r="Q21" s="4" t="str">
         <x:v>历史访问尝试：期刊官方文章页：标题、作者、2026 24(4)、页码 132-144 和 DOI 核验通过。
 期刊官方目录公开 PDF 下载端点 HTTP 200，文件头 %PDF，pypdf 解析 13 页。
 备注：正式中文期刊全文；官方文章页与 PDF 首页标题、作者、DOI 一致。PDF 首页标示 Vol.24 No.4, Aug.2026，网络首发日期为 2026-01-23。核心方法是结构化静态安全间隔与刺激-响应速度控制，再经一阶马尔科夫链映射到三参数基本图；核心结论是混合运行临界密度右移并出现高密度低速稳定平台。作者限制见 PDF p.12（正文 p.143）：二维单层、无三维分层/交汇/并线/换层；一阶马尔科夫链的长程相关性不足；稳态遍历/收敛和矩阵规模问题；参数主要覆盖有人机与中大型固定翼无人机。</x:v>
       </x:c>
     </x:row>
-    <x:row r="20" ht="178" customHeight="1">
-      <x:c r="A20" s="4" t="str">
+    <x:row r="22" ht="178" customHeight="1">
+      <x:c r="A22" s="4" t="str">
         <x:v>B09</x:v>
       </x:c>
-      <x:c r="B20" s="4" t="str">
+      <x:c r="B22" s="4" t="str">
         <x:v>★ Alexey A. Munishkin; Priyank Pradeep; Kenny Chour; Krishna M. Kalyanam</x:v>
       </x:c>
-      <x:c r="C20" s="4" t="str">
+      <x:c r="C22" s="4" t="str">
         <x:v>2023 IEEE/AIAA 42nd Digital Avionics Systems Conference (DASC), Barcelona</x:v>
       </x:c>
-      <x:c r="D20" s="4" t="n">
+      <x:c r="D22" s="4" t="n">
         <x:v>2023</x:v>
       </x:c>
-      <x:c r="E20" s="4" t="str">
+      <x:c r="E22" s="4" t="str">
         <x:v>10.1109/DASC58513.2023.10311198</x:v>
       </x:c>
-      <x:c r="F20" s="4" t="str">
+      <x:c r="F22" s="4" t="str">
         <x:v>https://ntrs.nasa.gov/citations/20230014065</x:v>
       </x:c>
-      <x:c r="G20" s="4" t="str">
+      <x:c r="G22" s="4" t="str">
         <x:v>https://ntrs.nasa.gov/api/citations/20230009759/downloads/20230009759_AlexeyMunishkin_DASC2023_v3.pdf</x:v>
       </x:c>
-      <x:c r="H20" s="4" t="str">
+      <x:c r="H22" s="4" t="str">
         <x:v>originals/B09.pdf</x:v>
       </x:c>
-      <x:c r="I20" s="4" t="str">
+      <x:c r="I22" s="4" t="str">
         <x:v>extracted/B09.txt</x:v>
       </x:c>
-      <x:c r="J20" s="4" t="str">
+      <x:c r="J22" s="4" t="str">
         <x:v>accepted</x:v>
       </x:c>
-      <x:c r="K20" s="4" t="str">
+      <x:c r="K22" s="4" t="str">
         <x:v>小型 UAS package delivery 的 depot-to-customer 网络，含固定空间 operational-volume blocks、交叉 waypoint、恒定巡航地速和单向巡航阶段；仿真示例含 2 个 depot、4 个 customer、3 个 crossing waypoint，2D 平面网络用于巡航分析；每个 depot 一个 vertipad，假设一次只能起飞一架。</x:v>
       </x:c>
-      <x:c r="L20" s="4" t="str">
+      <x:c r="L22" s="4" t="str">
         <x:v>仿真将 OV block 长度 L 从 100 m 到 1000 m 以 100 m 递增，固定宽度 W=20 m；每组仿真 10,000 s，depot 订单为平均 100 orders/h 的 Poisson 到达（PDF pp.7-8）。
 随着 L 增大，三种队列策略的 ground delay 和等待队列数上升，能够发射的无人机/订单比例下降；作者报告吞吐在超过 max-flow 密度后快速下降（PDF pp.1、8-9）。
 作者在均匀间隔段落说明交叉点最小时间间隔 Δt 会使每条边至少保持 2×Δt 间隔，并明确将所计算的均匀流解表述为真实最优解的 upper bound，因为流被过度约束；全文检索未见 lower bound 表述（PDF p.3）。</x:v>
       </x:c>
-      <x:c r="M20" s="4" t="str">
+      <x:c r="M22" s="4" t="str">
         <x:v>PDF p.1（摘要和研究假设）
 PDF pp.2-5（网络、最大流、交叉时间约束）
 PDF pp.5-6（队列模型和三种策略）
 PDF pp.7-9（L/W 参数、100 orders/h、延误/吞吐结果和未来工作）</x:v>
       </x:c>
-      <x:c r="N20" s="11" t="str">
-        <x:v>FULL_TEXT</x:v>
-      </x:c>
-      <x:c r="O20" s="4" t="str">
+      <x:c r="N22" s="11" t="str">
+        <x:v>FULL_TEXT</x:v>
+      </x:c>
+      <x:c r="O22" s="4" t="str">
         <x:v>PUBLISHED</x:v>
       </x:c>
-      <x:c r="P20" s="4" t="str">
+      <x:c r="P22" s="4" t="str">
         <x:v>VERIFIED_PRIMARY</x:v>
       </x:c>
-      <x:c r="Q20" s="4" t="str">
+      <x:c r="Q22" s="4" t="str">
         <x:v>历史访问尝试：NASA NTRS citation 20230014065：作者、会议、日期和公开使用权限核验通过。
 NASA NTRS PDF HTTP 200，文件头 %PDF，pypdf 解析 9 页。
 Crossref 公共元数据确认 DOI 10.1109/DASC58513.2023.10311198。
 备注：低空 UAV 网络流/战略去冲突条目；重点是宏观流约束与节点队列耦合，不以起降场调度为主。原文 p.3 的上下文为：均匀流至少保持 2×Δt 边间隔，作者随后写明计算解是 true optimal solution 的 upper bound，因为 over-constrain the flow；未见 lower bound 术语。</x:v>
       </x:c>
     </x:row>
-    <x:row r="21" ht="192" customHeight="1">
-      <x:c r="A21" s="4" t="str">
+    <x:row r="23" ht="192" customHeight="1">
+      <x:c r="A23" s="4" t="str">
         <x:v>B10</x:v>
       </x:c>
-      <x:c r="B21" s="4" t="str">
+      <x:c r="B23" s="4" t="str">
         <x:v>★ Kenny Chour; Pouria Razzaghi; Dhriti Verma; Min Xue; Alexey A. Munishkin; Krishna M. Kalyanam</x:v>
       </x:c>
-      <x:c r="C21" s="4" t="str">
+      <x:c r="C23" s="4" t="str">
         <x:v>AIAA AVIATION FORUM AND ASCEND 2024 / AIAA AVIATION Forum and Exposition</x:v>
       </x:c>
-      <x:c r="D21" s="4" t="n">
+      <x:c r="D23" s="4" t="n">
         <x:v>2024</x:v>
       </x:c>
-      <x:c r="E21" s="4" t="str">
+      <x:c r="E23" s="4" t="str">
         <x:v>10.2514/6.2024-4575</x:v>
       </x:c>
-      <x:c r="F21" s="4" t="str">
+      <x:c r="F23" s="4" t="str">
         <x:v>https://ntrs.nasa.gov/citations/20240007458</x:v>
       </x:c>
-      <x:c r="G21" s="4" t="str">
+      <x:c r="G23" s="4" t="str">
         <x:v>https://ntrs.nasa.gov/api/citations/20240007458/downloads/AIAA_2024_Conference_MFD_final.pdf?attachment=true</x:v>
       </x:c>
-      <x:c r="H21" s="4" t="str">
+      <x:c r="H23" s="4" t="str">
         <x:v>originals/B10.pdf</x:v>
       </x:c>
-      <x:c r="I21" s="4" t="str">
+      <x:c r="I23" s="4" t="str">
         <x:v>extracted/B10.txt</x:v>
       </x:c>
-      <x:c r="J21" s="4" t="str">
+      <x:c r="J23" s="4" t="str">
         <x:v>publisher</x:v>
       </x:c>
-      <x:c r="K21" s="4" t="str">
+      <x:c r="K23" s="4" t="str">
         <x:v>4 km² lattice multi-lane sky corridor，lane spacing 200 m、纵向邻近节点间距 2 km；source vertiports 0/5/10，destination 4/9/14；每个 source 的小时需求 50、150、400 veh/h 分段升降，最大 400 veh/h。仿真步长 0.05 s，1 Hz 采样，单一 Amazon Drone 类型，不计风，不施加到达率限制。</x:v>
       </x:c>
-      <x:c r="L21" s="4" t="str">
+      <x:c r="L23" s="4" t="str">
         <x:v>MFD 在 occupancy 0-60 vehicles 时 flow 近似线性增至 600 veh/h，之后散布增大并在约 600 veh/h 饱和；据此选择 60 vehicles setpoint（PDF pp.9-10）。
 无控制时总 departure 在第 10 h 超过 5000 vehicles、峰值 departure rate 超过 800 veh/h；控制后总 departure 略超 2500、departure rate 稳定约 275 veh/h（PDF pp.10-11）。
 无控制时 source queues 峰值约 450/300/100 vehicles；控制后约 1400/1000/400 vehicles（PDF p.11）。
 无控制时 total occupancy 在第 6 h 短暂约 140、holding 最多约 60；控制后 total 近似恒定，holding 平均约 8，holding 峰值约减少 80%，arrival throughput 约减少 20%（PDF pp.12-13）。</x:v>
       </x:c>
-      <x:c r="M21" s="4" t="str">
+      <x:c r="M23" s="4" t="str">
         <x:v>PDF pp.1-3（摘要、研究动机和微观 BlueSky/控制框架）
 PDF pp.4-7（MFD 定义、occupancy setpoint 和 PI controller）
 PDF pp.8-10（假设、4 km² multi-lane 场景、需求表和 MFD）
 PDF pp.10-13（departure/queue/arrival/occupancy 结果与 Future work）</x:v>
       </x:c>
-      <x:c r="N21" s="11" t="str">
-        <x:v>FULL_TEXT</x:v>
-      </x:c>
-      <x:c r="O21" s="4" t="str">
+      <x:c r="N23" s="11" t="str">
+        <x:v>FULL_TEXT</x:v>
+      </x:c>
+      <x:c r="O23" s="4" t="str">
         <x:v>PUBLISHED</x:v>
       </x:c>
-      <x:c r="P21" s="4" t="str">
+      <x:c r="P23" s="4" t="str">
         <x:v>VERIFIED_PRIMARY</x:v>
       </x:c>
-      <x:c r="Q21" s="4" t="str">
+      <x:c r="Q23" s="4" t="str">
         <x:v>历史访问尝试：NASA NTRS citation 20240007458：作者、会议、2024 和公开会议论文状态核验通过。
 NASA NTRS PDF HTTP 200，文件头 %PDF，pypdf 解析 15 页。
 Crossref 公共元数据确认 DOI 10.2514/6.2024-4575。
 备注：全文已读；论文把 MFD 用于 departure metering，未把 RL 直接用于底层飞行控制。</x:v>
       </x:c>
     </x:row>
-    <x:row r="22" ht="234" customHeight="1">
-      <x:c r="A22" s="4" t="str">
+    <x:row r="24" ht="234" customHeight="1">
+      <x:c r="A24" s="4" t="str">
         <x:v>B11</x:v>
       </x:c>
-      <x:c r="B22" s="4" t="str">
+      <x:c r="B24" s="4" t="str">
         <x:v>★ Jack Haddad; Boris Mirkin; Kfir Assor</x:v>
       </x:c>
-      <x:c r="C22" s="4" t="str">
+      <x:c r="C24" s="4" t="str">
         <x:v>Transportation Research Part C 133 (2021) 103380</x:v>
       </x:c>
-      <x:c r="D22" s="4" t="n">
+      <x:c r="D24" s="4" t="n">
         <x:v>2021</x:v>
       </x:c>
-      <x:c r="E22" s="4" t="str">
+      <x:c r="E24" s="4" t="str">
         <x:v>10.1016/j.trc.2021.103380</x:v>
       </x:c>
-      <x:c r="F22" s="4" t="str">
+      <x:c r="F24" s="4" t="str">
         <x:v>https://www.sciencedirect.com/science/article/pii/S0968090X21003806</x:v>
       </x:c>
-      <x:c r="G22" s="4" t="str">
+      <x:c r="G24" s="4" t="str">
         <x:v>https://www.sciencedirect.com/science/article/pii/S0968090X21003806</x:v>
       </x:c>
-      <x:c r="H22" s="4" t="str">
+      <x:c r="H24" s="4" t="str">
         <x:v>supplement/1-s2.0-S0968090X21003806-main.pdf</x:v>
       </x:c>
-      <x:c r="I22" s="4" t="str">
+      <x:c r="I24" s="4" t="str">
         <x:v>extracted/supplement_B11.txt</x:v>
       </x:c>
-      <x:c r="J22" s="4" t="str">
+      <x:c r="J24" s="4" t="str">
         <x:v>publisher</x:v>
       </x:c>
-      <x:c r="K22" s="4" t="str">
+      <x:c r="K24" s="4" t="str">
         <x:v>MFD识别为100 m边长正方形，起终点在不同边；well-clear 15 m、速度上限20 m/s、加速度5 m/s²、前视30 s，不安全起飞者在区外悬停后重试。各恒定流入运行30 min，最高65架/min，每30 s估计后整次平均。控制测试另设两层共3聚合区，MFD比例G2=0.8G1、G3=1.2G1，按0.85倍临界累积局部线性化并归一化/缩放时间；比较两组事件阈值，同控制器不重调（PDF pp.6、12–15）。</x:v>
       </x:c>
-      <x:c r="L22" s="4" t="str">
+      <x:c r="L24" s="4" t="str">
         <x:v>PDF pp.12–13 §5：三区域测试选ncr1=80架、指数a1=0.73，G2=0.8G1、G3=1.2G1，线性化点0.85ncr；均为选定聚合仿真参数，不是三块真实空域容量。
 PDF p.6：100 m平方、15 m well-clear、20 m/s速度下，以≤65架/min恒定需求各运行30 min；30 s聚合后整次平均为一MFD点，非动态加载滞回试验。
 PDF p.13：归一化/时间缩放后输入时延h12/h13/h21/h23/h31/h32=3/0.1/3/0.2/1/0.7；不能不加换算直接当实际秒级执行周期。
 PDF p.12 Theorem1及pp.16–18 Appendix：A1–A4下误差渐近为0、信号有界，事件间隔有正下界；这是理论性质，未给效率改善百分比。</x:v>
       </x:c>
-      <x:c r="M22" s="4" t="str">
+      <x:c r="M24" s="4" t="str">
         <x:v>p.1 metadata
 pp.5-6 microscopic MFD construction and Fig.3
 pp.6-8 fixed multilayer/region/gateway design and nonlinear conservation dynamics
@@ -2977,16 +3158,16 @@
 p.16 conclusions/future work
 pp.16-18 proof and non-Zeno property</x:v>
       </x:c>
-      <x:c r="N22" s="11" t="str">
-        <x:v>FULL_TEXT</x:v>
-      </x:c>
-      <x:c r="O22" s="4" t="str">
+      <x:c r="N24" s="11" t="str">
+        <x:v>FULL_TEXT</x:v>
+      </x:c>
+      <x:c r="O24" s="4" t="str">
         <x:v>PUBLISHED</x:v>
       </x:c>
-      <x:c r="P22" s="4" t="str">
+      <x:c r="P24" s="4" t="str">
         <x:v>VERIFIED_PRIMARY</x:v>
       </x:c>
-      <x:c r="Q22" s="4" t="str">
+      <x:c r="Q24" s="4" t="str">
         <x:v>历史访问尝试：ScienceDirect publisher record：标题、作者、卷期、文章号和 DOI 核验通过；PDF 端点返回 HTTP 403，未保存文件。
 Technion institutional publication page：正式元数据和摘要可访问，未提供公开 PDF。
 TRID、ResearchGate 和 LAAT-Flow 作者页面：可访问元数据/摘要或请求全文页面，未找到无需组织访问的合法全文。
@@ -2995,47 +3176,47 @@
 备注：2026-10-22用户提供20页正式期刊PDF，已全文阅读。微观MFD识别和聚合闭环测试分开；平稳加载限制已被后续B05的部分实验补足。</x:v>
       </x:c>
     </x:row>
-    <x:row r="23" ht="262" customHeight="1">
-      <x:c r="A23" s="4" t="str">
+    <x:row r="25" ht="262" customHeight="1">
+      <x:c r="A25" s="4" t="str">
         <x:v>B12</x:v>
       </x:c>
-      <x:c r="B23" s="4" t="str">
+      <x:c r="B25" s="4" t="str">
         <x:v>★ Yazan Safadi; Nikolas Geroliminis; Jack Haddad</x:v>
       </x:c>
-      <x:c r="C23" s="4" t="str">
+      <x:c r="C25" s="4" t="str">
         <x:v>Transportation Research Part B 189 (2024) 103020</x:v>
       </x:c>
-      <x:c r="D23" s="4" t="n">
+      <x:c r="D25" s="4" t="n">
         <x:v>2024</x:v>
       </x:c>
-      <x:c r="E23" s="4" t="str">
+      <x:c r="E25" s="4" t="str">
         <x:v>10.1016/j.trb.2024.103020</x:v>
       </x:c>
-      <x:c r="F23" s="4" t="str">
+      <x:c r="F25" s="4" t="str">
         <x:v>https://www.sciencedirect.com/science/article/pii/S0191261524001449</x:v>
       </x:c>
-      <x:c r="G23" s="4" t="str">
+      <x:c r="G25" s="4" t="str">
         <x:v>https://www.sciencedirect.com/science/article/pii/S0191261524001449</x:v>
       </x:c>
-      <x:c r="H23" s="4" t="str">
+      <x:c r="H25" s="4" t="str">
         <x:v>supplement/1-s2.0-S0191261524001449-main.pdf</x:v>
       </x:c>
-      <x:c r="I23" s="4" t="str">
+      <x:c r="I25" s="4" t="str">
         <x:v>extracted/supplement_B12.txt</x:v>
       </x:c>
-      <x:c r="J23" s="4" t="str">
+      <x:c r="J25" s="4" t="str">
         <x:v>publisher</x:v>
       </x:c>
-      <x:c r="K23" s="4" t="str">
+      <x:c r="K25" s="4" t="str">
         <x:v>固定1.5×1.5 km、120 m高无预设航路网络，中心与外围两区，地面均匀随机OD、VTOL和区域上方buffer。相同飞机vmax20 m/s、amax5 m/s²、安全/避让/探测半径15/22.5/45.5 m；仿真1 h、0.5 s步长，聚合/控制/MPC离散均60 s，预测300 s。NC/DC/BC/DBC同用梯形峰值2.5架/s，对照识别容量2.3架/s；各控制器分别标定权重（PDF pp.11–13 Table1）。</x:v>
       </x:c>
-      <x:c r="L23" s="4" t="str">
+      <x:c r="L25" s="4" t="str">
         <x:v>PDF pp.13、15 Figs7–8：同峰值2.5架/s、1 h需求与微观网络下，DC/BC/DBC的TTS相对NC分别降低32%/6.7%/40%；不是所有指标同比下降。
 PDF p.15 Fig8：以NC的TTS为共同分母，DC/DBC地面延误为2.5%/4.1%，DBC边界延误0.4%，换来额外8个百分点TTS下降；不是各策略内部组成比。
 PDF p.12：区域临界累积33/135架，累积与相应起飞/边界队列上界99/405架；网络识别容量2.3架/s，小于比较需求2.5架/s。
 PDF pp.11–12 Table1：0.5 s逐机仿真、60 s聚合和控制、5步预测；权重分别标定，不是同一固定目标权重下的纯动作维度对照。</x:v>
       </x:c>
-      <x:c r="M23" s="4" t="str">
+      <x:c r="M25" s="4" t="str">
         <x:v>p.1 metadata
 pp.4-5 Sections 2.1-2.3/Fig.2, plant and MFD feedback
 pp.6-8 Section 2.4/Equations 4-23, queue and optimization model
@@ -3045,16 +3226,16 @@
 pp.15-16 Section 4, limits and future work
 pp.17-19 Appendix B/Algorithm 4, simulation feedback structure</x:v>
       </x:c>
-      <x:c r="N23" s="11" t="str">
-        <x:v>FULL_TEXT</x:v>
-      </x:c>
-      <x:c r="O23" s="4" t="str">
+      <x:c r="N25" s="11" t="str">
+        <x:v>FULL_TEXT</x:v>
+      </x:c>
+      <x:c r="O25" s="4" t="str">
         <x:v>PUBLISHED</x:v>
       </x:c>
-      <x:c r="P23" s="4" t="str">
+      <x:c r="P25" s="4" t="str">
         <x:v>VERIFIED_PRIMARY</x:v>
       </x:c>
-      <x:c r="Q23" s="4" t="str">
+      <x:c r="Q25" s="4" t="str">
         <x:v>历史访问尝试：ScienceDirect publisher record：标题、全作者、2024、Transportation Research Part B: Methodological 卷189、文章号103020 和 DOI 核验通过；PDF 端点返回 HTTP 403，未保存文件。
 Technion institutional page：正式元数据、摘要和 DOI 可访问，未提供公开 PDF。
 EPFL Infoscience official record URL可定位该出版物，但页面返回 HTTP 405，未得到文件。
@@ -3064,44 +3245,44 @@
 备注：2026-10-22用户提供20页正式期刊PDF，已全文阅读。Fig3称3层、§3.2描述两功能层（飞行层含buffer），原文描述差异保留；并未把悬停动机当作已量化SOC可行性。</x:v>
       </x:c>
     </x:row>
-    <x:row r="24" ht="136" customHeight="1">
-      <x:c r="A24" s="4" t="str">
+    <x:row r="26" ht="136" customHeight="1">
+      <x:c r="A26" s="4" t="str">
         <x:v>C01</x:v>
       </x:c>
-      <x:c r="B24" s="4" t="str">
+      <x:c r="B26" s="4" t="str">
         <x:v>★ Flavia Causa; Armando Franzone; Giancarmine Fasano</x:v>
       </x:c>
-      <x:c r="C24" s="4" t="str">
+      <x:c r="C26" s="4" t="str">
         <x:v>Drones, 7(1), 11</x:v>
       </x:c>
-      <x:c r="D24" s="4" t="n">
+      <x:c r="D26" s="4" t="n">
         <x:v>2023</x:v>
       </x:c>
-      <x:c r="E24" s="4" t="str">
+      <x:c r="E26" s="4" t="str">
         <x:v>10.3390/drones7010011</x:v>
       </x:c>
-      <x:c r="F24" s="4" t="str">
+      <x:c r="F26" s="4" t="str">
         <x:v>https://www.mdpi.com/2504-446X/7/1/11</x:v>
       </x:c>
-      <x:c r="G24" s="4" t="str">
+      <x:c r="G26" s="4" t="str">
         <x:v>https://mdpi-res.com/d_attachment/drones/drones-07-00011/article_deploy/drones-07-00011-v2.pdf</x:v>
       </x:c>
-      <x:c r="H24" s="4" t="str">
+      <x:c r="H26" s="4" t="str">
         <x:v>originals/C01.pdf</x:v>
       </x:c>
-      <x:c r="I24" s="4" t="str">
+      <x:c r="I26" s="4" t="str">
         <x:v>extracted/C01.txt</x:v>
       </x:c>
-      <x:c r="J24" s="4" t="str">
+      <x:c r="J26" s="4" t="str">
         <x:v>publisher</x:v>
       </x:c>
-      <x:c r="K24" s="4" t="str">
+      <x:c r="K26" s="4" t="str">
         <x:v>两个用例均位于意大利Naples及周边。空中出租车从Capodichino机场飞往Naples商业中心或港口；医疗配送从大陆Monte di Procida药房飞往Procida岛医疗单元，直线约4 km，用以对比船运约16 min且冬季班次不足的情况。两类任务均使用真实地理/环境地图；医疗场景最高飞行高度150 m，统一风速5 m/s，未进行实飞。</x:v>
       </x:c>
-      <x:c r="L24" s="4" t="str">
+      <x:c r="L26" s="4" t="str">
         <x:v>医疗用例战略方案D1–D3的总目标代价约26,675–33,962，单方案计算时间53.0–60.3 s（表2）；战术解的总目标代价约26,686–30,160，计算时间1.7–5.2 s（表3），最大导航误差约1.19–1.25 m。论文结论称战略路径计算低于约60 s、战术层约5 s，适合约10 s级更新窗口；用例结果中规划路径均可飞行。</x:v>
       </x:c>
-      <x:c r="M24" s="4" t="str">
+      <x:c r="M26" s="4" t="str">
         <x:v>§2 Environment and Vehicle Based Constraints, pp.2–5
 §3 Path Planning Framework, pp.5–8
 §4 Use Cases, pp.8–11
@@ -3110,77 +3291,77 @@
 §6 Conclusions, pp.17–18
 Tables 1–5, pp.11–16</x:v>
       </x:c>
-      <x:c r="N24" s="11" t="str">
-        <x:v>FULL_TEXT</x:v>
-      </x:c>
-      <x:c r="O24" s="4" t="str">
+      <x:c r="N26" s="11" t="str">
+        <x:v>FULL_TEXT</x:v>
+      </x:c>
+      <x:c r="O26" s="4" t="str">
         <x:v>published</x:v>
       </x:c>
-      <x:c r="P24" s="4" t="str">
+      <x:c r="P26" s="4" t="str">
         <x:v>VERIFIED_PRIMARY</x:v>
       </x:c>
-      <x:c r="Q24" s="4" t="str">
+      <x:c r="Q26" s="4" t="str">
         <x:v>历史访问尝试：MDPI正式文章页面打开并核验标题、作者、期刊、DOI
 MDPI开放PDF下载成功
 本地PDF头为%PDF，pypdf解析18页成功
 备注：期刊卷期年份为2023；页面显示在线发表日期为2022-12-24。</x:v>
       </x:c>
     </x:row>
-    <x:row r="25" ht="220" customHeight="1">
-      <x:c r="A25" s="4" t="str">
+    <x:row r="27" ht="220" customHeight="1">
+      <x:c r="A27" s="4" t="str">
         <x:v>C02</x:v>
       </x:c>
-      <x:c r="B25" s="4" t="str">
+      <x:c r="B27" s="4" t="str">
         <x:v>★ Hualong Tang; Yu Zhang; Vahid Mohmoodian; Hadi Charkhgard</x:v>
       </x:c>
-      <x:c r="C25" s="4" t="str">
+      <x:c r="C27" s="4" t="str">
         <x:v>Transportation Research Part C: Emerging Technologies, 131, 103324</x:v>
       </x:c>
-      <x:c r="D25" s="4" t="n">
+      <x:c r="D27" s="4" t="n">
         <x:v>2021</x:v>
       </x:c>
-      <x:c r="E25" s="4" t="str">
+      <x:c r="E27" s="4" t="str">
         <x:v>10.1016/j.trc.2021.103324</x:v>
       </x:c>
-      <x:c r="F25" s="4" t="str">
+      <x:c r="F27" s="4" t="str">
         <x:v>https://doi.org/10.1016/j.trc.2021.103324</x:v>
       </x:c>
-      <x:c r="G25" s="4" t="str"/>
-      <x:c r="H25" s="4" t="str">
+      <x:c r="G27" s="4" t="str"/>
+      <x:c r="H27" s="4" t="str">
         <x:v>supplement/1-s2.0-S0968090X21003302-main.pdf</x:v>
       </x:c>
-      <x:c r="I25" s="4" t="str">
+      <x:c r="I27" s="4" t="str">
         <x:v>extracted/supplement_C02.txt</x:v>
       </x:c>
-      <x:c r="J25" s="4" t="str">
+      <x:c r="J27" s="4" t="str">
         <x:v>publisher</x:v>
       </x:c>
-      <x:c r="K25" s="4" t="str">
+      <x:c r="K27" s="4" t="str">
         <x:v>Tampa Bay 30个vertiport、7机场禁飞区及cuboid建筑包络，500–1400 ft共10层、层距100 ft；垂直起降后定层水平巡航，130 knots、垂直1000 fpm、最小分离0.3 NM。45 min内按5或3 min/takeoff需求生成270或450飞行，2/4/6运营方、四档NHHI；起飞时刻在2 min窗内均匀抽取。两模型分别用Gurobi与CPLEX，i7-4790/16 GB，未实施战术偏差回馈闭环（PDF pp.12–18 §4–5）。</x:v>
       </x:c>
-      <x:c r="L25" s="4" t="str">
+      <x:c r="L27" s="4" t="str">
         <x:v>PDF p.12 Table1/§4.1：30 vertiport、10层、0.3 NM分离，45 min内270/450飞行；安全结论限于给定时刻和速度模型。
 PDF pp.14–15 Fig11：求和模型两需求的系统成本2653/4380，乘积模型相对差不超过0.5%；原文该句不标成本物理单位，不换写成延误分钟或kWh。
 PDF p.14：3 min/takeoff、4运营方、NHHI=0.5时，乘积/求和模型平均飞行9.74/9.73 min；100 ft爬升仅6 s，结果依赖所测简单网络。
 PDF p.16 Tables2–3：5 min/takeoff、4运营方、NHHI=0.5，求和UBR=0.986/0.987/0.918/0.962，乘积=0.968/0.971/1.000/0.994；公平改善不等于各家收益增加。
 PDF p.16 Fig13：低密度图纵轴至1.6 s，高密度至1600 s；高密度低NHHI部分乘积求解约千秒。图读量级，不把全部实验称为实时。</x:v>
       </x:c>
-      <x:c r="M25" s="4" t="str">
+      <x:c r="M27" s="4" t="str">
         <x:v>PDF pp.1–2 title/DOI/Abstract/Introduction: 电池监测与充电属于tactical scheduling，区分本文planning与单机fuel-efficient trajectory。
 PDF pp.5–7 §2.5/§3.1/Fig1–4: layered near-free visibility graph route generation、预处理数据库及LAMS→LTMS。
 PDF pp.7–10 §3.2.1–3.2.2/Fig5–6/eq1–11: 三类冲突、固定出发时间、层决策、NSW/UBR与参考点。
 PDF pp.11–12 §3.2.3/§4/Table1: SOCP及Tampa参数；pp.13–16 §4.1–4.2/Figs8–13/Tables2–3及p.17 Tables4–5: 实验与比较；pp.17–18 §5: 未来闭环/不确定性/天气。</x:v>
       </x:c>
-      <x:c r="N25" s="11" t="str">
-        <x:v>FULL_TEXT</x:v>
-      </x:c>
-      <x:c r="O25" s="4" t="str">
+      <x:c r="N27" s="11" t="str">
+        <x:v>FULL_TEXT</x:v>
+      </x:c>
+      <x:c r="O27" s="4" t="str">
         <x:v>published</x:v>
       </x:c>
-      <x:c r="P25" s="4" t="str">
+      <x:c r="P27" s="4" t="str">
         <x:v>VERIFIED_PRIMARY</x:v>
       </x:c>
-      <x:c r="Q25" s="4" t="str">
+      <x:c r="Q27" s="4" t="str">
         <x:v>历史访问尝试：ScienceDirect/DOI页面打开，核验标题、作者、期刊、年份、DOI并读取摘要/预览
 直接publisher /pdfft请求返回Cloudflare访问页
 ResearchGate全文落地页可见但未获得可合法保存的直接PDF
@@ -3189,97 +3370,97 @@
 备注：2026-10-22用户提供19页正式期刊PDF，已阅读全文。作者名Mohmoodian按PDF/出版商拼写保留，部分索引写Mahmoodian；起飞时刻和速度是给定输入。</x:v>
       </x:c>
     </x:row>
-    <x:row r="26" ht="108" customHeight="1">
-      <x:c r="A26" s="4" t="str">
+    <x:row r="28" ht="108" customHeight="1">
+      <x:c r="A28" s="4" t="str">
         <x:v>C03</x:v>
       </x:c>
-      <x:c r="B26" s="4" t="str">
+      <x:c r="B28" s="4" t="str">
         <x:v>★ Kai Wang; Alexandre Jacquillat; Vikrant Vaze</x:v>
       </x:c>
-      <x:c r="C26" s="4" t="str">
+      <x:c r="C28" s="4" t="str">
         <x:v>Manufacturing &amp; Service Operations Management, 24(6), 3215–3235</x:v>
       </x:c>
-      <x:c r="D26" s="4" t="n">
+      <x:c r="D28" s="4" t="n">
         <x:v>2022</x:v>
       </x:c>
-      <x:c r="E26" s="4" t="str">
+      <x:c r="E28" s="4" t="str">
         <x:v>10.1287/msom.2022.1148</x:v>
       </x:c>
-      <x:c r="F26" s="4" t="str">
+      <x:c r="F28" s="4" t="str">
         <x:v>https://pubsonline.informs.org/doi/10.1287/msom.2022.1148</x:v>
       </x:c>
-      <x:c r="G26" s="4" t="str"/>
-      <x:c r="H26" s="4" t="str"/>
-      <x:c r="I26" s="4" t="str"/>
-      <x:c r="J26" s="4" t="str">
+      <x:c r="G28" s="4" t="str"/>
+      <x:c r="H28" s="4" t="str"/>
+      <x:c r="I28" s="4" t="str"/>
+      <x:c r="J28" s="4" t="str">
         <x:v>publisher</x:v>
       </x:c>
-      <x:c r="K26" s="4" t="str">
+      <x:c r="K28" s="4" t="str">
         <x:v>城市空中交通网络的vertiport规划与乘客需求分配；出版商摘要/页面描述不同候选网络、容量和需求情形，完整网络规模及实验设置未获全文。</x:v>
       </x:c>
-      <x:c r="L26" s="4" t="str">
+      <x:c r="L28" s="4" t="str">
         <x:v>出版商摘要明确报告可达到1%的最优性间隙；未获得正文实验表格，其他规模和时间数值无法核验。</x:v>
       </x:c>
-      <x:c r="M26" s="4" t="str">
+      <x:c r="M28" s="4" t="str">
         <x:v>INFORMS publisher abstract
 Publisher results paragraph; full-text page/section unavailable</x:v>
       </x:c>
-      <x:c r="N26" s="13" t="str">
+      <x:c r="N28" s="13" t="str">
         <x:v>ABSTRACT_ONLY</x:v>
       </x:c>
-      <x:c r="O26" s="4" t="str">
+      <x:c r="O28" s="4" t="str">
         <x:v>published</x:v>
       </x:c>
-      <x:c r="P26" s="4" t="str">
+      <x:c r="P28" s="4" t="str">
         <x:v>VERIFIED_PRIMARY</x:v>
       </x:c>
-      <x:c r="Q26" s="4" t="str">
+      <x:c r="Q28" s="4" t="str">
         <x:v>历史访问尝试：INFORMS正式页面打开并核验作者、在线日期、期刊、DOI、摘要和结果段
 未获得开放PDF或作者稿
 未保存本地PDF
 备注：正式期刊论文；在线发表日期为2022-09-21。 用户已于2026-10-22决定不继续追索该篇全文；保持ABSTRACT_ONLY，未补写未经全文验证的结果或限制。</x:v>
       </x:c>
     </x:row>
-    <x:row r="27" ht="276" customHeight="1">
-      <x:c r="A27" s="4" t="str">
+    <x:row r="29" ht="276" customHeight="1">
+      <x:c r="A29" s="4" t="str">
         <x:v>C04</x:v>
       </x:c>
-      <x:c r="B27" s="4" t="str">
+      <x:c r="B29" s="4" t="str">
         <x:v>★ Mercedes Pelegrín; Claudia D’Ambrosio; Rémi Delmas; Youssef Hamadi</x:v>
       </x:c>
-      <x:c r="C27" s="4" t="str">
+      <x:c r="C29" s="4" t="str">
         <x:v>Optimization Methods and Software, 38(6), 1311–1343</x:v>
       </x:c>
-      <x:c r="D27" s="4" t="n">
+      <x:c r="D29" s="4" t="n">
         <x:v>2023</x:v>
       </x:c>
-      <x:c r="E27" s="4" t="str">
+      <x:c r="E29" s="4" t="str">
         <x:v>10.1080/10556788.2023.2241148</x:v>
       </x:c>
-      <x:c r="F27" s="4" t="str">
+      <x:c r="F29" s="4" t="str">
         <x:v>https://www.tandfonline.com/doi/abs/10.1080/10556788.2023.2241148</x:v>
       </x:c>
-      <x:c r="G27" s="4" t="str"/>
-      <x:c r="H27" s="4" t="str">
+      <x:c r="G29" s="4" t="str"/>
+      <x:c r="H29" s="4" t="str">
         <x:v>supplement/Urban air mobility  from complex tactical conflict resolution to network design and fairness insights.pdf</x:v>
       </x:c>
-      <x:c r="I27" s="4" t="str">
+      <x:c r="I29" s="4" t="str">
         <x:v>extracted/supplement_C04.txt</x:v>
       </x:c>
-      <x:c r="J27" s="4" t="str">
+      <x:c r="J29" s="4" t="str">
         <x:v>publisher</x:v>
       </x:c>
-      <x:c r="K27" s="4" t="str">
+      <x:c r="K29" s="4" t="str">
         <x:v>三类合成单高度网络：Grid 8 vertiport、Airport 5、Metroplex 9且两中心单廊连接；每类两套名义计划，五个10 min需求批次，总时域约50 min。测试随机漂移/地面延误、新priority、固定直线noncooperative intruder；巡航150 mph、最小分离0.5 NM，速度可±5%或−5%/+10%，节点调速、边内匀速，爬升速度固定。MILP在扰动/检测时重排剩余全部航班（PDF pp.17–21 Tables1–5）。</x:v>
       </x:c>
-      <x:c r="L27" s="4" t="str">
+      <x:c r="L29" s="4" t="str">
         <x:v>PDF pp.21–23 Tables2–3：随机扰动60例中59可行，平均/最大CPU0.27/1.65 s；priority 60例全部可行，0.32/1.81 s，55%有priority延误。
 PDF p.25 Table4：intruder 180例中52可行、128不可行；r=1/5/10 min各60例不可行55/45/28，故r=10组内为28/60=46.7%，不能用28/180说该组仅15%。
 PDF p.29 §6.3.4：local intruder仅3/180可行，global52/180；为同MILP受限版本对照，非所有局部算法的结果。
 PDF p.30 Table6：公平目标在random/priority/intruder逐实例百分比平均中改善35.06%/39.87%/45.29%，总arrival delay劣化478.76%/430.39%/397.72%；不能用均值之比替代这些百分比。
 PDF p.30 Table6：总arrival delay均值原→公平为9.74→37.62、35.93→65.39、35.43→77.50 min；约半数实例每架平均调速原≤2次、公平可至13次（p.31 Fig11）。</x:v>
       </x:c>
-      <x:c r="M27" s="4" t="str">
+      <x:c r="M29" s="4" t="str">
         <x:v>PDF pp.1–2：cover及title/DOI；pp.3–6 §1及主要结论。
 PDF pp.7–9 §3/Fig3：固定track、固定altitude、nominal schedule、三扰动与空/地可用动作。
 PDF pp.9–13 §4/Figs4–6/eq1–8：追随与三类非追随冲突、保守危险区、转弯角关系。
@@ -3287,16 +3468,16 @@
 PDF pp.17–21 §6.1–6.2/Figs7–8/Table1：拓扑、schedule、扰动生成、性能/安全参数与测试规模。
 PDF pp.21–26 §6.3.1–6.3.3/Tables2–5：各用例结果；pp.26–29 §6.3.4/Figs9–10：local对照；pp.29–31 §6.3.5/eq10/Table6/Fig11：公平目标和代价；pp.31–32 §7：结论、能耗与多层/不确定性未来工作。</x:v>
       </x:c>
-      <x:c r="N27" s="11" t="str">
-        <x:v>FULL_TEXT</x:v>
-      </x:c>
-      <x:c r="O27" s="4" t="str">
+      <x:c r="N29" s="11" t="str">
+        <x:v>FULL_TEXT</x:v>
+      </x:c>
+      <x:c r="O29" s="4" t="str">
         <x:v>published</x:v>
       </x:c>
-      <x:c r="P27" s="4" t="str">
+      <x:c r="P29" s="4" t="str">
         <x:v>VERIFIED_PRIMARY</x:v>
       </x:c>
-      <x:c r="Q27" s="4" t="str">
+      <x:c r="Q29" s="4" t="str">
         <x:v>历史访问尝试：Taylor &amp; Francis正式摘要页打开并核验作者、在线发表日期、卷页、DOI和摘要
 正式全文页返回403
 未获得作者稿或开放PDF
@@ -3305,60 +3486,60 @@
 备注：2026-10-22用户提供34页正式PDF，含封面；正文1311页对应PDF p.2。p.25 Table4的Grid CPU均值0.60 s却最大0.20 s为原文内部不一致，未据此选值。</x:v>
       </x:c>
     </x:row>
-    <x:row r="28" ht="122" customHeight="1">
-      <x:c r="A28" s="4" t="str">
+    <x:row r="30" ht="122" customHeight="1">
+      <x:c r="A30" s="4" t="str">
         <x:v>C05</x:v>
       </x:c>
-      <x:c r="B28" s="4" t="str">
+      <x:c r="B30" s="4" t="str">
         <x:v>★ Shulu Chen; Antony D. Evans; Marc Brittain; Peng Wei</x:v>
       </x:c>
-      <x:c r="C28" s="4" t="str">
+      <x:c r="C30" s="4" t="str">
         <x:v>IEEE Transactions on Intelligent Transportation Systems, 25(8), 10049–10061</x:v>
       </x:c>
-      <x:c r="D28" s="4" t="n">
+      <x:c r="D30" s="4" t="n">
         <x:v>2024</x:v>
       </x:c>
-      <x:c r="E28" s="4" t="str">
+      <x:c r="E30" s="4" t="str">
         <x:v>10.1109/TITS.2024.3351049</x:v>
       </x:c>
-      <x:c r="F28" s="4" t="str">
+      <x:c r="F30" s="4" t="str">
         <x:v>https://doi.org/10.1109/TITS.2024.3351049</x:v>
       </x:c>
-      <x:c r="G28" s="4" t="str">
+      <x:c r="G30" s="4" t="str">
         <x:v>https://arxiv.org/pdf/2305.10556</x:v>
       </x:c>
-      <x:c r="H28" s="4" t="str">
+      <x:c r="H30" s="4" t="str">
         <x:v>originals/C05.pdf</x:v>
       </x:c>
-      <x:c r="I28" s="4" t="str">
+      <x:c r="I30" s="4" t="str">
         <x:v>extracted/C05.txt</x:v>
       </x:c>
-      <x:c r="J28" s="4" t="str">
+      <x:c r="J30" s="4" t="str">
         <x:v>preprint</x:v>
       </x:c>
-      <x:c r="K28" s="4" t="str">
+      <x:c r="K30" s="4" t="str">
         <x:v>BlueSky中三条共享航路：N-7→N-1→N-2→N-3、N-9→N-1→N-2→N-3、M-2→N-2→M-4；资源为N-1/N-2。表I含30个飞行计划和100张调度表；MARL训练150,000回合（2×RTX3090，约4 h），观测半径1500 m，同高度运行，时间窗200 s。安全阈值：LoWC 500 m、NMAC 150 m、MAC 10 m，风险比β=0.005。</x:v>
       </x:c>
-      <x:c r="L28" s="4" t="str">
+      <x:c r="L30" s="4" t="str">
         <x:v>仅DCB时可行容量C=1/200 s；规则战术可到C=4；MARL可到C=7。表III估计MAC/100,000 h：C=4时无战术75.51、规则0.74、MARL0.85；C=7时无战术122.14、规则115.34、MARL0.66；MARL在C=8、10时分别3.70、23.49。表IV高/中/低需求下，DCB+MARL（C=7）的LoWC为45.6/62.8/49.6，估计MAC为0.66/0.65/0.51，空中延误30.8/32.9/22.2 s、地面延误158.4/74.4/19.9 s；DCB+规则（C=4）的LoWC为25.9/34.8/30.8，估计MAC为0.74/0.77/0.92。</x:v>
       </x:c>
-      <x:c r="M28" s="4" t="str">
+      <x:c r="M30" s="4" t="str">
         <x:v>§II Problem Formulation, pp.3–4
 §III Strategic Conflict Management, pp.4–6
 §V Numerical Experiments, pp.8–11
 §VI Conclusions, pp.11–12
 Table I, pp.3–4; Table III, p.9; Table IV, p.11</x:v>
       </x:c>
-      <x:c r="N28" s="11" t="str">
-        <x:v>FULL_TEXT</x:v>
-      </x:c>
-      <x:c r="O28" s="4" t="str">
+      <x:c r="N30" s="11" t="str">
+        <x:v>FULL_TEXT</x:v>
+      </x:c>
+      <x:c r="O30" s="4" t="str">
         <x:v>published</x:v>
       </x:c>
-      <x:c r="P28" s="4" t="str">
+      <x:c r="P30" s="4" t="str">
         <x:v>VERIFIED_PRIMARY_DOI</x:v>
       </x:c>
-      <x:c r="Q28" s="4" t="str">
+      <x:c r="Q30" s="4" t="str">
         <x:v>历史访问尝试：IEEE正式记录/DOI页面核验标题、作者、期刊、卷页、年份和DOI；出版商正文受限
 arXiv公开作者预印本下载成功
 本地PDF头为%PDF，pypdf解析13页并通读正文
@@ -3366,61 +3547,61 @@
 备注：正式发表年份为2024（在线2024-01-18，卷期2024-08）；本地全文是arXiv公开预印本，不是IEEE排版版。</x:v>
       </x:c>
     </x:row>
-    <x:row r="29" ht="234" customHeight="1">
-      <x:c r="A29" s="4" t="str">
+    <x:row r="31" ht="234" customHeight="1">
+      <x:c r="A31" s="4" t="str">
         <x:v>C06</x:v>
       </x:c>
-      <x:c r="B29" s="4" t="str">
+      <x:c r="B31" s="4" t="str">
         <x:v>★ Julián Alberto Espejo-Díaz; Edgar Alfonso-Lizarazo; Jairo R. Montoya-Torres</x:v>
       </x:c>
-      <x:c r="C29" s="4" t="str">
+      <x:c r="C31" s="4" t="str">
         <x:v>Applied Mathematical Modelling, 123, 871–890</x:v>
       </x:c>
-      <x:c r="D29" s="4" t="n">
+      <x:c r="D31" s="4" t="n">
         <x:v>2023</x:v>
       </x:c>
-      <x:c r="E29" s="4" t="str">
+      <x:c r="E31" s="4" t="str">
         <x:v>10.1016/j.apm.2023.07.009</x:v>
       </x:c>
-      <x:c r="F29" s="4" t="str">
+      <x:c r="F31" s="4" t="str">
         <x:v>https://www.sciencedirect.com/science/article/pii/S0307904X23003062</x:v>
       </x:c>
-      <x:c r="G29" s="4" t="str"/>
-      <x:c r="H29" s="4" t="str">
+      <x:c r="G31" s="4" t="str"/>
+      <x:c r="H31" s="4" t="str">
         <x:v>supplement/1-s2.0-S0307904X23003062-main.pdf</x:v>
       </x:c>
-      <x:c r="I29" s="4" t="str">
+      <x:c r="I31" s="4" t="str">
         <x:v>extracted/supplement_C06.txt</x:v>
       </x:c>
-      <x:c r="J29" s="4" t="str">
+      <x:c r="J31" s="4" t="str">
         <x:v>publisher</x:v>
       </x:c>
-      <x:c r="K29" s="4" t="str">
+      <x:c r="K31" s="4" t="str">
         <x:v>合成n=10/20/30/40/50架次、起飞比例30%/50%/70%，三布局均一条taxiway1和taxiway2，gate/pad各2、3或4。TLOF处理15–90 s、gate30–600 s、taxiway5–90 s均匀抽样，同pad分离90 s；目标Tj按各阶段处理和及n生成随机窗。CPLEX限1800 s，Python启发式100000迭代，i7-10870H/16 GB。流程不允许额外缓冲区，等待会继续占当前组件（PDF pp.5–6、11–13 Table2）。</x:v>
       </x:c>
-      <x:c r="L29" s="4" t="str">
+      <x:c r="L31" s="4" t="str">
         <x:v>PDF p.12：5起飞5到达、3 gate/3 pad示例，makespan模型1118 s；另一目标偏差模型总偏差908 s、makespan1203 s，两个目标不可视为同一个最优值。
 PDF p.13 §6.3：MILP仅n=10证最优，部分n=40及全部n=50在1800 s无可行解；n=10已知最优对照下H1平均makespan相对误差21.11%，不代表大例近优。
 PDF p.14 Table3：2 gate/2 pad、10架中7起飞时，MILP makespan1175 s/CPU8.15 s，H1 1429 s/62.28 s，误差21.62%；同例偏差MILP121 s、H2 140 s。
 PDF p.14 Table3：2 gate/2 pad、50架各半起飞到达，MILP两目标1800 s无可行解；H1 makespan8238 s/CPU283.61 s，H2偏差16552 s/283.52 s。
 PDF pp.17–18 Table6：small/medium/large的H1均值5126.40/3691.54/2048.78 s，对NEH7367.72/5581.68/3162.94 s；原Difference用H1作分母，不能说相对NEH降低43.72%/51.20%/54.38%。</x:v>
       </x:c>
-      <x:c r="M29" s="4" t="str">
+      <x:c r="M31" s="4" t="str">
         <x:v>PDF p.1 title/DOI/abstract；pp.4–6 §3/Fig1–2：四阶段反向流、blocking、pad separation及battery-based target动机。
 PDF pp.6–8 §4.1–4.3/eq1–29：机器指派/排序、阶段完成时间、完整arrival流程makespan和target软偏差；p.8已渲染核对eq18–29。
 PDF pp.8–11 §5/Fig3/Algorithm1：H1/H2种子、FAVC、插入改进与迭代。
 PDF pp.11–13 §6.1–6.3/Figs4–5/Table2：实例生成参数/设定、示例及下界限制；pp.14–16 Tables3–5：CPLEX/heuristic比较；pp.17–18 §6.3–§7/Tables6–7：NEH/EDD比较与未来方向，p.18表已渲染核对。</x:v>
       </x:c>
-      <x:c r="N29" s="11" t="str">
-        <x:v>FULL_TEXT</x:v>
-      </x:c>
-      <x:c r="O29" s="4" t="str">
+      <x:c r="N31" s="11" t="str">
+        <x:v>FULL_TEXT</x:v>
+      </x:c>
+      <x:c r="O31" s="4" t="str">
         <x:v>published</x:v>
       </x:c>
-      <x:c r="P29" s="4" t="str">
+      <x:c r="P31" s="4" t="str">
         <x:v>VERIFIED_PRIMARY</x:v>
       </x:c>
-      <x:c r="Q29" s="4" t="str">
+      <x:c r="Q31" s="4" t="str">
         <x:v>历史访问尝试：ScienceDirect正式页面/DOI记录核验标题、作者、期刊、卷页、年份、摘要
 作者机构仓储元数据可见
 仓储bitstream请求返回HTML/bot内容（15040 bytes），不是PDF
@@ -3429,44 +3610,44 @@
 备注：2026-10-22用户提供20页正式期刊PDF，已全文阅读并核对公式。arrival目标对应最终地面stage1完成；目标时间的电池动机不等于SOC动态约束，启发式没有已证近优界。</x:v>
       </x:c>
     </x:row>
-    <x:row r="30" ht="94" customHeight="1">
-      <x:c r="A30" s="4" t="str">
+    <x:row r="32" ht="94" customHeight="1">
+      <x:c r="A32" s="4" t="str">
         <x:v>C07</x:v>
       </x:c>
-      <x:c r="B30" s="4" t="str">
+      <x:c r="B32" s="4" t="str">
         <x:v>★ S. Schier-Morgenthal; R. Abdellaoui; I. C. Metz</x:v>
       </x:c>
-      <x:c r="C30" s="4" t="str">
+      <x:c r="C32" s="4" t="str">
         <x:v>CEAS Aeronautical Journal, 16, 339–352</x:v>
       </x:c>
-      <x:c r="D30" s="4" t="n">
+      <x:c r="D32" s="4" t="n">
         <x:v>2025</x:v>
       </x:c>
-      <x:c r="E30" s="4" t="str">
+      <x:c r="E32" s="4" t="str">
         <x:v>10.1007/s13272-024-00802-1</x:v>
       </x:c>
-      <x:c r="F30" s="4" t="str">
+      <x:c r="F32" s="4" t="str">
         <x:v>https://doi.org/10.1007/s13272-024-00802-1</x:v>
       </x:c>
-      <x:c r="G30" s="4" t="str">
+      <x:c r="G32" s="4" t="str">
         <x:v>https://link.springer.com/content/pdf/10.1007/s13272-024-00802-1.pdf</x:v>
       </x:c>
-      <x:c r="H30" s="4" t="str">
+      <x:c r="H32" s="4" t="str">
         <x:v>originals/C07.pdf</x:v>
       </x:c>
-      <x:c r="I30" s="4" t="str">
+      <x:c r="I32" s="4" t="str">
         <x:v>extracted/C07.txt</x:v>
       </x:c>
-      <x:c r="J30" s="4" t="str">
+      <x:c r="J32" s="4" t="str">
         <x:v>publisher</x:v>
       </x:c>
-      <x:c r="K30" s="4" t="str">
+      <x:c r="K32" s="4" t="str">
         <x:v>汉堡机场控制区内VFR空中出租车；本文评价取自一次人机仿真场景中的15架空中出租车航班。到达交通在同一路线上采用1500 ft高度、离场交通采用2000 ft高度进行垂直分离。5分钟内超过6架时触发hold，walkthrough中4架收到交通负荷hold命令；Vertiport East另有4次holding decision。</x:v>
       </x:c>
-      <x:c r="L30" s="4" t="str">
+      <x:c r="L32" s="4" t="str">
         <x:v>相关DLR人机仿真中10名管制员在最高15架空中出租车/小时交通负荷下工作负荷约增加30%（引言/§2，属于相关工作数字）；本文walkthrough使用一次场景的15架空中出租车航班，4架收到交通负荷hold命令，另有Vertiport East的4次holding decision，共计算45项活动且所有航班到达终点。</x:v>
       </x:c>
-      <x:c r="M30" s="4" t="str">
+      <x:c r="M32" s="4" t="str">
         <x:v>Abstract, p.339
 §2 Existing work, p.340
 §3 Design, pp.341–344
@@ -3474,135 +3655,135 @@
 §5 Discussion, pp.347–348
 §6 Outlook, p.348</x:v>
       </x:c>
-      <x:c r="N30" s="11" t="str">
-        <x:v>FULL_TEXT</x:v>
-      </x:c>
-      <x:c r="O30" s="4" t="str">
+      <x:c r="N32" s="11" t="str">
+        <x:v>FULL_TEXT</x:v>
+      </x:c>
+      <x:c r="O32" s="4" t="str">
         <x:v>published</x:v>
       </x:c>
-      <x:c r="P30" s="4" t="str">
+      <x:c r="P32" s="4" t="str">
         <x:v>VERIFIED_PRIMARY</x:v>
       </x:c>
-      <x:c r="Q30" s="4" t="str">
+      <x:c r="Q32" s="4" t="str">
         <x:v>历史访问尝试：Springer正式文章/DOI页面核验标题、作者、期刊、年份和DOI
 Springer开放PDF下载成功
 本地PDF头为%PDF，pypdf解析14页并通读正文
 备注：在线发表日期为2025-01-18；期刊卷为16。</x:v>
       </x:c>
     </x:row>
-    <x:row r="31" ht="94" customHeight="1">
-      <x:c r="A31" s="4" t="str">
+    <x:row r="33" ht="94" customHeight="1">
+      <x:c r="A33" s="4" t="str">
         <x:v>C08</x:v>
       </x:c>
-      <x:c r="B31" s="4" t="str">
+      <x:c r="B33" s="4" t="str">
         <x:v>★ Nabih Naeem; Patrick Ratei; Prajwal Shiva Prakasha; Lukas Asmer; Roman Jaksche; Henry Pak; Karolin Schweiger; Asija Velieva; Fares Naser; Majed Swaid; Jan Pertz; Malte Niklaß</x:v>
       </x:c>
-      <x:c r="C31" s="4" t="str">
+      <x:c r="C33" s="4" t="str">
         <x:v>CEAS Aeronautical Journal, 16, 729–744</x:v>
       </x:c>
-      <x:c r="D31" s="4" t="n">
+      <x:c r="D33" s="4" t="n">
         <x:v>2025</x:v>
       </x:c>
-      <x:c r="E31" s="4" t="str">
+      <x:c r="E33" s="4" t="str">
         <x:v>10.1007/s13272-024-00796-w</x:v>
       </x:c>
-      <x:c r="F31" s="4" t="str">
+      <x:c r="F33" s="4" t="str">
         <x:v>https://doi.org/10.1007/s13272-024-00796-w</x:v>
       </x:c>
-      <x:c r="G31" s="4" t="str">
+      <x:c r="G33" s="4" t="str">
         <x:v>https://link.springer.com/content/pdf/10.1007/s13272-024-00796-w.pdf</x:v>
       </x:c>
-      <x:c r="H31" s="4" t="str">
+      <x:c r="H33" s="4" t="str">
         <x:v>originals/C08.pdf</x:v>
       </x:c>
-      <x:c r="I31" s="4" t="str">
+      <x:c r="I33" s="4" t="str">
         <x:v>extracted/C08.txt</x:v>
       </x:c>
-      <x:c r="J31" s="4" t="str">
+      <x:c r="J33" s="4" t="str">
         <x:v>publisher</x:v>
       </x:c>
-      <x:c r="K31" s="4" t="str">
+      <x:c r="K33" s="4" t="str">
         <x:v>汉堡20个vertiport、30架倾转旋翼机（3名乘客+1名飞行员），仿真时长4小时，票价2 EUR/km。本文轨迹工具采用爬升/下降3.556 m/s、巡航高度457 m、横向0.002°、垂直250 m、时间60 s间隔；共处理1239个飞行请求，其中43个UAM请求，模式份额3.4%。</x:v>
       </x:c>
-      <x:c r="L31" s="4" t="str">
+      <x:c r="L33" s="4" t="str">
         <x:v>仿真含20个vertiport、30架飞机、4 h、1239个飞行请求、43个UAM请求和3.4%模式份额；票价为2 EUR/km。冲突处理通过改变出发/到达时间，使用横向0.002°、垂直250 m、时间60 s约束。</x:v>
       </x:c>
-      <x:c r="M31" s="4" t="str">
+      <x:c r="M33" s="4" t="str">
         <x:v>§2.1–§2.2, pp.733–737
 §3 Results and discussion, pp.740–742
 §4 Opportunities and challenges, pp.742–743
 Abstract and table/figure descriptions, pp.729–744</x:v>
       </x:c>
-      <x:c r="N31" s="11" t="str">
-        <x:v>FULL_TEXT</x:v>
-      </x:c>
-      <x:c r="O31" s="4" t="str">
+      <x:c r="N33" s="11" t="str">
+        <x:v>FULL_TEXT</x:v>
+      </x:c>
+      <x:c r="O33" s="4" t="str">
         <x:v>published</x:v>
       </x:c>
-      <x:c r="P31" s="4" t="str">
+      <x:c r="P33" s="4" t="str">
         <x:v>VERIFIED_PRIMARY</x:v>
       </x:c>
-      <x:c r="Q31" s="4" t="str">
+      <x:c r="Q33" s="4" t="str">
         <x:v>历史访问尝试：Springer正式文章/DOI页面核验标题、全作者、期刊、年份和DOI
 Springer开放PDF下载成功
 本地PDF头为%PDF，pypdf解析16页并通读正文
 备注：在线发表日期为2024-12-23；期刊卷为16（2025）。</x:v>
       </x:c>
     </x:row>
-    <x:row r="32" ht="94" customHeight="1">
-      <x:c r="A32" s="4" t="str">
+    <x:row r="34" ht="94" customHeight="1">
+      <x:c r="A34" s="4" t="str">
         <x:v>C09</x:v>
       </x:c>
-      <x:c r="B32" s="4" t="str">
+      <x:c r="B34" s="4" t="str">
         <x:v>★ Hanbong Lee; Alan G. Lee; Levin Guillermo; Chin H. Seah; Kushal A. Moolchandani</x:v>
       </x:c>
-      <x:c r="C32" s="4" t="str">
+      <x:c r="C34" s="4" t="str">
         <x:v>AIAA Aviation Forum and Exposition 2024, AIAA-2024-3854</x:v>
       </x:c>
-      <x:c r="D32" s="4" t="n">
+      <x:c r="D34" s="4" t="n">
         <x:v>2024</x:v>
       </x:c>
-      <x:c r="E32" s="4" t="str">
+      <x:c r="E34" s="4" t="str">
         <x:v>10.2514/6.2024-3854</x:v>
       </x:c>
-      <x:c r="F32" s="4" t="str">
+      <x:c r="F34" s="4" t="str">
         <x:v>https://ntrs.nasa.gov/citations/20240007388</x:v>
       </x:c>
-      <x:c r="G32" s="4" t="str">
+      <x:c r="G34" s="4" t="str">
         <x:v>https://ntrs.nasa.gov/api/citations/20240007388/downloads/AIAA_Aviation_2024_HanbongLee_v3.pdf</x:v>
       </x:c>
-      <x:c r="H32" s="4" t="str">
+      <x:c r="H34" s="4" t="str">
         <x:v>originals/C09.pdf</x:v>
       </x:c>
-      <x:c r="I32" s="4" t="str">
+      <x:c r="I34" s="4" t="str">
         <x:v>extracted/C09.txt</x:v>
       </x:c>
-      <x:c r="J32" s="4" t="str">
+      <x:c r="J34" s="4" t="str">
         <x:v>publisher</x:v>
       </x:c>
-      <x:c r="K32" s="4" t="str">
+      <x:c r="K34" s="4" t="str">
         <x:v>DFW网络7个vertiport、10条OD航路、4个排序控制航路点；vertiport容量2次/12 min bin，控制点最小间隔2 min。单一飞机类型/速度；40架次、1.5 h，2个运营方各20架、每条航路每运营方2架。DCB提前6 min，S&amp;S在新起飞时刻前1 min或紧接DCB运行，最大延误1 h。</x:v>
       </x:c>
-      <x:c r="L32" s="4" t="str">
+      <x:c r="L34" s="4" t="str">
         <x:v>DCB案例每个运营方最多约8/7架并发，S&amp;S-only最多24架；启用DCB的案例因1 h最大延误各取消1架（40架中39架激活），S&amp;S-only无取消。Case 3中98.2%的地面延误来自DCB，25架/39架受延误；两个运营方各14架延误，平均分别23.7和27.6 min/架。DCB案例峰值并发量13。</x:v>
       </x:c>
-      <x:c r="M32" s="4" t="str">
+      <x:c r="M34" s="4" t="str">
         <x:v>§II System Architecture, pp.3–6
 §III Simulation Setup, pp.7–9
 §IV Results, pp.9–11
 §V Conclusions and Future Work, pp.11–12
 Tables 1–4, pp.7–11</x:v>
       </x:c>
-      <x:c r="N32" s="11" t="str">
-        <x:v>FULL_TEXT</x:v>
-      </x:c>
-      <x:c r="O32" s="4" t="str">
+      <x:c r="N34" s="11" t="str">
+        <x:v>FULL_TEXT</x:v>
+      </x:c>
+      <x:c r="O34" s="4" t="str">
         <x:v>published</x:v>
       </x:c>
-      <x:c r="P32" s="4" t="str">
+      <x:c r="P34" s="4" t="str">
         <x:v>VERIFIED_PRIMARY</x:v>
       </x:c>
-      <x:c r="Q32" s="4" t="str">
+      <x:c r="Q34" s="4" t="str">
         <x:v>历史访问尝试：NASA NTRS正式记录打开并核验标题、全作者、会议、年份和公开PDF
 AIAA DOI记录核验DOI
 NASA PDF下载成功
@@ -3610,44 +3791,44 @@
 备注：会议论文AIAA-2024-3854；NASA公开版本文件名含v3。</x:v>
       </x:c>
     </x:row>
-    <x:row r="33" ht="136" customHeight="1">
-      <x:c r="A33" s="4" t="str">
+    <x:row r="35" ht="136" customHeight="1">
+      <x:c r="A35" s="4" t="str">
         <x:v>C10</x:v>
       </x:c>
-      <x:c r="B33" s="4" t="str">
+      <x:c r="B35" s="4" t="str">
         <x:v>★ Canqiang Weng; Can Chen; Jingjun Tan; Tianlu Pan; Renxin Zhong</x:v>
       </x:c>
-      <x:c r="C33" s="4" t="str">
+      <x:c r="C35" s="4" t="str">
         <x:v>Transportation Research Part C: Emerging Technologies, 183, 105477</x:v>
       </x:c>
-      <x:c r="D33" s="4" t="n">
+      <x:c r="D35" s="4" t="n">
         <x:v>2026</x:v>
       </x:c>
-      <x:c r="E33" s="4" t="str">
+      <x:c r="E35" s="4" t="str">
         <x:v>10.1016/j.trc.2025.105477</x:v>
       </x:c>
-      <x:c r="F33" s="4" t="str">
+      <x:c r="F35" s="4" t="str">
         <x:v>https://www.sciencedirect.com/science/article/pii/S0968090X25004814</x:v>
       </x:c>
-      <x:c r="G33" s="4" t="str">
+      <x:c r="G35" s="4" t="str">
         <x:v>https://arxiv.org/pdf/2412.01235</x:v>
       </x:c>
-      <x:c r="H33" s="4" t="str">
+      <x:c r="H35" s="4" t="str">
         <x:v>originals/C10.pdf</x:v>
       </x:c>
-      <x:c r="I33" s="4" t="str">
+      <x:c r="I35" s="4" t="str">
         <x:v>extracted/C10.txt</x:v>
       </x:c>
-      <x:c r="J33" s="4" t="str">
+      <x:c r="J35" s="4" t="str">
         <x:v>preprint</x:v>
       </x:c>
-      <x:c r="K33" s="4" t="str">
+      <x:c r="K35" s="4" t="str">
         <x:v>抽象城市六边形空域和点对点需求，比较单层z=500 m、单层范围450–550/400–600 m及双层z=400/600 m；区域半径250 m、探测半径200 m、安全半径50 m、最大速度20 m/s、控制增益5、步长1 s。三种OD需求图案（+、#、*）和临界流附近固定需求；基线为无冲突虚拟走廊/自由飞行策略。</x:v>
       </x:c>
-      <x:c r="L33" s="4" t="str">
+      <x:c r="L35" s="4" t="str">
         <x:v>单层表3中，基线→提出方法：平均最小间距153.3→303.9 m（+98.2%），平均速度11.39→19.39 m/s（+70.2%），完成率0.083→0.191 trip/s（+130%），能耗0.0148→0.0114 kWh/trip（−23.0%），计算效率0.91→4.85 iteration/s（+433%）。双层相对单层平均最小间距+56.3%、速度+38.9%、完成率+40.1%。</x:v>
       </x:c>
-      <x:c r="M33" s="4" t="str">
+      <x:c r="M35" s="4" t="str">
         <x:v>§2.1 Airspace and route-guidance model, p.5
 §2.2 Assumptions, p.7
 §2.3 Route guidance, pp.7–12
@@ -3657,16 +3838,16 @@
 §3.2.2, p.20
 §4 Conclusion, p.24</x:v>
       </x:c>
-      <x:c r="N33" s="11" t="str">
-        <x:v>FULL_TEXT</x:v>
-      </x:c>
-      <x:c r="O33" s="4" t="str">
+      <x:c r="N35" s="11" t="str">
+        <x:v>FULL_TEXT</x:v>
+      </x:c>
+      <x:c r="O35" s="4" t="str">
         <x:v>published</x:v>
       </x:c>
-      <x:c r="P33" s="4" t="str">
+      <x:c r="P35" s="4" t="str">
         <x:v>VERIFIED_PRIMARY_DOI</x:v>
       </x:c>
-      <x:c r="Q33" s="4" t="str">
+      <x:c r="Q35" s="4" t="str">
         <x:v>历史访问尝试：ScienceDirect正式页面核验标题、作者、期刊、卷页、年份和DOI；publisher正文未下载
 arXiv公开记录https://arxiv.org/abs/2412.01235打开
 arXiv v2 PDF下载成功并完整读取26页
@@ -3675,44 +3856,44 @@
 备注：正式卷期页面显示2026年、文章号105477；DOI含2025。本地全文为arXiv v2（非出版社排版版）。</x:v>
       </x:c>
     </x:row>
-    <x:row r="34" ht="136" customHeight="1">
-      <x:c r="A34" s="4" t="str">
+    <x:row r="36" ht="136" customHeight="1">
+      <x:c r="A36" s="4" t="str">
         <x:v>C11</x:v>
       </x:c>
-      <x:c r="B34" s="4" t="str">
+      <x:c r="B36" s="4" t="str">
         <x:v>★ Yingqi Liu; Tianlu Pan; Jingjun Tan; Renxin Zhong; Can Chen</x:v>
       </x:c>
-      <x:c r="C34" s="4" t="str">
+      <x:c r="C36" s="4" t="str">
         <x:v>Transportation Research Part C: Emerging Technologies, 182, 105370</x:v>
       </x:c>
-      <x:c r="D34" s="4" t="n">
+      <x:c r="D36" s="4" t="n">
         <x:v>2026</x:v>
       </x:c>
-      <x:c r="E34" s="4" t="str">
+      <x:c r="E36" s="4" t="str">
         <x:v>10.1016/j.trc.2025.105370</x:v>
       </x:c>
-      <x:c r="F34" s="4" t="str">
+      <x:c r="F36" s="4" t="str">
         <x:v>https://www.sciencedirect.com/science/article/pii/S0968090X25003742</x:v>
       </x:c>
-      <x:c r="G34" s="4" t="str">
+      <x:c r="G36" s="4" t="str">
         <x:v>https://arxiv.org/pdf/2508.15395</x:v>
       </x:c>
-      <x:c r="H34" s="4" t="str">
+      <x:c r="H36" s="4" t="str">
         <x:v>originals/C11.pdf</x:v>
       </x:c>
-      <x:c r="I34" s="4" t="str">
+      <x:c r="I36" s="4" t="str">
         <x:v>extracted/C11.txt</x:v>
       </x:c>
-      <x:c r="J34" s="4" t="str">
+      <x:c r="J36" s="4" t="str">
         <x:v>preprint</x:v>
       </x:c>
-      <x:c r="K34" s="4" t="str">
+      <x:c r="K36" s="4" t="str">
         <x:v>Case 1为单走廊—单vertiport：走廊段长度Lc=305 m，起飞时刻[6,36,66,96,126,156] s，6架合流eVTOL；走廊流量以Bernoulli进入概率ρ=0.05（轻流）或0.15（重流）生成，初始5架走廊eVTOL，轻/重场景另有39/59架通过观察区。Case 2为多走廊—vertiport协同，4个vertiport、19架合流eVTOL和61架走廊eVTOL；参数含Tmax=230 s、Ls=50 m、T=6 s、最大速度40 m/s、最大爬升率9 m/s，使用MATLAB R2022b/GPOPS-II。</x:v>
       </x:c>
-      <x:c r="L34" s="4" t="str">
+      <x:c r="L36" s="4" t="str">
         <x:v>Case 1表2中，轻流6架任务的HCTMM完成时间为41.1、71.1、101.1、131.1、180.9、191.1 s；重流为41.1、71.1、101.1、131.1、193.9、216.8 s，ATFM在重流M6未在Tmax内完成。表3 HCTMM计算时间为轻流4.42 s、重流5.83 s；RES为9.67/10.84 s；GES为15.94/68.80 s，保留规划时间阈值T=6 s。Case 2含19架合流和61架走廊eVTOL，TM section将平均计算时间保持在6 s以下，约为无TM设计的二分之一至三分之一。</x:v>
       </x:c>
-      <x:c r="M34" s="4" t="str">
+      <x:c r="M36" s="4" t="str">
         <x:v>§2.1–§2.3, pp.5–10
 §3.1–§3.2, pp.10–14
 §4 Operational trajectory optimization, pp.15–17
@@ -3720,16 +3901,16 @@
 §6 Conclusion, p.24
 Tables 1–3, pp.18–23</x:v>
       </x:c>
-      <x:c r="N34" s="11" t="str">
-        <x:v>FULL_TEXT</x:v>
-      </x:c>
-      <x:c r="O34" s="4" t="str">
+      <x:c r="N36" s="11" t="str">
+        <x:v>FULL_TEXT</x:v>
+      </x:c>
+      <x:c r="O36" s="4" t="str">
         <x:v>published</x:v>
       </x:c>
-      <x:c r="P34" s="4" t="str">
+      <x:c r="P36" s="4" t="str">
         <x:v>VERIFIED_PRIMARY_DOI_CROSSREF</x:v>
       </x:c>
-      <x:c r="Q34" s="4" t="str">
+      <x:c r="Q36" s="4" t="str">
         <x:v>历史访问尝试：ScienceDirect正式文章搜索结果和Crossref DOI元数据核验标题、全作者、期刊、卷、文章号、年份和DOI；ScienceDirect正文请求返回403
 arXiv公开全文下载成功
 本地PDF头为%PDF，pypdf解析31页并完整读取正文
@@ -3740,7 +3921,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4f2f8f40aaea49f6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R28ab01809da84d95"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3778,7 +3959,7 @@
     </x:row>
     <x:row r="2" ht="30" customHeight="1">
       <x:c r="A2" s="18" t="str">
-        <x:v>已读HTML但无本地文件：1篇（A08）</x:v>
+        <x:v>已读全文但无本地文件：2篇</x:v>
       </x:c>
       <x:c r="B2" s="18"/>
       <x:c r="C2" s="18"/>
@@ -3791,7 +3972,7 @@
     </x:row>
     <x:row r="3" ht="58" customHeight="1">
       <x:c r="A3" s="25" t="str">
-        <x:v>说明：A08 公开 HTML 已读至正文结论，但本地 PDF/HTML 文件缺失；该项单独标注，不计入未全文阅读数量。</x:v>
+        <x:v>说明：A08（远程全文）、A11（阅读媒介为remote PDF（公开作者PDF），通过web全文文本分段覆盖全部8页，包括最终讨论、限制和参考文献；不是HTML阅读，也非仅核对相关摘要或局部段落。） 已完成全文阅读，但因本地离线文件缺失而单独列示；不计入未全文阅读数量。</x:v>
       </x:c>
       <x:c r="B3" s="25"/>
       <x:c r="C3" s="25"/>
@@ -3912,7 +4093,36 @@
 备注：已从公开 publisher HTML 连续阅读 Introduction、Sec. 2–4 和 Conclusion（HTML lines 150–526）；Wiley 直接下载被 Cloudflare/SSL 阻断，未保存本地 HTML/PDF/text。论文为开放获取，全文内容在公开 HTML 中可读。</x:v>
       </x:c>
       <x:c r="I8" s="27" t="str">
-        <x:v>公开 HTML 已读至正文结论，但本地 PDF/HTML 文件缺失；此行不计入未全文阅读数量</x:v>
+        <x:v>已全文阅读（远程全文），但本地 PDF/文本文件缺失；此行不计入未全文阅读数量</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="220" customHeight="1">
+      <x:c r="A9" s="4" t="str">
+        <x:v>A11</x:v>
+      </x:c>
+      <x:c r="B9" s="4" t="str">
+        <x:v>Coordinated Dense Aerial Traffic with Self-Driving Drones（2018）</x:v>
+      </x:c>
+      <x:c r="C9" s="26" t="str">
+        <x:v>FULL_TEXT</x:v>
+      </x:c>
+      <x:c r="D9" s="27" t="str"/>
+      <x:c r="E9" s="27" t="str"/>
+      <x:c r="F9" s="27" t="str">
+        <x:v>https://ieeexplore.ieee.org/document/8461073</x:v>
+      </x:c>
+      <x:c r="G9" s="27" t="str">
+        <x:v>https://hal.elte.hu/~vasarhelyi/doc/balazs2018coordinated.pdf</x:v>
+      </x:c>
+      <x:c r="H9" s="27" t="str">
+        <x:v>阅读媒介：阅读媒介为remote PDF（公开作者PDF），通过web全文文本分段覆盖全部8页，包括最终讨论、限制和参考文献；不是HTML阅读，也非仅核对相关摘要或局部段落。
+访问记录：公开作者PDF由web工具成功读取，8页，全文文本行0–956已分段连续核对，含方法、实验、讨论、图注及参考文献。
+本地普通沙箱下载遇WinError10013；获网络审批后的Python HTTPS遇SSL EOF，Windows Invoke-WebRequest重试仍SSL失败；同一已核作者站HTTP入口仅追加尝试一次，也返回请求发送错误；没有生成A11.pdf或A11.txt。
+IEEE文档8461073页面返回JavaScript机器人检查；正式发表信息由带IEEE版权和页码的公开正文核实，DOI另由Springer正式A07参考文献核对；未绕过访问限制。
+备注：2026-10-22补充。公开作者副本保留IEEE出版排版；FULL_TEXT表示本次已阅读全文8页，不表示本地PDF存在。local_pdf/local_text为空，因为本地下载失败；不虚构本地路径。</x:v>
+      </x:c>
+      <x:c r="I9" s="27" t="str">
+        <x:v>已全文阅读（阅读媒介为remote PDF（公开作者PDF），通过web全文文本分段覆盖全部8页，包括最终讨论、限制和参考文献；不是HTML阅读，也非仅核对相关摘要或局部段落。），但本地 PDF/文本文件缺失；此行不计入未全文阅读数量</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3923,7 +4133,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R509c468a2b9741f3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra5405236f5d145d3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>